<commit_message>
update latest spreadsheet and resolved known issues page
</commit_message>
<xml_diff>
--- a/tools/data/latest.xlsx
+++ b/tools/data/latest.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10911"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{61E23DC8-8D47-6F4E-8EAE-210DE2176164}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA4B8235-5C44-9C4C-A89A-6AE5D2B15A1B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="14900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="15060" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="🤩 public data release" sheetId="1" r:id="rId1"/>
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="712" uniqueCount="246">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="760" uniqueCount="264">
   <si>
     <t>Name</t>
   </si>
@@ -56,187 +56,718 @@
     <t>[DATA REQUEST]- calculate SGA (intergrowth curves, anthro) LT solution into DB</t>
   </si>
   <si>
+    <t>30.3</t>
+  </si>
+  <si>
+    <t>Santiago Torres Gomez</t>
+  </si>
+  <si>
+    <t>Active</t>
+  </si>
+  <si>
+    <t>ID-20</t>
+  </si>
+  <si>
+    <t>Physical Health</t>
+  </si>
+  <si>
+    <t>pending</t>
+  </si>
+  <si>
+    <t>Done</t>
+  </si>
+  <si>
+    <t>Anthropometrics</t>
+  </si>
+  <si>
+    <t>Yes</t>
+  </si>
+  <si>
+    <t>ERICA derived fields for reliability and codes QC</t>
+  </si>
+  <si>
+    <t>30.2</t>
+  </si>
+  <si>
+    <t>Dev Done</t>
+  </si>
+  <si>
+    <t>ID-21</t>
+  </si>
+  <si>
+    <t>Behavior &amp; Child-Caregiver Interaction</t>
+  </si>
+  <si>
+    <t>ERICA</t>
+  </si>
+  <si>
+    <t>Clean up crew: Multiple births</t>
+  </si>
+  <si>
+    <t>Dan Duhon</t>
+  </si>
+  <si>
+    <t>ETL to review</t>
+  </si>
+  <si>
+    <t>ID-22</t>
+  </si>
+  <si>
+    <t>All Data / General</t>
+  </si>
+  <si>
+    <t>Blank Fields for Siblings</t>
+  </si>
+  <si>
+    <t>[DATA ERROR]- FAD scoring issues at V06</t>
+  </si>
+  <si>
+    <t>unknown</t>
+  </si>
+  <si>
+    <t>LORIS review</t>
+  </si>
+  <si>
+    <t>ID-24</t>
+  </si>
+  <si>
+    <t>known_issue</t>
+  </si>
+  <si>
+    <t>FAD</t>
+  </si>
+  <si>
+    <t>[DATA ERROR]- MAPTSTL scores incorrectly marked as "not enough answers to compute score"</t>
+  </si>
+  <si>
+    <t>ID-26</t>
+  </si>
+  <si>
+    <t>MAPS-TL (Tod)</t>
+  </si>
+  <si>
+    <t>[DATA ERROR]- ecPROMIS child-caregiver infant</t>
+  </si>
+  <si>
+    <t>30.1</t>
+  </si>
+  <si>
+    <t>Jen Zink</t>
+  </si>
+  <si>
+    <t>Waiting on WG feedback</t>
+  </si>
+  <si>
+    <t>ID-27</t>
+  </si>
+  <si>
+    <t>ecPROMIS CC</t>
+  </si>
+  <si>
+    <t>[IMAGING] Add Cook's distance to tabulated imaging data</t>
+  </si>
+  <si>
+    <t>ID-28</t>
+  </si>
+  <si>
+    <t>MRI</t>
+  </si>
+  <si>
+    <t>Cook's Distance</t>
+  </si>
+  <si>
+    <t>[2.0 SCORING CORRECTION NEEDED]- V03 MAPS-TL</t>
+  </si>
+  <si>
+    <t>ID-30</t>
+  </si>
+  <si>
+    <t>MAPS-TL (&lt;1yr)</t>
+  </si>
+  <si>
+    <t>[DATA ERROR]- implausible gestational ages in multiple instruments (parameter-based filtering)</t>
+  </si>
+  <si>
+    <t>Santiago Torres Gomez, Stephanie Averill</t>
+  </si>
+  <si>
+    <t>ID-32</t>
+  </si>
+  <si>
+    <t>Implausible GA</t>
+  </si>
+  <si>
+    <t>[LORIS BUG]- adjusted age</t>
+  </si>
+  <si>
+    <t>ID-33</t>
+  </si>
+  <si>
+    <t>[DATA ERROR]- MAV01 in Release 2.0</t>
+  </si>
+  <si>
+    <t>ID-34</t>
+  </si>
+  <si>
+    <t>Demographics</t>
+  </si>
+  <si>
+    <t>Basic Demo</t>
+  </si>
+  <si>
+    <t>[DD ERROR] - push text in score fields to 'notes' fields (SPM2 &amp; ecPROMIS-PAGS)</t>
+  </si>
+  <si>
+    <t>ID-36</t>
+  </si>
+  <si>
+    <t>Score text</t>
+  </si>
+  <si>
+    <t>TLFB not parsed items</t>
+  </si>
+  <si>
     <t/>
   </si>
   <si>
-    <t>Santiago Torres Gomez, Jen Zink</t>
-  </si>
-  <si>
-    <t>Waiting on WG feedback</t>
-  </si>
-  <si>
-    <t>ID-20</t>
-  </si>
-  <si>
-    <t>Physical Health</t>
-  </si>
-  <si>
-    <t>pending</t>
-  </si>
-  <si>
-    <t>Done</t>
-  </si>
-  <si>
-    <t>Anthropometrics</t>
-  </si>
-  <si>
-    <t>Yes</t>
-  </si>
-  <si>
-    <t>ERICA derived fields for reliability and codes QC</t>
-  </si>
-  <si>
-    <t>30.1</t>
-  </si>
-  <si>
-    <t>Santiago Torres Gomez</t>
-  </si>
-  <si>
-    <t>Dev Done</t>
-  </si>
-  <si>
-    <t>ID-21</t>
-  </si>
-  <si>
-    <t>Behavior &amp; Child-Caregiver Interaction</t>
-  </si>
-  <si>
-    <t>ERICA</t>
-  </si>
-  <si>
-    <t>Clean up crew: Multiple births</t>
-  </si>
-  <si>
-    <t>ETL to review</t>
-  </si>
-  <si>
-    <t>ID-22</t>
-  </si>
-  <si>
-    <t>All Data / General</t>
-  </si>
-  <si>
-    <t>Blank Fields for Siblings</t>
-  </si>
-  <si>
-    <t>[DATA ERROR]- FAD scoring issues at V06</t>
-  </si>
-  <si>
-    <t>Jen Zink</t>
+    <t>Ongoing/DR independent</t>
+  </si>
+  <si>
+    <t>ID-37</t>
+  </si>
+  <si>
+    <t>TLFB</t>
+  </si>
+  <si>
+    <t>[DD+DATA ERROR] Nail type field added for 2.0 all "Unknown"</t>
+  </si>
+  <si>
+    <t>ID-42</t>
+  </si>
+  <si>
+    <t>Biospecimens &amp; Omics</t>
+  </si>
+  <si>
+    <t>Nails</t>
+  </si>
+  <si>
+    <t>[DATA REQUEST]- consistent ICD code names</t>
+  </si>
+  <si>
+    <t>ID-43</t>
+  </si>
+  <si>
+    <t>Pregnancy &amp; Environmental Exposure</t>
+  </si>
+  <si>
+    <t>PEX Health</t>
+  </si>
+  <si>
+    <t>Inclusion of Blood Spot Card Results data from USDTL. Addressing issue of incorrect cleaning practices at sites that affect test results PEth.</t>
   </si>
   <si>
     <t>Lasso review and ensure WG knows</t>
   </si>
   <si>
-    <t>ID-24</t>
-  </si>
-  <si>
-    <t>known_issue</t>
-  </si>
-  <si>
-    <t>FAD</t>
-  </si>
-  <si>
-    <t>[DATA ERROR]- MAPTSTL scores incorrectly marked as "not enough answers to compute score"</t>
-  </si>
-  <si>
-    <t>ID-26</t>
-  </si>
-  <si>
-    <t>MAPS-TL (Tod)</t>
-  </si>
-  <si>
-    <t>[DATA ERROR]- ecPROMIS child-caregiver infant</t>
-  </si>
-  <si>
-    <t>ID-27</t>
-  </si>
-  <si>
-    <t>ecPROMIS CC</t>
-  </si>
-  <si>
-    <t>[IMAGING] Add Cook's distance to tabulated imaging data</t>
-  </si>
-  <si>
-    <t>30.2</t>
-  </si>
-  <si>
-    <t>Active</t>
-  </si>
-  <si>
-    <t>ID-28</t>
-  </si>
-  <si>
-    <t>MRI</t>
-  </si>
-  <si>
-    <t>Cook's Distance</t>
-  </si>
-  <si>
-    <t>[2.0 SCORING CORRECTION NEEDED]- V03 MAPS-TL</t>
-  </si>
-  <si>
-    <t>ID-30</t>
-  </si>
-  <si>
-    <t>MAPS-TL (&lt;1yr)</t>
-  </si>
-  <si>
-    <t>[DATA ERROR]- implausible gestational ages in multiple instruments (parameter-based filtering)</t>
-  </si>
-  <si>
-    <t>Santiago Torres Gomez, Stephanie Averill</t>
-  </si>
-  <si>
-    <t>ID-32</t>
-  </si>
-  <si>
-    <t>Implausible GA</t>
-  </si>
-  <si>
-    <t>[LORIS BUG]- adjusted age</t>
-  </si>
-  <si>
-    <t>LORIS review</t>
-  </si>
-  <si>
-    <t>ID-33</t>
-  </si>
-  <si>
-    <t>[DATA ERROR]- MAV01 in Release 2.0</t>
-  </si>
-  <si>
-    <t>Dan Duhon</t>
-  </si>
-  <si>
-    <t>ID-34</t>
-  </si>
-  <si>
-    <t>Demographics</t>
-  </si>
-  <si>
-    <t>Basic Demo</t>
-  </si>
-  <si>
-    <t>[DD ERROR] - push text in score fields to 'notes' fields (SPM2 &amp; ecPROMIS-PAGS)</t>
-  </si>
-  <si>
-    <t>ID-36</t>
-  </si>
-  <si>
-    <t>Score text</t>
-  </si>
-  <si>
-    <t>TLFB not parsed items</t>
-  </si>
-  <si>
-    <t>Ongoing/DR independent</t>
-  </si>
-  <si>
-    <t>ID-37</t>
-  </si>
-  <si>
-    <t>TLFB</t>
+    <t>ID-44</t>
+  </si>
+  <si>
+    <t>Blood</t>
+  </si>
+  <si>
+    <t>[DATA REQUEST] ERICA - add age &amp; date_taken fields back to ERICA</t>
+  </si>
+  <si>
+    <t>ID-45</t>
+  </si>
+  <si>
+    <t>Anthro: [Incorrect Data] ph_ch_anthro_average_bmi</t>
+  </si>
+  <si>
+    <t>ID-47</t>
+  </si>
+  <si>
+    <t>Anthro: ph_ch_anthro_head_for_age_boys_z_score</t>
+  </si>
+  <si>
+    <t>ID-48</t>
+  </si>
+  <si>
+    <t>[DATA REQUEST]-household roster - sex variable</t>
+  </si>
+  <si>
+    <t>ID-50</t>
+  </si>
+  <si>
+    <t>Social &amp; Environmental Determinants</t>
+  </si>
+  <si>
+    <t>Demo</t>
+  </si>
+  <si>
+    <t>[POSSIBLE DATA ERROR]- relationship status at V03</t>
+  </si>
+  <si>
+    <t>ID-53</t>
+  </si>
+  <si>
+    <t>Bayley invalid subscores (-9999) (parameter-based filtering)</t>
+  </si>
+  <si>
+    <t>Patch</t>
+  </si>
+  <si>
+    <t>ID-54</t>
+  </si>
+  <si>
+    <t>Neurocognition &amp; Language</t>
+  </si>
+  <si>
+    <t>Bayley</t>
+  </si>
+  <si>
+    <t>[IMAGING] MRI bad frame removal workflow</t>
+  </si>
+  <si>
+    <t>Tanya Pandhi, Cecile Madjar</t>
+  </si>
+  <si>
+    <t>ID-59</t>
+  </si>
+  <si>
+    <t>fmap QC</t>
+  </si>
+  <si>
+    <t>[POSSIBLE DATA ERROR]- roster at V02 or V03 (parameter-based filtering is precursor)</t>
+  </si>
+  <si>
+    <t>ID-60</t>
+  </si>
+  <si>
+    <t>Geocoded Linkage from Home and Work Addresses</t>
+  </si>
+  <si>
+    <t>Matthew Schmidt</t>
+  </si>
+  <si>
+    <t>ID-66</t>
+  </si>
+  <si>
+    <t>GLED</t>
+  </si>
+  <si>
+    <t>Transition in Care Questionnaire</t>
+  </si>
+  <si>
+    <t>Tim Meyer, Stephanie Averill, regis.ongaro-carcy@mcin.ca</t>
+  </si>
+  <si>
+    <t>ID-71</t>
+  </si>
+  <si>
+    <t>TIC Questionnaire</t>
+  </si>
+  <si>
+    <t>[DATA ISSUE] - cdiwgen values over 100</t>
+  </si>
+  <si>
+    <t>ID-78</t>
+  </si>
+  <si>
+    <t>CDI</t>
+  </si>
+  <si>
+    <t>Participant status and withdrawal field harmonization</t>
+  </si>
+  <si>
+    <t>Dan Duhon, Matthew Schmidt</t>
+  </si>
+  <si>
+    <t>ID-79</t>
+  </si>
+  <si>
+    <t>Visit Info</t>
+  </si>
+  <si>
+    <t>[DATA ISSUE] - VABS reasons for missingness are wrong</t>
+  </si>
+  <si>
+    <t>ID-80</t>
+  </si>
+  <si>
+    <t>Vineland</t>
+  </si>
+  <si>
+    <t>Update JSON metadata to match Lasso/DEAP updates</t>
+  </si>
+  <si>
+    <t>Jen Zink, Santiago Torres Gomez</t>
+  </si>
+  <si>
+    <t>ID-83</t>
+  </si>
+  <si>
+    <t>Incorrect JSONs</t>
+  </si>
+  <si>
+    <t>Cleanup crew: Inclusion of family pregnancy ID</t>
+  </si>
+  <si>
+    <t>ID-84</t>
+  </si>
+  <si>
+    <t>FamilyID</t>
+  </si>
+  <si>
+    <t>MRI Derivatives - QSIprep - Generate tabular data for QSIRECON</t>
+  </si>
+  <si>
+    <t>ID-86</t>
+  </si>
+  <si>
+    <t>QSIRecon</t>
+  </si>
+  <si>
+    <t>XCP-D corrections and model output</t>
+  </si>
+  <si>
+    <t>Tanya Pandhi, Lucille Moore</t>
+  </si>
+  <si>
+    <t>ID-87</t>
+  </si>
+  <si>
+    <t>Postprocessing</t>
+  </si>
+  <si>
+    <t>[DATA REQUESTs] - novel tech QC feedback overview</t>
+  </si>
+  <si>
+    <t>ID-102</t>
+  </si>
+  <si>
+    <t>Novel Tech &amp; Wearable Sensors</t>
+  </si>
+  <si>
+    <t>unsure</t>
+  </si>
+  <si>
+    <t>TBD</t>
+  </si>
+  <si>
+    <t>[DATA ERRORS]- static table QC feedback</t>
+  </si>
+  <si>
+    <t>ID-106</t>
+  </si>
+  <si>
+    <t>UNSURE</t>
+  </si>
+  <si>
+    <t>Add scanner info as tabulated data</t>
+  </si>
+  <si>
+    <t>Eric Feczko</t>
+  </si>
+  <si>
+    <t>ID-108</t>
+  </si>
+  <si>
+    <t>Scanner info</t>
+  </si>
+  <si>
+    <t>[DATA ERROR]- home 21</t>
+  </si>
+  <si>
+    <t>ID-666</t>
+  </si>
+  <si>
+    <t>br_known_issue</t>
+  </si>
+  <si>
+    <t>Not done</t>
+  </si>
+  <si>
+    <t>HOME-21</t>
+  </si>
+  <si>
+    <t>Tabulated XCP-D derivatives all 0s for numeric fields</t>
+  </si>
+  <si>
+    <t>Cecile Madjar</t>
+  </si>
+  <si>
+    <t>ID-667</t>
+  </si>
+  <si>
+    <t>Tabulated XCP-D</t>
+  </si>
+  <si>
+    <t>[REMOVE INSTRUMENT]- incarceration questionnaire</t>
+  </si>
+  <si>
+    <t>ID-668</t>
+  </si>
+  <si>
+    <t>br_pending</t>
+  </si>
+  <si>
+    <t>Incarceration</t>
+  </si>
+  <si>
+    <t>[SCORING ERROR]- eHITS</t>
+  </si>
+  <si>
+    <t>New; needs discussion</t>
+  </si>
+  <si>
+    <t>ID-670</t>
+  </si>
+  <si>
+    <t>[DATA ERROR]- substance use flags in dynamic table</t>
+  </si>
+  <si>
+    <t>ID-671</t>
+  </si>
+  <si>
+    <t>[DATA UPDATE]- blank out implausible z scores in anthro data</t>
+  </si>
+  <si>
+    <t>ID-673</t>
+  </si>
+  <si>
+    <t>[DATA REQUEST]- revise formatting of vision screener files</t>
+  </si>
+  <si>
+    <t>ID-109</t>
+  </si>
+  <si>
+    <t>Vision Screener</t>
+  </si>
+  <si>
+    <t>Remove 'sequence' field from all tables in Lasso</t>
+  </si>
+  <si>
+    <t>Not started yet</t>
+  </si>
+  <si>
+    <t>ID-110</t>
+  </si>
+  <si>
+    <t>Sequence Field</t>
+  </si>
+  <si>
+    <t>[DATA ERROR]-MLDS  total hours per week of non-parental hours</t>
+  </si>
+  <si>
+    <t>ID-119</t>
+  </si>
+  <si>
+    <t>MLDS</t>
+  </si>
+  <si>
+    <t>Instruction metadata extraction from REDCap DD</t>
+  </si>
+  <si>
+    <t>ID-121</t>
+  </si>
+  <si>
+    <t>On hold- need more info</t>
+  </si>
+  <si>
+    <t>Instruction</t>
+  </si>
+  <si>
+    <t>BIDs run label not in chronological order</t>
+  </si>
+  <si>
+    <t>ID-128</t>
+  </si>
+  <si>
+    <t>Run ID</t>
+  </si>
+  <si>
+    <t>BISQR: infant sleep score - need to add</t>
+  </si>
+  <si>
+    <t>ID-134</t>
+  </si>
+  <si>
+    <t>BISQ-SF</t>
+  </si>
+  <si>
+    <t>pex_bm_healthv2_preg__exp__pnv_007__01 is completely blank</t>
+  </si>
+  <si>
+    <t>Stephanie Averill</t>
+  </si>
+  <si>
+    <t>ID-137</t>
+  </si>
+  <si>
+    <t>Healthv2 Preg</t>
+  </si>
+  <si>
+    <t>aspirin items in health v2 preg</t>
+  </si>
+  <si>
+    <t>ID-138</t>
+  </si>
+  <si>
+    <t>DD 'instruction' field all blank</t>
+  </si>
+  <si>
+    <t>ID-142</t>
+  </si>
+  <si>
+    <t>8 PNR not administered V1 portion of TLFB</t>
+  </si>
+  <si>
+    <t>Stephanie Averill, Santiago Torres Gomez</t>
+  </si>
+  <si>
+    <t>ID-144</t>
+  </si>
+  <si>
+    <t>Early Child Care and Education</t>
+  </si>
+  <si>
+    <t>regis.ongaro-carcy@mcin.ca</t>
+  </si>
+  <si>
+    <t>ID-146</t>
+  </si>
+  <si>
+    <t>ECHO</t>
+  </si>
+  <si>
+    <t>[DATA ISSUE] Diffusion MRI</t>
+  </si>
+  <si>
+    <t>ID-154</t>
+  </si>
+  <si>
+    <t>dMRI metadata</t>
+  </si>
+  <si>
+    <t>Add tabulated MR raw data QC</t>
+  </si>
+  <si>
+    <t>ID-155</t>
+  </si>
+  <si>
+    <t>Raw QC Metrics</t>
+  </si>
+  <si>
+    <t>[DATA ERROR]- age fields tied to visit start date</t>
+  </si>
+  <si>
+    <t>ID-55</t>
+  </si>
+  <si>
+    <t>EEG</t>
+  </si>
+  <si>
+    <t>Age fields</t>
+  </si>
+  <si>
+    <t>Gabi raw BIDs</t>
+  </si>
+  <si>
+    <t>30.0</t>
+  </si>
+  <si>
+    <t>Cecile Madjar, Harshitha Anuganti, Jesse Erdmann</t>
+  </si>
+  <si>
+    <t>ID-654</t>
+  </si>
+  <si>
+    <t>Archived to BR</t>
+  </si>
+  <si>
+    <t>GABI</t>
+  </si>
+  <si>
+    <t>MADE v1.7.0</t>
+  </si>
+  <si>
+    <t>Tanya Pandhi</t>
+  </si>
+  <si>
+    <t>ID-655</t>
+  </si>
+  <si>
+    <t>Add DICOMs to release</t>
+  </si>
+  <si>
+    <t>ID-657</t>
+  </si>
+  <si>
+    <t>Source DICOMs</t>
+  </si>
+  <si>
+    <t>MacArthur-Bates CDI-2 Language</t>
+  </si>
+  <si>
+    <t>ID-661</t>
+  </si>
+  <si>
+    <t>CDI-2</t>
+  </si>
+  <si>
+    <t>Medical History version 1</t>
+  </si>
+  <si>
+    <t>ID-662</t>
+  </si>
+  <si>
+    <t>Med History V1</t>
+  </si>
+  <si>
+    <t>Child Nutrition Questionnaire</t>
+  </si>
+  <si>
+    <t>ID-62</t>
+  </si>
+  <si>
+    <t>Child Nutrition</t>
+  </si>
+  <si>
+    <t>Deferred Imitation Task: Gong and Berry-Go-Round</t>
+  </si>
+  <si>
+    <t>ID-63</t>
+  </si>
+  <si>
+    <t>Deferred Imitation</t>
+  </si>
+  <si>
+    <t>Demographics V6 Adult</t>
+  </si>
+  <si>
+    <t>ID-64</t>
+  </si>
+  <si>
+    <t>Modified Checklist for Autism in Toddlers (MCHAT)</t>
+  </si>
+  <si>
+    <t>ID-69</t>
+  </si>
+  <si>
+    <t>MCHAT</t>
+  </si>
+  <si>
+    <t>PEDsQL</t>
+  </si>
+  <si>
+    <t>ID-70</t>
+  </si>
+  <si>
+    <t>Incarceration Questionnaire</t>
+  </si>
+  <si>
+    <t>ID-67</t>
   </si>
   <si>
     <t>All decline to answer will still report as zero - eHITS</t>
@@ -245,57 +776,12 @@
     <t>ID-38</t>
   </si>
   <si>
-    <t>Social &amp; Environmental Determinants</t>
+    <t>Add to archive</t>
   </si>
   <si>
     <t>eHITS</t>
   </si>
   <si>
-    <t>[TYPE_DATA INCORRECT] - ph_ch_anthro_average_bmi</t>
-  </si>
-  <si>
-    <t>ID-40</t>
-  </si>
-  <si>
-    <t>[DD+DATA ERROR] Nail type field added for 2.0 all "Unknown"</t>
-  </si>
-  <si>
-    <t>ID-42</t>
-  </si>
-  <si>
-    <t>Biospecimens &amp; Omics</t>
-  </si>
-  <si>
-    <t>Nails</t>
-  </si>
-  <si>
-    <t>[DATA REQUEST]- consistent ICD code names</t>
-  </si>
-  <si>
-    <t>ID-43</t>
-  </si>
-  <si>
-    <t>Pregnancy &amp; Environmental Exposure</t>
-  </si>
-  <si>
-    <t>PEX Health</t>
-  </si>
-  <si>
-    <t>Inclusion of Blood Spot Card Results data from USDTL. Addressing issue of incorrect cleaning practices at sites that affect test results PEth.</t>
-  </si>
-  <si>
-    <t>ID-44</t>
-  </si>
-  <si>
-    <t>Blood</t>
-  </si>
-  <si>
-    <t>[DATA REQUEST] ERICA - add age &amp; date_taken fields back to ERICA</t>
-  </si>
-  <si>
-    <t>ID-45</t>
-  </si>
-  <si>
     <t>[SCORING CORRECTION NEEDED]- EPDS</t>
   </si>
   <si>
@@ -305,69 +791,6 @@
     <t>EPDS</t>
   </si>
   <si>
-    <t>Anthro: ph_ch_anthro_head_for_age_boys_z_score</t>
-  </si>
-  <si>
-    <t>ID-48</t>
-  </si>
-  <si>
-    <t>[DATA REQUEST]-household roster - sex variable</t>
-  </si>
-  <si>
-    <t>ID-50</t>
-  </si>
-  <si>
-    <t>Demo</t>
-  </si>
-  <si>
-    <t>[POSSIBLE DATA ERROR]- relationship status at V03</t>
-  </si>
-  <si>
-    <t>ID-53</t>
-  </si>
-  <si>
-    <t>Bayley invalid subscores (-9999) (parameter-based filtering)</t>
-  </si>
-  <si>
-    <t>ID-54</t>
-  </si>
-  <si>
-    <t>Neurocognition &amp; Language</t>
-  </si>
-  <si>
-    <t>Bayley</t>
-  </si>
-  <si>
-    <t>[IMAGING] MRI bad frame removal workflow</t>
-  </si>
-  <si>
-    <t>Tanya Pandhi, Cecile Madjar</t>
-  </si>
-  <si>
-    <t>ID-59</t>
-  </si>
-  <si>
-    <t>fmap QC</t>
-  </si>
-  <si>
-    <t>[POSSIBLE DATA ERROR]- roster at V02 or V03 (parameter-based filtering is precursor)</t>
-  </si>
-  <si>
-    <t>ID-60</t>
-  </si>
-  <si>
-    <t>Geocoded Linkage from Home and Work Addresses</t>
-  </si>
-  <si>
-    <t>Matthew Schmidt</t>
-  </si>
-  <si>
-    <t>ID-66</t>
-  </si>
-  <si>
-    <t>GLED</t>
-  </si>
-  <si>
     <t>MAPS-EASI- Toddler</t>
   </si>
   <si>
@@ -377,382 +800,13 @@
     <t>MAPS-EASI</t>
   </si>
   <si>
-    <t>Transition in Care Questionnaire</t>
-  </si>
-  <si>
-    <t>Tim Meyer, Stephanie Averill, regis.ongaro-carcy@mcin.ca</t>
-  </si>
-  <si>
-    <t>ID-71</t>
-  </si>
-  <si>
-    <t>TIC Questionnaire</t>
-  </si>
-  <si>
-    <t>[DATA ISSUE] - cdiwgen values over 100</t>
-  </si>
-  <si>
-    <t>ID-78</t>
-  </si>
-  <si>
-    <t>CDI</t>
-  </si>
-  <si>
-    <t>Participant status and withdrawal field harmonization</t>
-  </si>
-  <si>
-    <t>Dan Duhon, Matthew Schmidt</t>
-  </si>
-  <si>
-    <t>ID-79</t>
-  </si>
-  <si>
-    <t>Visit Info</t>
-  </si>
-  <si>
-    <t>[DATA ISSUE] - VABS reasons for missingness are wrong</t>
-  </si>
-  <si>
-    <t>ID-80</t>
-  </si>
-  <si>
-    <t>Vineland</t>
-  </si>
-  <si>
     <t>[DATA ISSUE]- Screen_mother_race_multi  majority are 0</t>
   </si>
   <si>
     <t>ID-81</t>
   </si>
   <si>
-    <t>Update JSON metadata to match Lasso/DEAP updates</t>
-  </si>
-  <si>
-    <t>ID-83</t>
-  </si>
-  <si>
-    <t>Incorrect JSONs</t>
-  </si>
-  <si>
-    <t>Cleanup crew: Inclusion of family pregnancy ID</t>
-  </si>
-  <si>
-    <t>ID-84</t>
-  </si>
-  <si>
-    <t>FamilyID</t>
-  </si>
-  <si>
-    <t>MRI Derivatives - QSIprep - Generate tabular data for QSIRECON</t>
-  </si>
-  <si>
-    <t>Cecile Madjar</t>
-  </si>
-  <si>
-    <t>ID-86</t>
-  </si>
-  <si>
-    <t>QSIRecon</t>
-  </si>
-  <si>
-    <t>XCP-D corrections and model output</t>
-  </si>
-  <si>
-    <t>Tanya Pandhi, Lucille Moore</t>
-  </si>
-  <si>
-    <t>ID-87</t>
-  </si>
-  <si>
-    <t>Postprocessing</t>
-  </si>
-  <si>
-    <t>[DATA REQUESTs] - novel tech QC feedback overview</t>
-  </si>
-  <si>
-    <t>ID-102</t>
-  </si>
-  <si>
-    <t>Novel Tech &amp; Wearable Sensors</t>
-  </si>
-  <si>
-    <t>unsure</t>
-  </si>
-  <si>
-    <t>TBD</t>
-  </si>
-  <si>
-    <t>[DATA ERRORS]- static table QC feedback</t>
-  </si>
-  <si>
-    <t>ID-106</t>
-  </si>
-  <si>
-    <t>UNSURE</t>
-  </si>
-  <si>
-    <t>Add scanner info as tabulated data</t>
-  </si>
-  <si>
-    <t>ID-108</t>
-  </si>
-  <si>
-    <t>Scanner info</t>
-  </si>
-  <si>
-    <t>[DATA ERROR]- home 21</t>
-  </si>
-  <si>
-    <t>New; needs discussion</t>
-  </si>
-  <si>
-    <t>ID-666</t>
-  </si>
-  <si>
-    <t>Tabulated XCP-D derivatives all 0s for numeric fields</t>
-  </si>
-  <si>
-    <t>ID-667</t>
-  </si>
-  <si>
-    <t>br_known_issue</t>
-  </si>
-  <si>
-    <t>[DATA REQUEST]- revise formatting of vision screener files</t>
-  </si>
-  <si>
-    <t>ID-109</t>
-  </si>
-  <si>
-    <t>Vision Screener</t>
-  </si>
-  <si>
-    <t>Remove 'sequence' field from all tables in Lasso</t>
-  </si>
-  <si>
-    <t>Not started yet</t>
-  </si>
-  <si>
-    <t>ID-110</t>
-  </si>
-  <si>
-    <t>Sequence Field</t>
-  </si>
-  <si>
-    <t>[DATA ERROR]-MLDS  total hours per week of non-parental hours</t>
-  </si>
-  <si>
-    <t>ID-119</t>
-  </si>
-  <si>
-    <t>MLDS</t>
-  </si>
-  <si>
-    <t>Instruction metadata extraction from REDCap DD</t>
-  </si>
-  <si>
-    <t>ID-121</t>
-  </si>
-  <si>
-    <t>On hold- need more info</t>
-  </si>
-  <si>
-    <t>Instruction</t>
-  </si>
-  <si>
-    <t>BIDs run label not in chronological order</t>
-  </si>
-  <si>
-    <t>ID-128</t>
-  </si>
-  <si>
-    <t>Run ID</t>
-  </si>
-  <si>
-    <t>BISQR: infant sleep score - need to add</t>
-  </si>
-  <si>
-    <t>ID-134</t>
-  </si>
-  <si>
-    <t>BISQ-SF</t>
-  </si>
-  <si>
-    <t>pex_bm_healthv2_preg__exp__pnv_007__01 is completely blank</t>
-  </si>
-  <si>
-    <t>Stephanie Averill</t>
-  </si>
-  <si>
-    <t>ID-137</t>
-  </si>
-  <si>
-    <t>Healthv2 Preg</t>
-  </si>
-  <si>
-    <t>aspirin items in health v2 preg</t>
-  </si>
-  <si>
-    <t>ID-138</t>
-  </si>
-  <si>
-    <t>DD 'instruction' field all blank</t>
-  </si>
-  <si>
-    <t>ID-142</t>
-  </si>
-  <si>
-    <t>8 PNR not administered V1 portion of TLFB</t>
-  </si>
-  <si>
-    <t>Stephanie Averill, Santiago Torres Gomez</t>
-  </si>
-  <si>
-    <t>ID-144</t>
-  </si>
-  <si>
-    <t>Early Child Care and Education</t>
-  </si>
-  <si>
-    <t>regis.ongaro-carcy@mcin.ca</t>
-  </si>
-  <si>
-    <t>ID-146</t>
-  </si>
-  <si>
-    <t>ECHO</t>
-  </si>
-  <si>
-    <t>[DATA ISSUE] Diffusion MRI</t>
-  </si>
-  <si>
-    <t>ID-154</t>
-  </si>
-  <si>
-    <t>dMRI metadata</t>
-  </si>
-  <si>
-    <t>Add tabulated MR raw data QC</t>
-  </si>
-  <si>
-    <t>ID-155</t>
-  </si>
-  <si>
-    <t>Raw QC Metrics</t>
-  </si>
-  <si>
-    <t>[DATA ERROR]- age fields tied to visit start date</t>
-  </si>
-  <si>
-    <t>ID-55</t>
-  </si>
-  <si>
-    <t>EEG</t>
-  </si>
-  <si>
-    <t>Age fields</t>
-  </si>
-  <si>
-    <t>Gabi raw BIDs</t>
-  </si>
-  <si>
-    <t>30.0</t>
-  </si>
-  <si>
-    <t>Cecile Madjar, Harshitha Anuganti, Jesse Erdmann</t>
-  </si>
-  <si>
-    <t>ID-654</t>
-  </si>
-  <si>
-    <t>Archived to BR</t>
-  </si>
-  <si>
-    <t>GABI</t>
-  </si>
-  <si>
-    <t>MADE v1.7.0</t>
-  </si>
-  <si>
-    <t>Tanya Pandhi</t>
-  </si>
-  <si>
-    <t>ID-655</t>
-  </si>
-  <si>
-    <t>Add DICOMs to release</t>
-  </si>
-  <si>
-    <t>ID-657</t>
-  </si>
-  <si>
-    <t>Source DICOMs</t>
-  </si>
-  <si>
-    <t>MacArthur-Bates CDI-2 Language</t>
-  </si>
-  <si>
-    <t>ID-661</t>
-  </si>
-  <si>
-    <t>CDI-2</t>
-  </si>
-  <si>
-    <t>Medical History version 1</t>
-  </si>
-  <si>
-    <t>ID-662</t>
-  </si>
-  <si>
-    <t>Med History V1</t>
-  </si>
-  <si>
-    <t>Child Nutrition Questionnaire</t>
-  </si>
-  <si>
-    <t>ID-62</t>
-  </si>
-  <si>
-    <t>Child Nutrition</t>
-  </si>
-  <si>
-    <t>Deferred Imitation Task: Gong and Berry-Go-Round</t>
-  </si>
-  <si>
-    <t>ID-63</t>
-  </si>
-  <si>
-    <t>Deferred Imitation</t>
-  </si>
-  <si>
-    <t>Demographics V6 Adult</t>
-  </si>
-  <si>
-    <t>ID-64</t>
-  </si>
-  <si>
-    <t>Modified Checklist for Autism in Toddlers (MCHAT)</t>
-  </si>
-  <si>
-    <t>ID-69</t>
-  </si>
-  <si>
-    <t>MCHAT</t>
-  </si>
-  <si>
-    <t>PEDsQL</t>
-  </si>
-  <si>
-    <t>ID-70</t>
-  </si>
-  <si>
-    <t>Incarceration Questionnaire</t>
-  </si>
-  <si>
-    <t>ID-67</t>
-  </si>
-  <si>
-    <t>Incarceration</t>
+    <t>Static table</t>
   </si>
 </sst>
 </file>
@@ -778,7 +832,7 @@
       <name val="Calibri"/>
     </font>
   </fonts>
-  <fills count="22">
+  <fills count="24">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -797,7 +851,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF563E3E"/>
+        <fgColor rgb="FFFDAB3D"/>
       </patternFill>
     </fill>
     <fill>
@@ -812,7 +866,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF9D50DD"/>
+        <fgColor rgb="FF037F4C"/>
       </patternFill>
     </fill>
     <fill>
@@ -837,17 +891,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFBB3354"/>
+        <fgColor rgb="FF579BFC"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFDAB3D"/>
+        <fgColor rgb="FF9D50DD"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF037F4C"/>
+        <fgColor rgb="FF563E3E"/>
       </patternFill>
     </fill>
     <fill>
@@ -863,6 +917,16 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFCB00"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFBB3354"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF7F5347"/>
       </patternFill>
     </fill>
     <fill>
@@ -898,7 +962,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -964,6 +1028,12 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="21" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="22" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="23" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1305,7 +1375,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:L69"/>
+  <dimension ref="A1:L73"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="150" customWidth="1"/>
@@ -1410,16 +1480,16 @@
         <v>23</v>
       </c>
       <c r="E3" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="F3" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="F3" s="9" t="s">
+      <c r="G3" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="G3" s="3" t="s">
+      <c r="H3" s="10" t="s">
         <v>26</v>
-      </c>
-      <c r="H3" s="10" t="s">
-        <v>27</v>
       </c>
       <c r="I3" s="7" t="s">
         <v>18</v>
@@ -1428,7 +1498,7 @@
         <v>19</v>
       </c>
       <c r="K3" s="3" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="L3" s="6" t="s">
         <v>21</v>
@@ -1436,7 +1506,7 @@
     </row>
     <row r="4" spans="1:12" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B4" s="3">
         <v>3</v>
@@ -1448,7 +1518,7 @@
         <v>13</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="F4" s="11" t="s">
         <v>30</v>
@@ -1482,22 +1552,22 @@
       <c r="C5" s="3">
         <v>30</v>
       </c>
-      <c r="D5" s="8" t="s">
-        <v>23</v>
+      <c r="D5" s="13" t="s">
+        <v>35</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="F5" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="F5" s="10" t="s">
         <v>36</v>
       </c>
       <c r="G5" s="3" t="s">
         <v>37</v>
       </c>
       <c r="H5" s="10" t="s">
-        <v>27</v>
-      </c>
-      <c r="I5" s="14" t="s">
+        <v>26</v>
+      </c>
+      <c r="I5" s="5" t="s">
         <v>38</v>
       </c>
       <c r="J5" s="6" t="s">
@@ -1520,20 +1590,20 @@
       <c r="C6" s="3">
         <v>30</v>
       </c>
-      <c r="D6" s="8" t="s">
-        <v>23</v>
+      <c r="D6" s="13" t="s">
+        <v>35</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="F6" s="13" t="s">
-        <v>36</v>
+        <v>14</v>
+      </c>
+      <c r="F6" s="5" t="s">
+        <v>15</v>
       </c>
       <c r="G6" s="3" t="s">
         <v>41</v>
       </c>
       <c r="H6" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="I6" s="7" t="s">
         <v>18</v>
@@ -1558,29 +1628,29 @@
       <c r="C7" s="3">
         <v>30</v>
       </c>
-      <c r="D7" s="8" t="s">
-        <v>23</v>
+      <c r="D7" s="14" t="s">
+        <v>44</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="F7" s="13" t="s">
-        <v>36</v>
+        <v>45</v>
+      </c>
+      <c r="F7" s="15" t="s">
+        <v>46</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="H7" s="10" t="s">
-        <v>27</v>
-      </c>
-      <c r="I7" s="14" t="s">
+        <v>26</v>
+      </c>
+      <c r="I7" s="5" t="s">
         <v>38</v>
       </c>
       <c r="J7" s="6" t="s">
         <v>19</v>
       </c>
       <c r="K7" s="3" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="L7" s="6" t="s">
         <v>21</v>
@@ -1588,7 +1658,7 @@
     </row>
     <row r="8" spans="1:12" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="2" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="B8" s="3">
         <v>3</v>
@@ -1596,20 +1666,20 @@
       <c r="C8" s="3">
         <v>30</v>
       </c>
-      <c r="D8" s="15" t="s">
-        <v>47</v>
+      <c r="D8" s="8" t="s">
+        <v>23</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="F8" s="14" t="s">
-        <v>48</v>
+        <v>45</v>
+      </c>
+      <c r="F8" s="5" t="s">
+        <v>15</v>
       </c>
       <c r="G8" s="3" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="H8" s="16" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="I8" s="7" t="s">
         <v>18</v>
@@ -1618,7 +1688,7 @@
         <v>19</v>
       </c>
       <c r="K8" s="3" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="L8" s="6" t="s">
         <v>21</v>
@@ -1626,7 +1696,7 @@
     </row>
     <row r="9" spans="1:12" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="2" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B9" s="3">
         <v>3</v>
@@ -1634,29 +1704,29 @@
       <c r="C9" s="3">
         <v>30</v>
       </c>
-      <c r="D9" s="8" t="s">
-        <v>23</v>
+      <c r="D9" s="13" t="s">
+        <v>35</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="F9" s="13" t="s">
-        <v>36</v>
+        <v>14</v>
+      </c>
+      <c r="F9" s="9" t="s">
+        <v>24</v>
       </c>
       <c r="G9" s="3" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="H9" s="10" t="s">
-        <v>27</v>
-      </c>
-      <c r="I9" s="14" t="s">
+        <v>26</v>
+      </c>
+      <c r="I9" s="5" t="s">
         <v>38</v>
       </c>
       <c r="J9" s="6" t="s">
         <v>19</v>
       </c>
       <c r="K9" s="3" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="L9" s="6" t="s">
         <v>21</v>
@@ -1664,7 +1734,7 @@
     </row>
     <row r="10" spans="1:12" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="2" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B10" s="3">
         <v>3</v>
@@ -1672,29 +1742,29 @@
       <c r="C10" s="3">
         <v>30.1</v>
       </c>
-      <c r="D10" s="15" t="s">
-        <v>47</v>
+      <c r="D10" s="8" t="s">
+        <v>23</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="F10" s="14" t="s">
-        <v>48</v>
+        <v>57</v>
+      </c>
+      <c r="F10" s="5" t="s">
+        <v>15</v>
       </c>
       <c r="G10" s="3" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="H10" s="12" t="s">
         <v>32</v>
       </c>
-      <c r="I10" s="14" t="s">
+      <c r="I10" s="5" t="s">
         <v>38</v>
       </c>
       <c r="J10" s="6" t="s">
         <v>19</v>
       </c>
       <c r="K10" s="3" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="L10" s="6" t="s">
         <v>21</v>
@@ -1702,7 +1772,7 @@
     </row>
     <row r="11" spans="1:12" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="2" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B11" s="3">
         <v>3</v>
@@ -1714,10 +1784,10 @@
         <v>13</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="F11" s="10" t="s">
-        <v>60</v>
+        <v>14</v>
+      </c>
+      <c r="F11" s="5" t="s">
+        <v>15</v>
       </c>
       <c r="G11" s="3" t="s">
         <v>61</v>
@@ -1725,7 +1795,7 @@
       <c r="H11" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="I11" s="14" t="s">
+      <c r="I11" s="5" t="s">
         <v>38</v>
       </c>
       <c r="J11" s="6" t="s">
@@ -1752,25 +1822,25 @@
         <v>13</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>63</v>
+        <v>29</v>
       </c>
       <c r="F12" s="11" t="s">
         <v>30</v>
       </c>
       <c r="G12" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="H12" s="17" t="s">
         <v>64</v>
       </c>
-      <c r="H12" s="17" t="s">
+      <c r="I12" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="J12" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="K12" s="3" t="s">
         <v>65</v>
-      </c>
-      <c r="I12" s="14" t="s">
-        <v>38</v>
-      </c>
-      <c r="J12" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="K12" s="3" t="s">
-        <v>66</v>
       </c>
       <c r="L12" s="6" t="s">
         <v>21</v>
@@ -1778,7 +1848,7 @@
     </row>
     <row r="13" spans="1:12" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B13" s="3">
         <v>3</v>
@@ -1786,29 +1856,29 @@
       <c r="C13" s="3">
         <v>30.2</v>
       </c>
-      <c r="D13" s="15" t="s">
-        <v>47</v>
+      <c r="D13" s="8" t="s">
+        <v>23</v>
       </c>
       <c r="E13" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="F13" s="14" t="s">
-        <v>48</v>
+        <v>14</v>
+      </c>
+      <c r="F13" s="5" t="s">
+        <v>15</v>
       </c>
       <c r="G13" s="3" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="H13" s="12" t="s">
         <v>32</v>
       </c>
-      <c r="I13" s="14" t="s">
+      <c r="I13" s="5" t="s">
         <v>38</v>
       </c>
       <c r="J13" s="6" t="s">
         <v>19</v>
       </c>
       <c r="K13" s="3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="L13" s="6" t="s">
         <v>21</v>
@@ -1816,19 +1886,19 @@
     </row>
     <row r="14" spans="1:12" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="2" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B14" s="3">
         <v>3</v>
       </c>
       <c r="C14" t="s">
-        <v>13</v>
+        <v>70</v>
       </c>
       <c r="D14" s="4" t="s">
         <v>13</v>
       </c>
       <c r="E14" s="3" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="F14" s="12" t="s">
         <v>71</v>
@@ -1837,9 +1907,9 @@
         <v>72</v>
       </c>
       <c r="H14" s="17" t="s">
-        <v>65</v>
-      </c>
-      <c r="I14" s="14" t="s">
+        <v>64</v>
+      </c>
+      <c r="I14" s="5" t="s">
         <v>38</v>
       </c>
       <c r="J14" s="6" t="s">
@@ -1862,22 +1932,22 @@
       <c r="C15" s="3">
         <v>30.1</v>
       </c>
-      <c r="D15" s="8" t="s">
-        <v>23</v>
+      <c r="D15" s="4" t="s">
+        <v>13</v>
       </c>
       <c r="E15" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="F15" s="9" t="s">
-        <v>25</v>
+        <v>14</v>
+      </c>
+      <c r="F15" s="5" t="s">
+        <v>15</v>
       </c>
       <c r="G15" s="3" t="s">
         <v>75</v>
       </c>
-      <c r="H15" s="8" t="s">
+      <c r="H15" s="18" t="s">
         <v>76</v>
       </c>
-      <c r="I15" s="14" t="s">
+      <c r="I15" s="5" t="s">
         <v>38</v>
       </c>
       <c r="J15" s="6" t="s">
@@ -1898,31 +1968,31 @@
         <v>3</v>
       </c>
       <c r="C16" s="3">
-        <v>30.2</v>
-      </c>
-      <c r="D16" s="15" t="s">
-        <v>47</v>
+        <v>30.1</v>
+      </c>
+      <c r="D16" s="4" t="s">
+        <v>13</v>
       </c>
       <c r="E16" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="F16" s="14" t="s">
-        <v>48</v>
+        <v>14</v>
+      </c>
+      <c r="F16" s="10" t="s">
+        <v>36</v>
       </c>
       <c r="G16" s="3" t="s">
         <v>79</v>
       </c>
-      <c r="H16" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="I16" s="14" t="s">
-        <v>38</v>
+      <c r="H16" s="5" t="s">
+        <v>80</v>
+      </c>
+      <c r="I16" s="7" t="s">
+        <v>18</v>
       </c>
       <c r="J16" s="6" t="s">
         <v>19</v>
       </c>
       <c r="K16" s="3" t="s">
-        <v>20</v>
+        <v>81</v>
       </c>
       <c r="L16" s="6" t="s">
         <v>21</v>
@@ -1930,37 +2000,37 @@
     </row>
     <row r="17" spans="1:12" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="2" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B17" s="3">
         <v>3</v>
       </c>
       <c r="C17" s="3">
-        <v>30.2</v>
-      </c>
-      <c r="D17" s="15" t="s">
-        <v>47</v>
+        <v>30.1</v>
+      </c>
+      <c r="D17" s="14" t="s">
+        <v>44</v>
       </c>
       <c r="E17" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="F17" s="14" t="s">
-        <v>48</v>
+        <v>45</v>
+      </c>
+      <c r="F17" s="19" t="s">
+        <v>83</v>
       </c>
       <c r="G17" s="3" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="H17" s="18" t="s">
-        <v>82</v>
-      </c>
-      <c r="I17" s="14" t="s">
-        <v>38</v>
+        <v>76</v>
+      </c>
+      <c r="I17" s="7" t="s">
+        <v>18</v>
       </c>
       <c r="J17" s="6" t="s">
         <v>19</v>
       </c>
       <c r="K17" s="3" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="L17" s="6" t="s">
         <v>21</v>
@@ -1968,28 +2038,28 @@
     </row>
     <row r="18" spans="1:12" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="2" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="B18" s="3">
         <v>3</v>
       </c>
       <c r="C18" s="3">
-        <v>30.1</v>
-      </c>
-      <c r="D18" s="4" t="s">
-        <v>13</v>
+        <v>30.2</v>
+      </c>
+      <c r="D18" s="8" t="s">
+        <v>23</v>
       </c>
       <c r="E18" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="F18" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="F18" s="10" t="s">
-        <v>60</v>
-      </c>
       <c r="G18" s="3" t="s">
-        <v>85</v>
-      </c>
-      <c r="H18" s="14" t="s">
-        <v>86</v>
+        <v>87</v>
+      </c>
+      <c r="H18" s="10" t="s">
+        <v>26</v>
       </c>
       <c r="I18" s="7" t="s">
         <v>18</v>
@@ -1998,7 +2068,7 @@
         <v>19</v>
       </c>
       <c r="K18" s="3" t="s">
-        <v>87</v>
+        <v>27</v>
       </c>
       <c r="L18" s="6" t="s">
         <v>21</v>
@@ -2014,29 +2084,29 @@
       <c r="C19" s="3">
         <v>30.1</v>
       </c>
-      <c r="D19" s="8" t="s">
-        <v>23</v>
+      <c r="D19" s="4" t="s">
+        <v>13</v>
       </c>
       <c r="E19" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="F19" s="9" t="s">
         <v>24</v>
-      </c>
-      <c r="F19" s="9" t="s">
-        <v>25</v>
       </c>
       <c r="G19" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="H19" s="18" t="s">
-        <v>82</v>
-      </c>
-      <c r="I19" s="7" t="s">
-        <v>18</v>
+      <c r="H19" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="I19" s="5" t="s">
+        <v>38</v>
       </c>
       <c r="J19" s="6" t="s">
         <v>19</v>
       </c>
       <c r="K19" s="3" t="s">
-        <v>90</v>
+        <v>20</v>
       </c>
       <c r="L19" s="6" t="s">
         <v>21</v>
@@ -2044,37 +2114,37 @@
     </row>
     <row r="20" spans="1:12" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="B20" s="3">
+        <v>3</v>
+      </c>
+      <c r="C20" s="3">
+        <v>30.1</v>
+      </c>
+      <c r="D20" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="E20" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="F20" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="G20" s="3" t="s">
         <v>91</v>
       </c>
-      <c r="B20" s="3">
-        <v>3</v>
-      </c>
-      <c r="C20" s="3">
-        <v>30.2</v>
-      </c>
-      <c r="D20" s="15" t="s">
-        <v>47</v>
-      </c>
-      <c r="E20" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="F20" s="14" t="s">
-        <v>48</v>
-      </c>
-      <c r="G20" s="3" t="s">
-        <v>92</v>
-      </c>
-      <c r="H20" s="10" t="s">
-        <v>27</v>
-      </c>
-      <c r="I20" s="7" t="s">
-        <v>18</v>
+      <c r="H20" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="I20" s="5" t="s">
+        <v>38</v>
       </c>
       <c r="J20" s="6" t="s">
         <v>19</v>
       </c>
       <c r="K20" s="3" t="s">
-        <v>28</v>
+        <v>20</v>
       </c>
       <c r="L20" s="6" t="s">
         <v>21</v>
@@ -2082,31 +2152,31 @@
     </row>
     <row r="21" spans="1:12" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="2" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B21" s="3">
         <v>3</v>
       </c>
       <c r="C21" s="3">
-        <v>30</v>
+        <v>30.1</v>
       </c>
       <c r="D21" s="8" t="s">
         <v>23</v>
       </c>
       <c r="E21" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="F21" s="13" t="s">
-        <v>36</v>
+        <v>14</v>
+      </c>
+      <c r="F21" s="5" t="s">
+        <v>15</v>
       </c>
       <c r="G21" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="H21" s="14" t="s">
         <v>94</v>
       </c>
-      <c r="H21" s="14" t="s">
-        <v>86</v>
-      </c>
-      <c r="I21" s="14" t="s">
-        <v>38</v>
+      <c r="I21" s="7" t="s">
+        <v>18</v>
       </c>
       <c r="J21" s="6" t="s">
         <v>19</v>
@@ -2126,13 +2196,13 @@
         <v>3</v>
       </c>
       <c r="C22" s="3">
-        <v>30.1</v>
-      </c>
-      <c r="D22" s="4" t="s">
-        <v>13</v>
+        <v>30.2</v>
+      </c>
+      <c r="D22" s="8" t="s">
+        <v>23</v>
       </c>
       <c r="E22" s="3" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="F22" s="5" t="s">
         <v>15</v>
@@ -2140,17 +2210,17 @@
       <c r="G22" s="3" t="s">
         <v>97</v>
       </c>
-      <c r="H22" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="I22" s="14" t="s">
+      <c r="H22" s="14" t="s">
+        <v>94</v>
+      </c>
+      <c r="I22" s="5" t="s">
         <v>38</v>
       </c>
       <c r="J22" s="6" t="s">
         <v>19</v>
       </c>
       <c r="K22" s="3" t="s">
-        <v>20</v>
+        <v>95</v>
       </c>
       <c r="L22" s="6" t="s">
         <v>21</v>
@@ -2164,31 +2234,31 @@
         <v>3</v>
       </c>
       <c r="C23" s="3">
-        <v>30.1</v>
-      </c>
-      <c r="D23" s="15" t="s">
-        <v>47</v>
+        <v>30.2</v>
+      </c>
+      <c r="D23" s="13" t="s">
+        <v>35</v>
       </c>
       <c r="E23" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="F23" s="14" t="s">
-        <v>48</v>
+        <v>14</v>
+      </c>
+      <c r="F23" s="20" t="s">
+        <v>99</v>
       </c>
       <c r="G23" s="3" t="s">
-        <v>99</v>
-      </c>
-      <c r="H23" s="8" t="s">
-        <v>76</v>
-      </c>
-      <c r="I23" s="7" t="s">
-        <v>18</v>
+        <v>100</v>
+      </c>
+      <c r="H23" s="15" t="s">
+        <v>101</v>
+      </c>
+      <c r="I23" s="5" t="s">
+        <v>38</v>
       </c>
       <c r="J23" s="6" t="s">
         <v>19</v>
       </c>
       <c r="K23" s="3" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="L23" s="6" t="s">
         <v>21</v>
@@ -2196,37 +2266,37 @@
     </row>
     <row r="24" spans="1:12" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="2" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="B24" s="3">
         <v>3</v>
       </c>
       <c r="C24" s="3">
-        <v>30.2</v>
-      </c>
-      <c r="D24" s="15" t="s">
-        <v>47</v>
+        <v>30.1</v>
+      </c>
+      <c r="D24" s="8" t="s">
+        <v>23</v>
       </c>
       <c r="E24" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="F24" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="F24" s="14" t="s">
-        <v>48</v>
-      </c>
       <c r="G24" s="3" t="s">
-        <v>102</v>
-      </c>
-      <c r="H24" s="8" t="s">
-        <v>76</v>
-      </c>
-      <c r="I24" s="14" t="s">
-        <v>38</v>
+        <v>105</v>
+      </c>
+      <c r="H24" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="I24" s="7" t="s">
+        <v>18</v>
       </c>
       <c r="J24" s="6" t="s">
         <v>19</v>
       </c>
       <c r="K24" s="3" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="L24" s="6" t="s">
         <v>21</v>
@@ -2234,37 +2304,37 @@
     </row>
     <row r="25" spans="1:12" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="2" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="B25" s="3">
         <v>3</v>
       </c>
       <c r="C25" s="3">
-        <v>30.2</v>
-      </c>
-      <c r="D25" s="15" t="s">
-        <v>47</v>
+        <v>30.1</v>
+      </c>
+      <c r="D25" s="14" t="s">
+        <v>44</v>
       </c>
       <c r="E25" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="F25" s="14" t="s">
-        <v>48</v>
+        <v>45</v>
+      </c>
+      <c r="F25" s="15" t="s">
+        <v>46</v>
       </c>
       <c r="G25" s="3" t="s">
-        <v>104</v>
-      </c>
-      <c r="H25" s="5" t="s">
-        <v>105</v>
-      </c>
-      <c r="I25" s="14" t="s">
+        <v>108</v>
+      </c>
+      <c r="H25" s="14" t="s">
+        <v>94</v>
+      </c>
+      <c r="I25" s="5" t="s">
         <v>38</v>
       </c>
       <c r="J25" s="6" t="s">
         <v>19</v>
       </c>
       <c r="K25" s="3" t="s">
-        <v>106</v>
+        <v>95</v>
       </c>
       <c r="L25" s="6" t="s">
         <v>21</v>
@@ -2272,7 +2342,7 @@
     </row>
     <row r="26" spans="1:12" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="2" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="B26" s="3">
         <v>3</v>
@@ -2280,20 +2350,20 @@
       <c r="C26" s="3">
         <v>30.1</v>
       </c>
-      <c r="D26" s="15" t="s">
-        <v>47</v>
+      <c r="D26" s="4" t="s">
+        <v>13</v>
       </c>
       <c r="E26" s="3" t="s">
-        <v>108</v>
-      </c>
-      <c r="F26" s="14" t="s">
-        <v>48</v>
+        <v>110</v>
+      </c>
+      <c r="F26" s="11" t="s">
+        <v>30</v>
       </c>
       <c r="G26" s="3" t="s">
-        <v>109</v>
-      </c>
-      <c r="H26" s="16" t="s">
-        <v>50</v>
+        <v>111</v>
+      </c>
+      <c r="H26" s="14" t="s">
+        <v>94</v>
       </c>
       <c r="I26" s="7" t="s">
         <v>18</v>
@@ -2302,7 +2372,7 @@
         <v>19</v>
       </c>
       <c r="K26" s="3" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="L26" s="6" t="s">
         <v>21</v>
@@ -2310,7 +2380,7 @@
     </row>
     <row r="27" spans="1:12" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="2" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="B27" s="3">
         <v>3</v>
@@ -2322,25 +2392,25 @@
         <v>23</v>
       </c>
       <c r="E27" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="F27" s="13" t="s">
-        <v>36</v>
+        <v>114</v>
+      </c>
+      <c r="F27" s="5" t="s">
+        <v>15</v>
       </c>
       <c r="G27" s="3" t="s">
-        <v>112</v>
-      </c>
-      <c r="H27" s="8" t="s">
-        <v>76</v>
-      </c>
-      <c r="I27" s="14" t="s">
-        <v>38</v>
+        <v>115</v>
+      </c>
+      <c r="H27" s="14" t="s">
+        <v>94</v>
+      </c>
+      <c r="I27" s="7" t="s">
+        <v>18</v>
       </c>
       <c r="J27" s="6" t="s">
         <v>19</v>
       </c>
       <c r="K27" s="3" t="s">
-        <v>100</v>
+        <v>116</v>
       </c>
       <c r="L27" s="6" t="s">
         <v>21</v>
@@ -2348,7 +2418,7 @@
     </row>
     <row r="28" spans="1:12" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="2" t="s">
-        <v>113</v>
+        <v>117</v>
       </c>
       <c r="B28" s="3">
         <v>3</v>
@@ -2356,29 +2426,29 @@
       <c r="C28" s="3">
         <v>30.1</v>
       </c>
-      <c r="D28" s="4" t="s">
-        <v>13</v>
+      <c r="D28" s="14" t="s">
+        <v>44</v>
       </c>
       <c r="E28" s="3" t="s">
-        <v>114</v>
-      </c>
-      <c r="F28" s="11" t="s">
-        <v>30</v>
+        <v>45</v>
+      </c>
+      <c r="F28" s="15" t="s">
+        <v>46</v>
       </c>
       <c r="G28" s="3" t="s">
-        <v>115</v>
-      </c>
-      <c r="H28" s="8" t="s">
-        <v>76</v>
-      </c>
-      <c r="I28" s="7" t="s">
-        <v>18</v>
+        <v>118</v>
+      </c>
+      <c r="H28" s="15" t="s">
+        <v>101</v>
+      </c>
+      <c r="I28" s="5" t="s">
+        <v>38</v>
       </c>
       <c r="J28" s="6" t="s">
         <v>19</v>
       </c>
       <c r="K28" s="3" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="L28" s="6" t="s">
         <v>21</v>
@@ -2386,37 +2456,37 @@
     </row>
     <row r="29" spans="1:12" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="2" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="B29" s="3">
         <v>3</v>
       </c>
       <c r="C29" s="3">
+        <v>30.1</v>
+      </c>
+      <c r="D29" s="13" t="s">
+        <v>35</v>
+      </c>
+      <c r="E29" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="F29" s="11" t="s">
         <v>30</v>
       </c>
-      <c r="D29" s="8" t="s">
-        <v>23</v>
-      </c>
-      <c r="E29" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="F29" s="13" t="s">
-        <v>36</v>
-      </c>
       <c r="G29" s="3" t="s">
-        <v>118</v>
-      </c>
-      <c r="H29" s="10" t="s">
-        <v>27</v>
-      </c>
-      <c r="I29" s="7" t="s">
-        <v>18</v>
+        <v>122</v>
+      </c>
+      <c r="H29" s="17" t="s">
+        <v>64</v>
+      </c>
+      <c r="I29" s="5" t="s">
+        <v>38</v>
       </c>
       <c r="J29" s="6" t="s">
         <v>19</v>
       </c>
       <c r="K29" s="3" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="L29" s="6" t="s">
         <v>21</v>
@@ -2424,7 +2494,7 @@
     </row>
     <row r="30" spans="1:12" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="2" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="B30" s="3">
         <v>3</v>
@@ -2432,29 +2502,29 @@
       <c r="C30" s="3">
         <v>30.1</v>
       </c>
-      <c r="D30" s="15" t="s">
-        <v>47</v>
+      <c r="D30" s="8" t="s">
+        <v>23</v>
       </c>
       <c r="E30" s="3" t="s">
-        <v>121</v>
-      </c>
-      <c r="F30" s="14" t="s">
-        <v>48</v>
+        <v>14</v>
+      </c>
+      <c r="F30" s="5" t="s">
+        <v>15</v>
       </c>
       <c r="G30" s="3" t="s">
-        <v>122</v>
-      </c>
-      <c r="H30" s="8" t="s">
-        <v>76</v>
-      </c>
-      <c r="I30" s="7" t="s">
-        <v>18</v>
+        <v>125</v>
+      </c>
+      <c r="H30" s="15" t="s">
+        <v>101</v>
+      </c>
+      <c r="I30" s="5" t="s">
+        <v>38</v>
       </c>
       <c r="J30" s="6" t="s">
         <v>19</v>
       </c>
       <c r="K30" s="3" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="L30" s="6" t="s">
         <v>21</v>
@@ -2462,7 +2532,7 @@
     </row>
     <row r="31" spans="1:12" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="2" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="B31" s="3">
         <v>3</v>
@@ -2470,29 +2540,29 @@
       <c r="C31" s="3">
         <v>30.1</v>
       </c>
-      <c r="D31" s="8" t="s">
-        <v>23</v>
+      <c r="D31" s="14" t="s">
+        <v>44</v>
       </c>
       <c r="E31" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="F31" s="9" t="s">
-        <v>25</v>
+        <v>128</v>
+      </c>
+      <c r="F31" s="19" t="s">
+        <v>83</v>
       </c>
       <c r="G31" s="3" t="s">
-        <v>125</v>
-      </c>
-      <c r="H31" s="5" t="s">
-        <v>105</v>
-      </c>
-      <c r="I31" s="14" t="s">
+        <v>129</v>
+      </c>
+      <c r="H31" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="I31" s="5" t="s">
         <v>38</v>
       </c>
       <c r="J31" s="6" t="s">
         <v>19</v>
       </c>
       <c r="K31" s="3" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="L31" s="6" t="s">
         <v>21</v>
@@ -2500,7 +2570,7 @@
     </row>
     <row r="32" spans="1:12" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="2" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="B32" s="3">
         <v>3</v>
@@ -2512,25 +2582,25 @@
         <v>13</v>
       </c>
       <c r="E32" s="3" t="s">
-        <v>128</v>
-      </c>
-      <c r="F32" s="11" t="s">
-        <v>30</v>
+        <v>29</v>
+      </c>
+      <c r="F32" s="5" t="s">
+        <v>15</v>
       </c>
       <c r="G32" s="3" t="s">
-        <v>129</v>
-      </c>
-      <c r="H32" s="17" t="s">
-        <v>65</v>
-      </c>
-      <c r="I32" s="14" t="s">
-        <v>38</v>
+        <v>132</v>
+      </c>
+      <c r="H32" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="I32" s="7" t="s">
+        <v>18</v>
       </c>
       <c r="J32" s="6" t="s">
         <v>19</v>
       </c>
       <c r="K32" s="3" t="s">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="L32" s="6" t="s">
         <v>21</v>
@@ -2538,37 +2608,37 @@
     </row>
     <row r="33" spans="1:12" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="2" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="B33" s="3">
         <v>3</v>
       </c>
       <c r="C33" s="3">
-        <v>30.1</v>
-      </c>
-      <c r="D33" s="15" t="s">
-        <v>47</v>
+        <v>30.2</v>
+      </c>
+      <c r="D33" s="14" t="s">
+        <v>44</v>
       </c>
       <c r="E33" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="F33" s="14" t="s">
-        <v>48</v>
+        <v>45</v>
+      </c>
+      <c r="F33" s="19" t="s">
+        <v>83</v>
       </c>
       <c r="G33" s="3" t="s">
-        <v>132</v>
-      </c>
-      <c r="H33" s="5" t="s">
-        <v>105</v>
-      </c>
-      <c r="I33" s="14" t="s">
-        <v>38</v>
+        <v>135</v>
+      </c>
+      <c r="H33" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="I33" s="7" t="s">
+        <v>18</v>
       </c>
       <c r="J33" s="6" t="s">
         <v>19</v>
       </c>
       <c r="K33" s="3" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="L33" s="6" t="s">
         <v>21</v>
@@ -2576,37 +2646,37 @@
     </row>
     <row r="34" spans="1:12" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" s="2" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="B34" s="3">
         <v>3</v>
       </c>
       <c r="C34" s="3">
-        <v>30</v>
-      </c>
-      <c r="D34" s="8" t="s">
-        <v>23</v>
+        <v>30.2</v>
+      </c>
+      <c r="D34" s="13" t="s">
+        <v>35</v>
       </c>
       <c r="E34" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="F34" s="13" t="s">
-        <v>36</v>
+        <v>138</v>
+      </c>
+      <c r="F34" s="5" t="s">
+        <v>15</v>
       </c>
       <c r="G34" s="3" t="s">
-        <v>135</v>
-      </c>
-      <c r="H34" s="17" t="s">
-        <v>65</v>
-      </c>
-      <c r="I34" s="14" t="s">
-        <v>38</v>
+        <v>139</v>
+      </c>
+      <c r="H34" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="I34" s="7" t="s">
+        <v>18</v>
       </c>
       <c r="J34" s="6" t="s">
         <v>19</v>
       </c>
       <c r="K34" s="3" t="s">
-        <v>66</v>
+        <v>140</v>
       </c>
       <c r="L34" s="6" t="s">
         <v>21</v>
@@ -2614,104 +2684,104 @@
     </row>
     <row r="35" spans="1:12" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="2" t="s">
-        <v>136</v>
+        <v>141</v>
       </c>
       <c r="B35" s="3">
         <v>3</v>
       </c>
       <c r="C35" s="3">
-        <v>30.1</v>
-      </c>
-      <c r="D35" s="8" t="s">
-        <v>23</v>
+        <v>30.2</v>
+      </c>
+      <c r="D35" s="4" t="s">
+        <v>13</v>
       </c>
       <c r="E35" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="F35" s="13" t="s">
-        <v>36</v>
+        <v>14</v>
+      </c>
+      <c r="F35" s="5" t="s">
+        <v>15</v>
       </c>
       <c r="G35" s="3" t="s">
-        <v>137</v>
-      </c>
-      <c r="H35" s="12" t="s">
-        <v>32</v>
-      </c>
-      <c r="I35" s="14" t="s">
-        <v>38</v>
-      </c>
-      <c r="J35" s="6" t="s">
-        <v>19</v>
+        <v>142</v>
+      </c>
+      <c r="H35" s="8" t="s">
+        <v>143</v>
+      </c>
+      <c r="I35" s="21" t="s">
+        <v>144</v>
+      </c>
+      <c r="J35" s="4" t="s">
+        <v>145</v>
       </c>
       <c r="K35" s="3" t="s">
-        <v>138</v>
-      </c>
-      <c r="L35" s="6" t="s">
-        <v>21</v>
+        <v>70</v>
+      </c>
+      <c r="L35" s="4" t="s">
+        <v>145</v>
       </c>
     </row>
     <row r="36" spans="1:12" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="2" t="s">
-        <v>139</v>
+        <v>146</v>
       </c>
       <c r="B36" s="3">
         <v>3</v>
       </c>
       <c r="C36" s="3">
-        <v>30.1</v>
-      </c>
-      <c r="D36" s="4" t="s">
-        <v>13</v>
+        <v>30.2</v>
+      </c>
+      <c r="D36" s="8" t="s">
+        <v>23</v>
       </c>
       <c r="E36" s="3" t="s">
-        <v>63</v>
-      </c>
-      <c r="F36" s="14" t="s">
-        <v>48</v>
+        <v>14</v>
+      </c>
+      <c r="F36" s="5" t="s">
+        <v>15</v>
       </c>
       <c r="G36" s="3" t="s">
-        <v>140</v>
-      </c>
-      <c r="H36" s="12" t="s">
-        <v>32</v>
-      </c>
-      <c r="I36" s="7" t="s">
-        <v>18</v>
-      </c>
-      <c r="J36" s="6" t="s">
-        <v>19</v>
+        <v>147</v>
+      </c>
+      <c r="H36" s="4" t="s">
+        <v>148</v>
+      </c>
+      <c r="I36" s="21" t="s">
+        <v>144</v>
+      </c>
+      <c r="J36" s="4" t="s">
+        <v>145</v>
       </c>
       <c r="K36" s="3" t="s">
-        <v>141</v>
-      </c>
-      <c r="L36" s="6" t="s">
-        <v>21</v>
+        <v>70</v>
+      </c>
+      <c r="L36" s="4" t="s">
+        <v>145</v>
       </c>
     </row>
     <row r="37" spans="1:12" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A37" s="2" t="s">
-        <v>142</v>
+        <v>149</v>
       </c>
       <c r="B37" s="3">
         <v>3</v>
       </c>
       <c r="C37" s="3">
-        <v>30.2</v>
-      </c>
-      <c r="D37" s="8" t="s">
-        <v>23</v>
+        <v>30.1</v>
+      </c>
+      <c r="D37" s="14" t="s">
+        <v>44</v>
       </c>
       <c r="E37" s="3" t="s">
-        <v>143</v>
-      </c>
-      <c r="F37" s="9" t="s">
-        <v>25</v>
+        <v>150</v>
+      </c>
+      <c r="F37" s="15" t="s">
+        <v>46</v>
       </c>
       <c r="G37" s="3" t="s">
-        <v>144</v>
+        <v>151</v>
       </c>
       <c r="H37" s="16" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="I37" s="7" t="s">
         <v>18</v>
@@ -2720,7 +2790,7 @@
         <v>19</v>
       </c>
       <c r="K37" s="3" t="s">
-        <v>145</v>
+        <v>152</v>
       </c>
       <c r="L37" s="6" t="s">
         <v>21</v>
@@ -2728,45 +2798,45 @@
     </row>
     <row r="38" spans="1:12" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A38" s="2" t="s">
-        <v>146</v>
-      </c>
-      <c r="B38" s="3">
-        <v>3</v>
-      </c>
-      <c r="C38" s="3">
-        <v>30.2</v>
+        <v>153</v>
+      </c>
+      <c r="B38" t="s">
+        <v>70</v>
+      </c>
+      <c r="C38" t="s">
+        <v>70</v>
       </c>
       <c r="D38" s="4" t="s">
         <v>13</v>
       </c>
       <c r="E38" s="3" t="s">
-        <v>147</v>
-      </c>
-      <c r="F38" s="14" t="s">
-        <v>48</v>
+        <v>14</v>
+      </c>
+      <c r="F38" s="10" t="s">
+        <v>36</v>
       </c>
       <c r="G38" s="3" t="s">
-        <v>148</v>
-      </c>
-      <c r="H38" s="16" t="s">
-        <v>50</v>
-      </c>
-      <c r="I38" s="7" t="s">
-        <v>18</v>
-      </c>
-      <c r="J38" s="6" t="s">
-        <v>19</v>
+        <v>154</v>
+      </c>
+      <c r="H38" s="14" t="s">
+        <v>94</v>
+      </c>
+      <c r="I38" s="22" t="s">
+        <v>155</v>
+      </c>
+      <c r="J38" s="21" t="s">
+        <v>156</v>
       </c>
       <c r="K38" s="3" t="s">
-        <v>149</v>
-      </c>
-      <c r="L38" s="6" t="s">
-        <v>21</v>
+        <v>157</v>
+      </c>
+      <c r="L38" s="4" t="s">
+        <v>145</v>
       </c>
     </row>
     <row r="39" spans="1:12" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A39" s="2" t="s">
-        <v>150</v>
+        <v>158</v>
       </c>
       <c r="B39" s="3">
         <v>3</v>
@@ -2778,203 +2848,203 @@
         <v>13</v>
       </c>
       <c r="E39" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="F39" s="10" t="s">
-        <v>60</v>
+        <v>159</v>
+      </c>
+      <c r="F39" s="5" t="s">
+        <v>15</v>
       </c>
       <c r="G39" s="3" t="s">
-        <v>151</v>
-      </c>
-      <c r="H39" s="15" t="s">
-        <v>152</v>
-      </c>
-      <c r="I39" s="19" t="s">
-        <v>153</v>
-      </c>
-      <c r="J39" s="4" t="s">
-        <v>154</v>
+        <v>160</v>
+      </c>
+      <c r="H39" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="I39" s="22" t="s">
+        <v>155</v>
+      </c>
+      <c r="J39" s="6" t="s">
+        <v>19</v>
       </c>
       <c r="K39" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="L39" s="4" t="s">
-        <v>154</v>
+        <v>161</v>
+      </c>
+      <c r="L39" s="6" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="40" spans="1:12" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A40" s="2" t="s">
-        <v>155</v>
-      </c>
-      <c r="B40" s="3">
-        <v>3</v>
-      </c>
-      <c r="C40" s="3">
-        <v>30.2</v>
-      </c>
-      <c r="D40" s="15" t="s">
-        <v>47</v>
-      </c>
-      <c r="E40" s="3" t="s">
+        <v>162</v>
+      </c>
+      <c r="B40" t="s">
+        <v>70</v>
+      </c>
+      <c r="C40" t="s">
+        <v>70</v>
+      </c>
+      <c r="D40" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="E40" t="s">
+        <v>70</v>
+      </c>
+      <c r="F40" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="F40" s="14" t="s">
-        <v>48</v>
-      </c>
       <c r="G40" s="3" t="s">
-        <v>156</v>
-      </c>
-      <c r="H40" s="4" t="s">
-        <v>157</v>
-      </c>
-      <c r="I40" s="19" t="s">
-        <v>153</v>
-      </c>
-      <c r="J40" s="4" t="s">
-        <v>154</v>
+        <v>163</v>
+      </c>
+      <c r="H40" s="14" t="s">
+        <v>94</v>
+      </c>
+      <c r="I40" s="23" t="s">
+        <v>164</v>
+      </c>
+      <c r="J40" s="6" t="s">
+        <v>19</v>
       </c>
       <c r="K40" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="L40" s="4" t="s">
-        <v>154</v>
+        <v>165</v>
+      </c>
+      <c r="L40" s="6" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="41" spans="1:12" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A41" s="2" t="s">
-        <v>158</v>
-      </c>
-      <c r="B41" s="3">
-        <v>3</v>
-      </c>
-      <c r="C41" s="3">
-        <v>30.1</v>
-      </c>
-      <c r="D41" s="8" t="s">
-        <v>23</v>
+        <v>166</v>
+      </c>
+      <c r="B41" t="s">
+        <v>70</v>
+      </c>
+      <c r="C41" t="s">
+        <v>70</v>
+      </c>
+      <c r="D41" s="4" t="s">
+        <v>13</v>
       </c>
       <c r="E41" s="3" t="s">
-        <v>143</v>
-      </c>
-      <c r="F41" s="9" t="s">
-        <v>25</v>
+        <v>14</v>
+      </c>
+      <c r="F41" s="16" t="s">
+        <v>167</v>
       </c>
       <c r="G41" s="3" t="s">
-        <v>159</v>
-      </c>
-      <c r="H41" s="16" t="s">
-        <v>50</v>
-      </c>
-      <c r="I41" s="7" t="s">
-        <v>18</v>
-      </c>
-      <c r="J41" s="6" t="s">
-        <v>19</v>
+        <v>168</v>
+      </c>
+      <c r="H41" s="14" t="s">
+        <v>94</v>
+      </c>
+      <c r="I41" s="21" t="s">
+        <v>144</v>
+      </c>
+      <c r="J41" s="21" t="s">
+        <v>156</v>
       </c>
       <c r="K41" s="3" t="s">
-        <v>160</v>
-      </c>
-      <c r="L41" s="6" t="s">
-        <v>21</v>
+        <v>70</v>
+      </c>
+      <c r="L41" s="4" t="s">
+        <v>145</v>
       </c>
     </row>
     <row r="42" spans="1:12" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A42" s="2" t="s">
-        <v>161</v>
+        <v>169</v>
       </c>
       <c r="B42" t="s">
-        <v>13</v>
+        <v>70</v>
       </c>
       <c r="C42" t="s">
-        <v>13</v>
+        <v>70</v>
       </c>
       <c r="D42" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="E42" t="s">
-        <v>13</v>
-      </c>
-      <c r="F42" s="16" t="s">
-        <v>162</v>
+      <c r="E42" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="F42" s="10" t="s">
+        <v>36</v>
       </c>
       <c r="G42" s="3" t="s">
-        <v>163</v>
+        <v>170</v>
       </c>
       <c r="H42" s="4" t="s">
-        <v>157</v>
-      </c>
-      <c r="I42" s="4" t="s">
-        <v>154</v>
+        <v>148</v>
+      </c>
+      <c r="I42" s="21" t="s">
+        <v>144</v>
       </c>
       <c r="J42" s="4" t="s">
-        <v>154</v>
+        <v>145</v>
       </c>
       <c r="K42" s="3" t="s">
-        <v>13</v>
+        <v>70</v>
       </c>
       <c r="L42" s="4" t="s">
-        <v>154</v>
+        <v>145</v>
       </c>
     </row>
     <row r="43" spans="1:12" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A43" s="2" t="s">
-        <v>164</v>
-      </c>
-      <c r="B43" s="3">
-        <v>3</v>
-      </c>
-      <c r="C43" s="3">
-        <v>30.2</v>
+        <v>171</v>
+      </c>
+      <c r="B43" t="s">
+        <v>70</v>
+      </c>
+      <c r="C43" t="s">
+        <v>70</v>
       </c>
       <c r="D43" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="E43" s="3" t="s">
-        <v>143</v>
+      <c r="E43" t="s">
+        <v>70</v>
       </c>
       <c r="F43" s="16" t="s">
-        <v>162</v>
+        <v>167</v>
       </c>
       <c r="G43" s="3" t="s">
-        <v>165</v>
-      </c>
-      <c r="H43" s="16" t="s">
-        <v>50</v>
-      </c>
-      <c r="I43" s="20" t="s">
-        <v>166</v>
-      </c>
-      <c r="J43" s="6" t="s">
-        <v>19</v>
+        <v>172</v>
+      </c>
+      <c r="H43" s="4" t="s">
+        <v>148</v>
+      </c>
+      <c r="I43" s="21" t="s">
+        <v>144</v>
+      </c>
+      <c r="J43" s="4" t="s">
+        <v>145</v>
       </c>
       <c r="K43" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="L43" s="6" t="s">
-        <v>21</v>
+        <v>70</v>
+      </c>
+      <c r="L43" s="4" t="s">
+        <v>145</v>
       </c>
     </row>
     <row r="44" spans="1:12" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A44" s="2" t="s">
-        <v>167</v>
+        <v>173</v>
       </c>
       <c r="B44" t="s">
-        <v>13</v>
+        <v>70</v>
       </c>
       <c r="C44" t="s">
-        <v>13</v>
+        <v>70</v>
       </c>
       <c r="D44" s="4" t="s">
         <v>13</v>
       </c>
       <c r="E44" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="F44" s="14" t="s">
-        <v>48</v>
+        <v>14</v>
+      </c>
+      <c r="F44" s="5" t="s">
+        <v>15</v>
       </c>
       <c r="G44" s="3" t="s">
-        <v>168</v>
+        <v>174</v>
       </c>
       <c r="H44" s="6" t="s">
         <v>17</v>
@@ -2986,7 +3056,7 @@
         <v>19</v>
       </c>
       <c r="K44" s="3" t="s">
-        <v>169</v>
+        <v>175</v>
       </c>
       <c r="L44" s="6" t="s">
         <v>21</v>
@@ -2994,25 +3064,25 @@
     </row>
     <row r="45" spans="1:12" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A45" s="2" t="s">
-        <v>170</v>
+        <v>176</v>
       </c>
       <c r="B45" t="s">
-        <v>13</v>
+        <v>70</v>
       </c>
       <c r="C45" t="s">
-        <v>13</v>
+        <v>70</v>
       </c>
       <c r="D45" s="4" t="s">
         <v>13</v>
       </c>
       <c r="E45" s="3" t="s">
-        <v>35</v>
+        <v>45</v>
       </c>
       <c r="F45" s="4" t="s">
-        <v>171</v>
+        <v>177</v>
       </c>
       <c r="G45" s="3" t="s">
-        <v>172</v>
+        <v>178</v>
       </c>
       <c r="H45" s="12" t="s">
         <v>32</v>
@@ -3024,7 +3094,7 @@
         <v>19</v>
       </c>
       <c r="K45" s="3" t="s">
-        <v>173</v>
+        <v>179</v>
       </c>
       <c r="L45" s="6" t="s">
         <v>21</v>
@@ -3032,37 +3102,37 @@
     </row>
     <row r="46" spans="1:12" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A46" s="2" t="s">
-        <v>174</v>
+        <v>180</v>
       </c>
       <c r="B46" t="s">
-        <v>13</v>
+        <v>70</v>
       </c>
       <c r="C46" t="s">
-        <v>13</v>
+        <v>70</v>
       </c>
       <c r="D46" s="4" t="s">
         <v>13</v>
       </c>
       <c r="E46" s="3" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="F46" s="4" t="s">
-        <v>171</v>
+        <v>177</v>
       </c>
       <c r="G46" s="3" t="s">
-        <v>175</v>
-      </c>
-      <c r="H46" s="5" t="s">
-        <v>105</v>
-      </c>
-      <c r="I46" s="14" t="s">
+        <v>181</v>
+      </c>
+      <c r="H46" s="15" t="s">
+        <v>101</v>
+      </c>
+      <c r="I46" s="5" t="s">
         <v>38</v>
       </c>
       <c r="J46" s="6" t="s">
         <v>19</v>
       </c>
       <c r="K46" s="3" t="s">
-        <v>176</v>
+        <v>182</v>
       </c>
       <c r="L46" s="6" t="s">
         <v>21</v>
@@ -3070,75 +3140,75 @@
     </row>
     <row r="47" spans="1:12" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A47" s="2" t="s">
-        <v>177</v>
+        <v>183</v>
       </c>
       <c r="B47" t="s">
-        <v>13</v>
+        <v>70</v>
       </c>
       <c r="C47" t="s">
-        <v>13</v>
+        <v>70</v>
       </c>
       <c r="D47" s="4" t="s">
         <v>13</v>
       </c>
       <c r="E47" s="3" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="F47" s="4" t="s">
-        <v>171</v>
+        <v>177</v>
       </c>
       <c r="G47" s="3" t="s">
-        <v>178</v>
+        <v>184</v>
       </c>
       <c r="H47" s="12" t="s">
         <v>32</v>
       </c>
-      <c r="I47" s="14" t="s">
+      <c r="I47" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="J47" s="8" t="s">
-        <v>179</v>
+      <c r="J47" s="14" t="s">
+        <v>185</v>
       </c>
       <c r="K47" s="3" t="s">
-        <v>180</v>
+        <v>186</v>
       </c>
       <c r="L47" s="4" t="s">
-        <v>154</v>
+        <v>145</v>
       </c>
     </row>
     <row r="48" spans="1:12" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A48" s="2" t="s">
-        <v>181</v>
+        <v>187</v>
       </c>
       <c r="B48" t="s">
-        <v>13</v>
+        <v>70</v>
       </c>
       <c r="C48" t="s">
-        <v>13</v>
+        <v>70</v>
       </c>
       <c r="D48" s="4" t="s">
         <v>13</v>
       </c>
       <c r="E48" s="3" t="s">
-        <v>143</v>
+        <v>159</v>
       </c>
       <c r="F48" s="4" t="s">
-        <v>171</v>
+        <v>177</v>
       </c>
       <c r="G48" s="3" t="s">
-        <v>182</v>
+        <v>188</v>
       </c>
       <c r="H48" s="16" t="s">
-        <v>50</v>
-      </c>
-      <c r="I48" s="14" t="s">
+        <v>51</v>
+      </c>
+      <c r="I48" s="5" t="s">
         <v>38</v>
       </c>
       <c r="J48" s="6" t="s">
         <v>19</v>
       </c>
       <c r="K48" s="3" t="s">
-        <v>183</v>
+        <v>189</v>
       </c>
       <c r="L48" s="6" t="s">
         <v>21</v>
@@ -3146,25 +3216,25 @@
     </row>
     <row r="49" spans="1:12" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A49" s="2" t="s">
-        <v>184</v>
+        <v>190</v>
       </c>
       <c r="B49" t="s">
-        <v>13</v>
+        <v>70</v>
       </c>
       <c r="C49" t="s">
-        <v>13</v>
+        <v>70</v>
       </c>
       <c r="D49" s="4" t="s">
         <v>13</v>
       </c>
       <c r="E49" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="F49" s="5" t="s">
-        <v>15</v>
+        <v>14</v>
+      </c>
+      <c r="F49" s="15" t="s">
+        <v>46</v>
       </c>
       <c r="G49" s="3" t="s">
-        <v>185</v>
+        <v>191</v>
       </c>
       <c r="H49" s="6" t="s">
         <v>17</v>
@@ -3176,7 +3246,7 @@
         <v>19</v>
       </c>
       <c r="K49" s="3" t="s">
-        <v>186</v>
+        <v>192</v>
       </c>
       <c r="L49" s="6" t="s">
         <v>21</v>
@@ -3184,37 +3254,37 @@
     </row>
     <row r="50" spans="1:12" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A50" s="2" t="s">
-        <v>187</v>
+        <v>193</v>
       </c>
       <c r="B50" t="s">
-        <v>13</v>
+        <v>70</v>
       </c>
       <c r="C50" t="s">
-        <v>13</v>
+        <v>70</v>
       </c>
       <c r="D50" s="4" t="s">
         <v>13</v>
       </c>
       <c r="E50" s="3" t="s">
-        <v>188</v>
+        <v>194</v>
       </c>
       <c r="F50" s="12" t="s">
         <v>71</v>
       </c>
       <c r="G50" s="3" t="s">
-        <v>189</v>
-      </c>
-      <c r="H50" s="14" t="s">
-        <v>86</v>
-      </c>
-      <c r="I50" s="14" t="s">
+        <v>195</v>
+      </c>
+      <c r="H50" s="5" t="s">
+        <v>80</v>
+      </c>
+      <c r="I50" s="5" t="s">
         <v>38</v>
       </c>
       <c r="J50" s="6" t="s">
         <v>19</v>
       </c>
       <c r="K50" s="3" t="s">
-        <v>190</v>
+        <v>196</v>
       </c>
       <c r="L50" s="6" t="s">
         <v>21</v>
@@ -3222,37 +3292,37 @@
     </row>
     <row r="51" spans="1:12" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A51" s="2" t="s">
-        <v>191</v>
+        <v>197</v>
       </c>
       <c r="B51" t="s">
-        <v>13</v>
+        <v>70</v>
       </c>
       <c r="C51" t="s">
-        <v>13</v>
+        <v>70</v>
       </c>
       <c r="D51" s="4" t="s">
         <v>13</v>
       </c>
       <c r="E51" s="3" t="s">
-        <v>188</v>
+        <v>194</v>
       </c>
       <c r="F51" s="12" t="s">
         <v>71</v>
       </c>
       <c r="G51" s="3" t="s">
-        <v>192</v>
-      </c>
-      <c r="H51" s="14" t="s">
-        <v>86</v>
-      </c>
-      <c r="I51" s="14" t="s">
+        <v>198</v>
+      </c>
+      <c r="H51" s="5" t="s">
+        <v>80</v>
+      </c>
+      <c r="I51" s="5" t="s">
         <v>38</v>
       </c>
       <c r="J51" s="6" t="s">
         <v>19</v>
       </c>
       <c r="K51" s="3" t="s">
-        <v>190</v>
+        <v>196</v>
       </c>
       <c r="L51" s="6" t="s">
         <v>21</v>
@@ -3260,37 +3330,37 @@
     </row>
     <row r="52" spans="1:12" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A52" s="2" t="s">
-        <v>193</v>
+        <v>199</v>
       </c>
       <c r="B52" t="s">
-        <v>13</v>
+        <v>70</v>
       </c>
       <c r="C52" t="s">
-        <v>13</v>
+        <v>70</v>
       </c>
       <c r="D52" s="4" t="s">
         <v>13</v>
       </c>
       <c r="E52" s="3" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="F52" s="10" t="s">
-        <v>60</v>
+        <v>36</v>
       </c>
       <c r="G52" s="3" t="s">
-        <v>194</v>
+        <v>200</v>
       </c>
       <c r="H52" s="12" t="s">
         <v>32</v>
       </c>
-      <c r="I52" s="14" t="s">
+      <c r="I52" s="5" t="s">
         <v>38</v>
       </c>
       <c r="J52" s="6" t="s">
         <v>19</v>
       </c>
       <c r="K52" s="3" t="s">
-        <v>180</v>
+        <v>186</v>
       </c>
       <c r="L52" s="6" t="s">
         <v>21</v>
@@ -3298,31 +3368,31 @@
     </row>
     <row r="53" spans="1:12" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A53" s="2" t="s">
-        <v>195</v>
+        <v>201</v>
       </c>
       <c r="B53" t="s">
-        <v>13</v>
+        <v>70</v>
       </c>
       <c r="C53" t="s">
-        <v>13</v>
+        <v>70</v>
       </c>
       <c r="D53" s="4" t="s">
         <v>13</v>
       </c>
       <c r="E53" s="3" t="s">
-        <v>196</v>
+        <v>202</v>
       </c>
       <c r="F53" s="4" t="s">
-        <v>171</v>
+        <v>177</v>
       </c>
       <c r="G53" s="3" t="s">
-        <v>197</v>
-      </c>
-      <c r="H53" s="14" t="s">
-        <v>86</v>
-      </c>
-      <c r="I53" s="19" t="s">
-        <v>153</v>
+        <v>203</v>
+      </c>
+      <c r="H53" s="5" t="s">
+        <v>80</v>
+      </c>
+      <c r="I53" s="21" t="s">
+        <v>144</v>
       </c>
       <c r="J53" s="6" t="s">
         <v>19</v>
@@ -3331,33 +3401,33 @@
         <v>73</v>
       </c>
       <c r="L53" s="4" t="s">
-        <v>154</v>
+        <v>145</v>
       </c>
     </row>
     <row r="54" spans="1:12" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A54" s="2" t="s">
-        <v>198</v>
+        <v>204</v>
       </c>
       <c r="B54" t="s">
-        <v>13</v>
+        <v>70</v>
       </c>
       <c r="C54" t="s">
-        <v>13</v>
+        <v>70</v>
       </c>
       <c r="D54" s="4" t="s">
         <v>13</v>
       </c>
       <c r="E54" s="3" t="s">
-        <v>199</v>
+        <v>205</v>
       </c>
       <c r="F54" s="4" t="s">
-        <v>171</v>
+        <v>177</v>
       </c>
       <c r="G54" s="3" t="s">
-        <v>200</v>
+        <v>206</v>
       </c>
       <c r="H54" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="I54" s="7" t="s">
         <v>18</v>
@@ -3366,7 +3436,7 @@
         <v>19</v>
       </c>
       <c r="K54" s="3" t="s">
-        <v>201</v>
+        <v>207</v>
       </c>
       <c r="L54" s="6" t="s">
         <v>21</v>
@@ -3374,37 +3444,37 @@
     </row>
     <row r="55" spans="1:12" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A55" s="2" t="s">
-        <v>202</v>
+        <v>208</v>
       </c>
       <c r="B55" t="s">
-        <v>13</v>
+        <v>70</v>
       </c>
       <c r="C55" t="s">
-        <v>13</v>
+        <v>70</v>
       </c>
       <c r="D55" s="4" t="s">
         <v>13</v>
       </c>
       <c r="E55" s="3" t="s">
-        <v>143</v>
+        <v>159</v>
       </c>
       <c r="F55" s="4" t="s">
-        <v>171</v>
+        <v>177</v>
       </c>
       <c r="G55" s="3" t="s">
-        <v>203</v>
+        <v>209</v>
       </c>
       <c r="H55" s="16" t="s">
-        <v>50</v>
-      </c>
-      <c r="I55" s="14" t="s">
+        <v>51</v>
+      </c>
+      <c r="I55" s="5" t="s">
         <v>38</v>
       </c>
       <c r="J55" s="6" t="s">
         <v>19</v>
       </c>
       <c r="K55" s="3" t="s">
-        <v>204</v>
+        <v>210</v>
       </c>
       <c r="L55" s="6" t="s">
         <v>21</v>
@@ -3412,28 +3482,28 @@
     </row>
     <row r="56" spans="1:12" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A56" s="2" t="s">
-        <v>205</v>
+        <v>211</v>
       </c>
       <c r="B56" t="s">
-        <v>13</v>
+        <v>70</v>
       </c>
       <c r="C56" t="s">
-        <v>13</v>
+        <v>70</v>
       </c>
       <c r="D56" s="4" t="s">
         <v>13</v>
       </c>
       <c r="E56" t="s">
-        <v>13</v>
+        <v>70</v>
       </c>
       <c r="F56" s="16" t="s">
-        <v>162</v>
+        <v>167</v>
       </c>
       <c r="G56" s="3" t="s">
-        <v>206</v>
+        <v>212</v>
       </c>
       <c r="H56" s="16" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="I56" s="7" t="s">
         <v>18</v>
@@ -3442,7 +3512,7 @@
         <v>19</v>
       </c>
       <c r="K56" s="3" t="s">
-        <v>207</v>
+        <v>213</v>
       </c>
       <c r="L56" s="6" t="s">
         <v>21</v>
@@ -3450,37 +3520,37 @@
     </row>
     <row r="57" spans="1:12" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A57" s="2" t="s">
-        <v>208</v>
+        <v>214</v>
       </c>
       <c r="B57" s="3">
         <v>3.1</v>
       </c>
       <c r="C57" t="s">
-        <v>13</v>
+        <v>70</v>
       </c>
       <c r="D57" s="4" t="s">
         <v>13</v>
       </c>
       <c r="E57" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="F57" s="14" t="s">
-        <v>48</v>
+        <v>14</v>
+      </c>
+      <c r="F57" s="12" t="s">
+        <v>71</v>
       </c>
       <c r="G57" s="3" t="s">
-        <v>209</v>
-      </c>
-      <c r="H57" s="21" t="s">
-        <v>210</v>
-      </c>
-      <c r="I57" s="14" t="s">
+        <v>215</v>
+      </c>
+      <c r="H57" s="23" t="s">
+        <v>216</v>
+      </c>
+      <c r="I57" s="5" t="s">
         <v>38</v>
       </c>
       <c r="J57" s="6" t="s">
         <v>19</v>
       </c>
       <c r="K57" s="3" t="s">
-        <v>211</v>
+        <v>217</v>
       </c>
       <c r="L57" s="6" t="s">
         <v>21</v>
@@ -3488,7 +3558,7 @@
     </row>
     <row r="58" spans="1:12" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A58" s="2" t="s">
-        <v>212</v>
+        <v>218</v>
       </c>
       <c r="B58" s="3">
         <v>3</v>
@@ -3497,28 +3567,28 @@
         <v>30</v>
       </c>
       <c r="D58" s="12" t="s">
-        <v>213</v>
+        <v>219</v>
       </c>
       <c r="E58" s="3" t="s">
-        <v>214</v>
+        <v>220</v>
       </c>
       <c r="F58" s="6" t="s">
         <v>19</v>
       </c>
       <c r="G58" s="3" t="s">
-        <v>215</v>
-      </c>
-      <c r="H58" s="15" t="s">
-        <v>152</v>
+        <v>221</v>
+      </c>
+      <c r="H58" s="8" t="s">
+        <v>143</v>
       </c>
       <c r="I58" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="J58" s="22" t="s">
-        <v>216</v>
+      <c r="J58" s="24" t="s">
+        <v>222</v>
       </c>
       <c r="K58" s="3" t="s">
-        <v>217</v>
+        <v>223</v>
       </c>
       <c r="L58" s="6" t="s">
         <v>21</v>
@@ -3526,7 +3596,7 @@
     </row>
     <row r="59" spans="1:12" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A59" s="2" t="s">
-        <v>218</v>
+        <v>224</v>
       </c>
       <c r="B59" s="3">
         <v>3</v>
@@ -3535,28 +3605,28 @@
         <v>30</v>
       </c>
       <c r="D59" s="12" t="s">
-        <v>213</v>
+        <v>219</v>
       </c>
       <c r="E59" s="3" t="s">
-        <v>219</v>
+        <v>225</v>
       </c>
       <c r="F59" s="6" t="s">
         <v>19</v>
       </c>
       <c r="G59" s="3" t="s">
-        <v>220</v>
-      </c>
-      <c r="H59" s="21" t="s">
-        <v>210</v>
+        <v>226</v>
+      </c>
+      <c r="H59" s="23" t="s">
+        <v>216</v>
       </c>
       <c r="I59" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="J59" s="22" t="s">
-        <v>216</v>
+      <c r="J59" s="24" t="s">
+        <v>222</v>
       </c>
       <c r="K59" s="3" t="s">
-        <v>218</v>
+        <v>224</v>
       </c>
       <c r="L59" s="6" t="s">
         <v>21</v>
@@ -3564,7 +3634,7 @@
     </row>
     <row r="60" spans="1:12" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A60" s="2" t="s">
-        <v>221</v>
+        <v>227</v>
       </c>
       <c r="B60" s="3">
         <v>3</v>
@@ -3573,28 +3643,28 @@
         <v>30.1</v>
       </c>
       <c r="D60" s="12" t="s">
-        <v>213</v>
+        <v>219</v>
       </c>
       <c r="E60" s="3" t="s">
-        <v>219</v>
+        <v>225</v>
       </c>
       <c r="F60" s="6" t="s">
         <v>19</v>
       </c>
       <c r="G60" s="3" t="s">
-        <v>222</v>
+        <v>228</v>
       </c>
       <c r="H60" s="16" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="I60" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="J60" s="22" t="s">
-        <v>216</v>
+      <c r="J60" s="24" t="s">
+        <v>222</v>
       </c>
       <c r="K60" s="3" t="s">
-        <v>223</v>
+        <v>229</v>
       </c>
       <c r="L60" s="6" t="s">
         <v>21</v>
@@ -3602,7 +3672,7 @@
     </row>
     <row r="61" spans="1:12" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A61" s="2" t="s">
-        <v>224</v>
+        <v>230</v>
       </c>
       <c r="B61" s="3">
         <v>3</v>
@@ -3611,28 +3681,28 @@
         <v>30</v>
       </c>
       <c r="D61" s="12" t="s">
-        <v>213</v>
+        <v>219</v>
       </c>
       <c r="E61" s="3" t="s">
-        <v>35</v>
+        <v>45</v>
       </c>
       <c r="F61" s="6" t="s">
         <v>19</v>
       </c>
       <c r="G61" s="3" t="s">
-        <v>225</v>
-      </c>
-      <c r="H61" s="5" t="s">
-        <v>105</v>
+        <v>231</v>
+      </c>
+      <c r="H61" s="15" t="s">
+        <v>101</v>
       </c>
       <c r="I61" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="J61" s="22" t="s">
-        <v>216</v>
+      <c r="J61" s="24" t="s">
+        <v>222</v>
       </c>
       <c r="K61" s="3" t="s">
-        <v>226</v>
+        <v>232</v>
       </c>
       <c r="L61" s="6" t="s">
         <v>21</v>
@@ -3640,7 +3710,7 @@
     </row>
     <row r="62" spans="1:12" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A62" s="2" t="s">
-        <v>227</v>
+        <v>233</v>
       </c>
       <c r="B62" s="3">
         <v>3</v>
@@ -3649,16 +3719,16 @@
         <v>30</v>
       </c>
       <c r="D62" s="12" t="s">
-        <v>213</v>
+        <v>219</v>
       </c>
       <c r="E62" s="3" t="s">
-        <v>35</v>
+        <v>45</v>
       </c>
       <c r="F62" s="6" t="s">
         <v>19</v>
       </c>
       <c r="G62" s="3" t="s">
-        <v>228</v>
+        <v>234</v>
       </c>
       <c r="H62" s="6" t="s">
         <v>17</v>
@@ -3666,11 +3736,11 @@
       <c r="I62" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="J62" s="22" t="s">
-        <v>216</v>
+      <c r="J62" s="24" t="s">
+        <v>222</v>
       </c>
       <c r="K62" s="3" t="s">
-        <v>229</v>
+        <v>235</v>
       </c>
       <c r="L62" s="6" t="s">
         <v>21</v>
@@ -3678,7 +3748,7 @@
     </row>
     <row r="63" spans="1:12" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A63" s="2" t="s">
-        <v>230</v>
+        <v>236</v>
       </c>
       <c r="B63" s="3">
         <v>3</v>
@@ -3687,16 +3757,16 @@
         <v>30</v>
       </c>
       <c r="D63" s="12" t="s">
-        <v>213</v>
+        <v>219</v>
       </c>
       <c r="E63" s="3" t="s">
-        <v>35</v>
+        <v>45</v>
       </c>
       <c r="F63" s="6" t="s">
         <v>19</v>
       </c>
       <c r="G63" s="3" t="s">
-        <v>231</v>
+        <v>237</v>
       </c>
       <c r="H63" s="6" t="s">
         <v>17</v>
@@ -3704,11 +3774,11 @@
       <c r="I63" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="J63" s="22" t="s">
-        <v>216</v>
+      <c r="J63" s="24" t="s">
+        <v>222</v>
       </c>
       <c r="K63" s="3" t="s">
-        <v>232</v>
+        <v>238</v>
       </c>
       <c r="L63" s="6" t="s">
         <v>21</v>
@@ -3716,7 +3786,7 @@
     </row>
     <row r="64" spans="1:12" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A64" s="2" t="s">
-        <v>233</v>
+        <v>239</v>
       </c>
       <c r="B64" s="3">
         <v>3</v>
@@ -3725,28 +3795,28 @@
         <v>30</v>
       </c>
       <c r="D64" s="12" t="s">
-        <v>213</v>
+        <v>219</v>
       </c>
       <c r="E64" s="3" t="s">
-        <v>35</v>
+        <v>45</v>
       </c>
       <c r="F64" s="6" t="s">
         <v>19</v>
       </c>
       <c r="G64" s="3" t="s">
-        <v>234</v>
-      </c>
-      <c r="H64" s="5" t="s">
-        <v>105</v>
+        <v>240</v>
+      </c>
+      <c r="H64" s="15" t="s">
+        <v>101</v>
       </c>
       <c r="I64" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="J64" s="22" t="s">
-        <v>216</v>
+      <c r="J64" s="24" t="s">
+        <v>222</v>
       </c>
       <c r="K64" s="3" t="s">
-        <v>235</v>
+        <v>241</v>
       </c>
       <c r="L64" s="6" t="s">
         <v>21</v>
@@ -3754,7 +3824,7 @@
     </row>
     <row r="65" spans="1:12" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A65" s="2" t="s">
-        <v>236</v>
+        <v>242</v>
       </c>
       <c r="B65" s="3">
         <v>3</v>
@@ -3763,28 +3833,28 @@
         <v>30</v>
       </c>
       <c r="D65" s="12" t="s">
-        <v>213</v>
+        <v>219</v>
       </c>
       <c r="E65" s="3" t="s">
-        <v>35</v>
+        <v>45</v>
       </c>
       <c r="F65" s="6" t="s">
         <v>19</v>
       </c>
       <c r="G65" s="3" t="s">
-        <v>237</v>
-      </c>
-      <c r="H65" s="8" t="s">
-        <v>76</v>
+        <v>243</v>
+      </c>
+      <c r="H65" s="14" t="s">
+        <v>94</v>
       </c>
       <c r="I65" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="J65" s="22" t="s">
-        <v>216</v>
+      <c r="J65" s="24" t="s">
+        <v>222</v>
       </c>
       <c r="K65" s="3" t="s">
-        <v>100</v>
+        <v>95</v>
       </c>
       <c r="L65" s="6" t="s">
         <v>21</v>
@@ -3792,7 +3862,7 @@
     </row>
     <row r="66" spans="1:12" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A66" s="2" t="s">
-        <v>238</v>
+        <v>244</v>
       </c>
       <c r="B66" s="3">
         <v>3</v>
@@ -3801,28 +3871,28 @@
         <v>30</v>
       </c>
       <c r="D66" s="12" t="s">
-        <v>213</v>
+        <v>219</v>
       </c>
       <c r="E66" s="3" t="s">
-        <v>35</v>
+        <v>45</v>
       </c>
       <c r="F66" s="6" t="s">
         <v>19</v>
       </c>
       <c r="G66" s="3" t="s">
-        <v>239</v>
+        <v>245</v>
       </c>
       <c r="H66" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="I66" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="J66" s="22" t="s">
-        <v>216</v>
+      <c r="J66" s="24" t="s">
+        <v>222</v>
       </c>
       <c r="K66" s="3" t="s">
-        <v>240</v>
+        <v>246</v>
       </c>
       <c r="L66" s="6" t="s">
         <v>21</v>
@@ -3830,7 +3900,7 @@
     </row>
     <row r="67" spans="1:12" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A67" s="2" t="s">
-        <v>241</v>
+        <v>247</v>
       </c>
       <c r="B67" s="3">
         <v>3</v>
@@ -3839,16 +3909,16 @@
         <v>30</v>
       </c>
       <c r="D67" s="12" t="s">
-        <v>213</v>
+        <v>219</v>
       </c>
       <c r="E67" s="3" t="s">
-        <v>35</v>
+        <v>45</v>
       </c>
       <c r="F67" s="6" t="s">
         <v>19</v>
       </c>
       <c r="G67" s="3" t="s">
-        <v>242</v>
+        <v>248</v>
       </c>
       <c r="H67" s="6" t="s">
         <v>17</v>
@@ -3856,11 +3926,11 @@
       <c r="I67" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="J67" s="22" t="s">
-        <v>216</v>
+      <c r="J67" s="24" t="s">
+        <v>222</v>
       </c>
       <c r="K67" s="3" t="s">
-        <v>241</v>
+        <v>247</v>
       </c>
       <c r="L67" s="6" t="s">
         <v>21</v>
@@ -3868,7 +3938,7 @@
     </row>
     <row r="68" spans="1:12" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A68" s="2" t="s">
-        <v>243</v>
+        <v>249</v>
       </c>
       <c r="B68" s="3">
         <v>3</v>
@@ -3877,34 +3947,186 @@
         <v>30</v>
       </c>
       <c r="D68" s="12" t="s">
-        <v>213</v>
+        <v>219</v>
       </c>
       <c r="E68" s="3" t="s">
-        <v>35</v>
+        <v>45</v>
       </c>
       <c r="F68" s="6" t="s">
         <v>19</v>
       </c>
       <c r="G68" s="3" t="s">
-        <v>244</v>
-      </c>
-      <c r="H68" s="8" t="s">
-        <v>76</v>
+        <v>250</v>
+      </c>
+      <c r="H68" s="14" t="s">
+        <v>94</v>
       </c>
       <c r="I68" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="J68" s="22" t="s">
-        <v>216</v>
+      <c r="J68" s="24" t="s">
+        <v>222</v>
       </c>
       <c r="K68" s="3" t="s">
-        <v>245</v>
+        <v>165</v>
       </c>
       <c r="L68" s="6" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="69" spans="1:12" ht="26.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="69" spans="1:12" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A69" s="2" t="s">
+        <v>251</v>
+      </c>
+      <c r="B69" s="3">
+        <v>3</v>
+      </c>
+      <c r="C69" s="3">
+        <v>30.1</v>
+      </c>
+      <c r="D69" s="14" t="s">
+        <v>44</v>
+      </c>
+      <c r="E69" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="F69" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="G69" s="3" t="s">
+        <v>252</v>
+      </c>
+      <c r="H69" s="14" t="s">
+        <v>94</v>
+      </c>
+      <c r="I69" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="J69" s="12" t="s">
+        <v>253</v>
+      </c>
+      <c r="K69" s="3" t="s">
+        <v>254</v>
+      </c>
+      <c r="L69" s="6" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="70" spans="1:12" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A70" s="2" t="s">
+        <v>255</v>
+      </c>
+      <c r="B70" s="3">
+        <v>3</v>
+      </c>
+      <c r="C70" s="3">
+        <v>30</v>
+      </c>
+      <c r="D70" s="14" t="s">
+        <v>44</v>
+      </c>
+      <c r="E70" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="F70" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="G70" s="3" t="s">
+        <v>256</v>
+      </c>
+      <c r="H70" s="5" t="s">
+        <v>80</v>
+      </c>
+      <c r="I70" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="J70" s="12" t="s">
+        <v>253</v>
+      </c>
+      <c r="K70" s="3" t="s">
+        <v>257</v>
+      </c>
+      <c r="L70" s="6" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="71" spans="1:12" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A71" s="2" t="s">
+        <v>258</v>
+      </c>
+      <c r="B71" s="3">
+        <v>3</v>
+      </c>
+      <c r="C71" s="3">
+        <v>30</v>
+      </c>
+      <c r="D71" s="14" t="s">
+        <v>44</v>
+      </c>
+      <c r="E71" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="F71" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="G71" s="3" t="s">
+        <v>259</v>
+      </c>
+      <c r="H71" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="I71" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="J71" s="12" t="s">
+        <v>253</v>
+      </c>
+      <c r="K71" s="3" t="s">
+        <v>260</v>
+      </c>
+      <c r="L71" s="6" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="72" spans="1:12" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A72" s="2" t="s">
+        <v>261</v>
+      </c>
+      <c r="B72" s="3">
+        <v>3</v>
+      </c>
+      <c r="C72" s="3">
+        <v>30</v>
+      </c>
+      <c r="D72" s="14" t="s">
+        <v>44</v>
+      </c>
+      <c r="E72" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="F72" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="G72" s="3" t="s">
+        <v>262</v>
+      </c>
+      <c r="H72" s="17" t="s">
+        <v>64</v>
+      </c>
+      <c r="I72" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="J72" s="12" t="s">
+        <v>253</v>
+      </c>
+      <c r="K72" s="3" t="s">
+        <v>263</v>
+      </c>
+      <c r="L72" s="6" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="73" spans="1:12" ht="26.75" customHeight="1" x14ac:dyDescent="0.2"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>

</xml_diff>

<commit_message>
finalize  30.1 and 30.2 release notes and latest spreadsheet
</commit_message>
<xml_diff>
--- a/tools/data/latest.xlsx
+++ b/tools/data/latest.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="996" uniqueCount="431">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="996" uniqueCount="430">
   <si>
     <t>Name</t>
   </si>
@@ -281,9 +281,6 @@
   </si>
   <si>
     <t>Ongoing/DR independent</t>
-  </si>
-  <si>
-    <t>Demographics</t>
   </si>
   <si>
     <t>[DD+DATA ERROR] Nail type field added for 2.0 all "Unknown"</t>
@@ -1316,7 +1313,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="x14ac">
   <numFmts count="0"/>
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1327,19 +1324,25 @@
     <font>
       <b/>
       <sz val="11"/>
-      <color theme="1"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFffffff"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFffffff"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
@@ -1551,7 +1554,7 @@
     <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="3" applyFont="1" fillId="17" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="4" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="3" applyFont="1" fillId="18" applyFill="1" applyAlignment="1">
@@ -1563,14 +1566,14 @@
     <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="3" applyFont="1" fillId="20" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="4" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="3" applyFont="1" fillId="21" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
+      <alignment horizontal="left"/>
     </xf>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -2459,7 +2462,7 @@
         <v>88</v>
       </c>
       <c r="K15" s="23" t="s">
-        <v>89</v>
+        <v>79</v>
       </c>
       <c r="L15" s="18" t="s">
         <v>47</v>
@@ -2467,7 +2470,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="26.75">
       <c r="A16" s="3" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B16" s="4">
         <v>3</v>
@@ -2479,16 +2482,16 @@
         <v>23</v>
       </c>
       <c r="E16" s="7" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F16" s="7" t="s">
         <v>15</v>
       </c>
       <c r="G16" s="7" t="s">
+        <v>91</v>
+      </c>
+      <c r="H16" s="7" t="s">
         <v>92</v>
-      </c>
-      <c r="H16" s="7" t="s">
-        <v>93</v>
       </c>
       <c r="I16" s="8" t="s">
         <v>18</v>
@@ -2497,7 +2500,7 @@
         <v>27</v>
       </c>
       <c r="K16" s="24" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="L16" s="18" t="s">
         <v>47</v>
@@ -2505,7 +2508,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="26.75">
       <c r="A17" s="3" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B17" s="4">
         <v>3</v>
@@ -2517,25 +2520,25 @@
         <v>35</v>
       </c>
       <c r="E17" s="7" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="F17" s="7" t="s">
         <v>15</v>
       </c>
       <c r="G17" s="7" t="s">
+        <v>96</v>
+      </c>
+      <c r="H17" s="7" t="s">
         <v>97</v>
       </c>
-      <c r="H17" s="7" t="s">
+      <c r="I17" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="J17" s="14" t="s">
         <v>98</v>
       </c>
-      <c r="I17" s="8" t="s">
-        <v>18</v>
-      </c>
-      <c r="J17" s="14" t="s">
+      <c r="K17" s="12" t="s">
         <v>99</v>
-      </c>
-      <c r="K17" s="12" t="s">
-        <v>100</v>
       </c>
       <c r="L17" s="13" t="s">
         <v>28</v>
@@ -2543,7 +2546,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="26.75">
       <c r="A18" s="3" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B18" s="4">
         <v>3</v>
@@ -2555,16 +2558,16 @@
         <v>43</v>
       </c>
       <c r="E18" s="7" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="F18" s="7" t="s">
         <v>54</v>
       </c>
       <c r="G18" s="7" t="s">
+        <v>102</v>
+      </c>
+      <c r="H18" s="7" t="s">
         <v>103</v>
-      </c>
-      <c r="H18" s="7" t="s">
-        <v>104</v>
       </c>
       <c r="I18" s="8" t="s">
         <v>18</v>
@@ -2573,7 +2576,7 @@
         <v>57</v>
       </c>
       <c r="K18" s="24" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="L18" s="13" t="s">
         <v>28</v>
@@ -2581,7 +2584,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="26.75">
       <c r="A19" s="3" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B19" s="4">
         <v>3</v>
@@ -2593,7 +2596,7 @@
         <v>13</v>
       </c>
       <c r="E19" s="7" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="F19" s="7" t="s">
         <v>15</v>
@@ -2602,7 +2605,7 @@
         <v>31</v>
       </c>
       <c r="H19" s="7" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="I19" s="8" t="s">
         <v>18</v>
@@ -2619,7 +2622,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="26.75">
       <c r="A20" s="3" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B20" s="4">
         <v>3</v>
@@ -2631,7 +2634,7 @@
         <v>13</v>
       </c>
       <c r="E20" s="7" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="F20" s="7" t="s">
         <v>15</v>
@@ -2640,7 +2643,7 @@
         <v>25</v>
       </c>
       <c r="H20" s="7" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="I20" s="8" t="s">
         <v>18</v>
@@ -2657,7 +2660,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="21" customHeight="1" ht="26.75">
       <c r="A21" s="3" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B21" s="4">
         <v>3</v>
@@ -2669,7 +2672,7 @@
         <v>13</v>
       </c>
       <c r="E21" s="7" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="F21" s="7" t="s">
         <v>15</v>
@@ -2678,7 +2681,7 @@
         <v>25</v>
       </c>
       <c r="H21" s="7" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="I21" s="8" t="s">
         <v>18</v>
@@ -2695,7 +2698,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="22" customHeight="1" ht="26.75">
       <c r="A22" s="3" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B22" s="4">
         <v>3</v>
@@ -2707,16 +2710,16 @@
         <v>13</v>
       </c>
       <c r="E22" s="7" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="F22" s="7" t="s">
         <v>15</v>
       </c>
       <c r="G22" s="7" t="s">
+        <v>115</v>
+      </c>
+      <c r="H22" s="7" t="s">
         <v>116</v>
-      </c>
-      <c r="H22" s="7" t="s">
-        <v>117</v>
       </c>
       <c r="I22" s="8" t="s">
         <v>18</v>
@@ -2725,7 +2728,7 @@
         <v>19</v>
       </c>
       <c r="K22" s="17" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="L22" s="13" t="s">
         <v>28</v>
@@ -2733,7 +2736,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="23" customHeight="1" ht="26.75">
       <c r="A23" s="3" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="B23" s="4">
         <v>3</v>
@@ -2745,16 +2748,16 @@
         <v>23</v>
       </c>
       <c r="E23" s="7" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="F23" s="7" t="s">
         <v>15</v>
       </c>
       <c r="G23" s="7" t="s">
+        <v>120</v>
+      </c>
+      <c r="H23" s="7" t="s">
         <v>121</v>
-      </c>
-      <c r="H23" s="7" t="s">
-        <v>122</v>
       </c>
       <c r="I23" s="8" t="s">
         <v>18</v>
@@ -2766,12 +2769,12 @@
         <v>33</v>
       </c>
       <c r="L23" s="25" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="24" customHeight="1" ht="26.75">
       <c r="A24" s="3" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="B24" s="4">
         <v>3</v>
@@ -2783,16 +2786,16 @@
         <v>13</v>
       </c>
       <c r="E24" s="7" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F24" s="7" t="s">
         <v>15</v>
       </c>
       <c r="G24" s="7" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="H24" s="7" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="I24" s="8" t="s">
         <v>18</v>
@@ -2801,7 +2804,7 @@
         <v>19</v>
       </c>
       <c r="K24" s="17" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="L24" s="18" t="s">
         <v>47</v>
@@ -2809,7 +2812,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="25" customHeight="1" ht="26.75">
       <c r="A25" s="3" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B25" s="4">
         <v>3</v>
@@ -2821,16 +2824,16 @@
         <v>13</v>
       </c>
       <c r="E25" s="7" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="F25" s="7" t="s">
         <v>54</v>
       </c>
       <c r="G25" s="7" t="s">
+        <v>128</v>
+      </c>
+      <c r="H25" s="7" t="s">
         <v>129</v>
-      </c>
-      <c r="H25" s="7" t="s">
-        <v>130</v>
       </c>
       <c r="I25" s="8" t="s">
         <v>18</v>
@@ -2839,7 +2842,7 @@
         <v>19</v>
       </c>
       <c r="K25" s="6" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="L25" s="13" t="s">
         <v>28</v>
@@ -2847,7 +2850,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="26" customHeight="1" ht="26.75">
       <c r="A26" s="3" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B26" s="4">
         <v>3</v>
@@ -2859,16 +2862,16 @@
         <v>13</v>
       </c>
       <c r="E26" s="7" t="s">
+        <v>132</v>
+      </c>
+      <c r="F26" s="7" t="s">
         <v>133</v>
       </c>
-      <c r="F26" s="7" t="s">
+      <c r="G26" s="7" t="s">
         <v>134</v>
       </c>
-      <c r="G26" s="7" t="s">
+      <c r="H26" s="7" t="s">
         <v>135</v>
-      </c>
-      <c r="H26" s="7" t="s">
-        <v>136</v>
       </c>
       <c r="I26" s="8" t="s">
         <v>18</v>
@@ -2885,7 +2888,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="27" customHeight="1" ht="26.75">
       <c r="A27" s="3" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="B27" s="4">
         <v>3</v>
@@ -2897,25 +2900,25 @@
         <v>43</v>
       </c>
       <c r="E27" s="7" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="F27" s="7" t="s">
         <v>54</v>
       </c>
       <c r="G27" s="7" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="H27" s="7" t="s">
+        <v>138</v>
+      </c>
+      <c r="I27" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="J27" s="8" t="s">
         <v>139</v>
       </c>
-      <c r="I27" s="8" t="s">
-        <v>18</v>
-      </c>
-      <c r="J27" s="8" t="s">
-        <v>140</v>
-      </c>
       <c r="K27" s="17" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="L27" s="18" t="s">
         <v>47</v>
@@ -2923,7 +2926,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="28" customHeight="1" ht="26.75">
       <c r="A28" s="3" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="B28" s="4">
         <v>3</v>
@@ -2935,16 +2938,16 @@
         <v>35</v>
       </c>
       <c r="E28" s="7" t="s">
+        <v>141</v>
+      </c>
+      <c r="F28" s="7" t="s">
         <v>142</v>
       </c>
-      <c r="F28" s="7" t="s">
+      <c r="G28" s="7" t="s">
         <v>143</v>
       </c>
-      <c r="G28" s="7" t="s">
+      <c r="H28" s="7" t="s">
         <v>144</v>
-      </c>
-      <c r="H28" s="7" t="s">
-        <v>145</v>
       </c>
       <c r="I28" s="8" t="s">
         <v>18</v>
@@ -2953,7 +2956,7 @@
         <v>40</v>
       </c>
       <c r="K28" s="17" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="L28" s="13" t="s">
         <v>28</v>
@@ -2961,7 +2964,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="29" customHeight="1" ht="26.75">
       <c r="A29" s="3" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="B29" s="4">
         <v>3</v>
@@ -2973,16 +2976,16 @@
         <v>43</v>
       </c>
       <c r="E29" s="7" t="s">
+        <v>146</v>
+      </c>
+      <c r="F29" s="7" t="s">
         <v>147</v>
       </c>
-      <c r="F29" s="7" t="s">
+      <c r="G29" s="7" t="s">
         <v>148</v>
       </c>
-      <c r="G29" s="7" t="s">
+      <c r="H29" s="7" t="s">
         <v>149</v>
-      </c>
-      <c r="H29" s="7" t="s">
-        <v>150</v>
       </c>
       <c r="I29" s="8" t="s">
         <v>18</v>
@@ -2991,7 +2994,7 @@
         <v>19</v>
       </c>
       <c r="K29" s="17" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="L29" s="13" t="s">
         <v>28</v>
@@ -2999,7 +3002,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="30" customHeight="1" ht="26.75">
       <c r="A30" s="3" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="B30" s="4">
         <v>3</v>
@@ -3011,16 +3014,16 @@
         <v>13</v>
       </c>
       <c r="E30" s="7" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="F30" s="7" t="s">
         <v>15</v>
       </c>
       <c r="G30" s="7" t="s">
+        <v>152</v>
+      </c>
+      <c r="H30" s="7" t="s">
         <v>153</v>
-      </c>
-      <c r="H30" s="7" t="s">
-        <v>154</v>
       </c>
       <c r="I30" s="8" t="s">
         <v>18</v>
@@ -3037,7 +3040,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="31" customHeight="1" ht="26.75">
       <c r="A31" s="3" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="B31" s="4">
         <v>3</v>
@@ -3049,25 +3052,25 @@
         <v>43</v>
       </c>
       <c r="E31" s="7" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="F31" s="7" t="s">
         <v>54</v>
       </c>
       <c r="G31" s="7" t="s">
+        <v>156</v>
+      </c>
+      <c r="H31" s="7" t="s">
         <v>157</v>
       </c>
-      <c r="H31" s="7" t="s">
+      <c r="I31" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="J31" s="8" t="s">
+        <v>139</v>
+      </c>
+      <c r="K31" s="19" t="s">
         <v>158</v>
-      </c>
-      <c r="I31" s="8" t="s">
-        <v>18</v>
-      </c>
-      <c r="J31" s="8" t="s">
-        <v>140</v>
-      </c>
-      <c r="K31" s="19" t="s">
-        <v>159</v>
       </c>
       <c r="L31" s="18" t="s">
         <v>47</v>
@@ -3075,7 +3078,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="32" customHeight="1" ht="26.75">
       <c r="A32" s="3" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="B32" s="4">
         <v>3</v>
@@ -3087,16 +3090,16 @@
         <v>23</v>
       </c>
       <c r="E32" s="7" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="F32" s="7" t="s">
         <v>15</v>
       </c>
       <c r="G32" s="7" t="s">
+        <v>161</v>
+      </c>
+      <c r="H32" s="7" t="s">
         <v>162</v>
-      </c>
-      <c r="H32" s="7" t="s">
-        <v>163</v>
       </c>
       <c r="I32" s="8" t="s">
         <v>18</v>
@@ -3105,7 +3108,7 @@
         <v>27</v>
       </c>
       <c r="K32" s="19" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="L32" s="18" t="s">
         <v>47</v>
@@ -3113,7 +3116,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="33" customHeight="1" ht="26.75">
       <c r="A33" s="3" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="B33" s="4">
         <v>3</v>
@@ -3125,22 +3128,22 @@
         <v>43</v>
       </c>
       <c r="E33" s="7" t="s">
+        <v>164</v>
+      </c>
+      <c r="F33" s="7" t="s">
         <v>165</v>
       </c>
-      <c r="F33" s="7" t="s">
+      <c r="G33" s="7" t="s">
         <v>166</v>
       </c>
-      <c r="G33" s="7" t="s">
+      <c r="H33" s="7" t="s">
         <v>167</v>
       </c>
-      <c r="H33" s="7" t="s">
+      <c r="I33" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="J33" s="21" t="s">
         <v>168</v>
-      </c>
-      <c r="I33" s="8" t="s">
-        <v>18</v>
-      </c>
-      <c r="J33" s="21" t="s">
-        <v>169</v>
       </c>
       <c r="K33" s="16" t="s">
         <v>41</v>
@@ -3151,7 +3154,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="34" customHeight="1" ht="26.75">
       <c r="A34" s="3" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="B34" s="4">
         <v>3</v>
@@ -3163,16 +3166,16 @@
         <v>23</v>
       </c>
       <c r="E34" s="7" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="F34" s="7" t="s">
         <v>37</v>
       </c>
       <c r="G34" s="7" t="s">
+        <v>171</v>
+      </c>
+      <c r="H34" s="7" t="s">
         <v>172</v>
-      </c>
-      <c r="H34" s="7" t="s">
-        <v>173</v>
       </c>
       <c r="I34" s="8" t="s">
         <v>18</v>
@@ -3189,7 +3192,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="35" customHeight="1" ht="26.75">
       <c r="A35" s="3" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="B35" s="4">
         <v>3</v>
@@ -3201,22 +3204,22 @@
         <v>43</v>
       </c>
       <c r="E35" s="7" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="F35" s="7" t="s">
         <v>54</v>
       </c>
       <c r="G35" s="7" t="s">
+        <v>175</v>
+      </c>
+      <c r="H35" s="7" t="s">
         <v>176</v>
       </c>
-      <c r="H35" s="7" t="s">
-        <v>177</v>
-      </c>
       <c r="I35" s="8" t="s">
         <v>18</v>
       </c>
       <c r="J35" s="21" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="K35" s="20" t="s">
         <v>62</v>
@@ -3227,7 +3230,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="36" customHeight="1" ht="26.75">
       <c r="A36" s="3" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="B36" s="4">
         <v>3</v>
@@ -3239,16 +3242,16 @@
         <v>13</v>
       </c>
       <c r="E36" s="7" t="s">
+        <v>178</v>
+      </c>
+      <c r="F36" s="7" t="s">
         <v>179</v>
-      </c>
-      <c r="F36" s="7" t="s">
-        <v>180</v>
       </c>
       <c r="G36" s="7" t="s">
         <v>45</v>
       </c>
       <c r="H36" s="7" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="I36" s="8" t="s">
         <v>18</v>
@@ -3265,7 +3268,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="37" customHeight="1" ht="26.75">
       <c r="A37" s="3" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="B37" s="4">
         <v>3</v>
@@ -3277,16 +3280,16 @@
         <v>13</v>
       </c>
       <c r="E37" s="7" t="s">
+        <v>182</v>
+      </c>
+      <c r="F37" s="7" t="s">
+        <v>179</v>
+      </c>
+      <c r="G37" s="7" t="s">
         <v>183</v>
       </c>
-      <c r="F37" s="7" t="s">
+      <c r="H37" s="7" t="s">
         <v>180</v>
-      </c>
-      <c r="G37" s="7" t="s">
-        <v>184</v>
-      </c>
-      <c r="H37" s="7" t="s">
-        <v>181</v>
       </c>
       <c r="I37" s="8" t="s">
         <v>18</v>
@@ -3303,7 +3306,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="38" customHeight="1" ht="26.75">
       <c r="A38" s="3" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="B38" s="4">
         <v>3</v>
@@ -3315,16 +3318,16 @@
         <v>13</v>
       </c>
       <c r="E38" s="7" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="F38" s="7" t="s">
         <v>15</v>
       </c>
       <c r="G38" s="7" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="H38" s="7" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="I38" s="8" t="s">
         <v>18</v>
@@ -3333,7 +3336,7 @@
         <v>19</v>
       </c>
       <c r="K38" s="19" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="L38" s="10" t="s">
         <v>21</v>
@@ -3341,7 +3344,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="39" customHeight="1" ht="26.75">
       <c r="A39" s="3" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B39" s="4">
         <v>3</v>
@@ -3353,16 +3356,16 @@
         <v>13</v>
       </c>
       <c r="E39" s="7" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="F39" s="7" t="s">
         <v>15</v>
       </c>
       <c r="G39" s="7" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="H39" s="7" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="I39" s="8" t="s">
         <v>18</v>
@@ -3371,7 +3374,7 @@
         <v>19</v>
       </c>
       <c r="K39" s="19" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="L39" s="13" t="s">
         <v>28</v>
@@ -3379,7 +3382,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="40" customHeight="1" ht="26.75">
       <c r="A40" s="3" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="B40" s="4">
         <v>3</v>
@@ -3391,16 +3394,16 @@
         <v>13</v>
       </c>
       <c r="E40" s="7" t="s">
+        <v>191</v>
+      </c>
+      <c r="F40" s="7" t="s">
+        <v>179</v>
+      </c>
+      <c r="G40" s="7" t="s">
         <v>192</v>
       </c>
-      <c r="F40" s="7" t="s">
+      <c r="H40" s="7" t="s">
         <v>180</v>
-      </c>
-      <c r="G40" s="7" t="s">
-        <v>193</v>
-      </c>
-      <c r="H40" s="7" t="s">
-        <v>181</v>
       </c>
       <c r="I40" s="8" t="s">
         <v>18</v>
@@ -3409,15 +3412,15 @@
         <v>19</v>
       </c>
       <c r="K40" s="17" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="L40" s="13" t="s">
         <v>28</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="41" customHeight="1" ht="26.75">
+    <row x14ac:dyDescent="0.25" r="41" customHeight="1" ht="19.5">
       <c r="A41" s="3" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="B41" s="4">
         <v>3</v>
@@ -3429,16 +3432,16 @@
         <v>13</v>
       </c>
       <c r="E41" s="7" t="s">
+        <v>194</v>
+      </c>
+      <c r="F41" s="7" t="s">
+        <v>179</v>
+      </c>
+      <c r="G41" s="7" t="s">
         <v>195</v>
       </c>
-      <c r="F41" s="7" t="s">
+      <c r="H41" s="7" t="s">
         <v>180</v>
-      </c>
-      <c r="G41" s="7" t="s">
-        <v>196</v>
-      </c>
-      <c r="H41" s="7" t="s">
-        <v>181</v>
       </c>
       <c r="I41" s="8" t="s">
         <v>18</v>
@@ -3453,9 +3456,9 @@
         <v>28</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="42" customHeight="1" ht="26.75">
+    <row x14ac:dyDescent="0.25" r="42" customHeight="1" ht="19.5">
       <c r="A42" s="3" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B42" s="4">
         <v>3</v>
@@ -3467,16 +3470,16 @@
         <v>13</v>
       </c>
       <c r="E42" s="7" t="s">
+        <v>197</v>
+      </c>
+      <c r="F42" s="7" t="s">
+        <v>179</v>
+      </c>
+      <c r="G42" s="7" t="s">
         <v>198</v>
       </c>
-      <c r="F42" s="7" t="s">
+      <c r="H42" s="7" t="s">
         <v>180</v>
-      </c>
-      <c r="G42" s="7" t="s">
-        <v>199</v>
-      </c>
-      <c r="H42" s="7" t="s">
-        <v>181</v>
       </c>
       <c r="I42" s="8" t="s">
         <v>18</v>
@@ -3491,9 +3494,9 @@
         <v>28</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="43" customHeight="1" ht="26.75">
+    <row x14ac:dyDescent="0.25" r="43" customHeight="1" ht="46.5">
       <c r="A43" s="3" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="B43" s="4">
         <v>3</v>
@@ -3505,16 +3508,16 @@
         <v>13</v>
       </c>
       <c r="E43" s="7" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="F43" s="7" t="s">
         <v>15</v>
       </c>
       <c r="G43" s="7" t="s">
+        <v>201</v>
+      </c>
+      <c r="H43" s="7" t="s">
         <v>202</v>
-      </c>
-      <c r="H43" s="7" t="s">
-        <v>203</v>
       </c>
       <c r="I43" s="8" t="s">
         <v>18</v>
@@ -3529,9 +3532,9 @@
         <v>21</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="44" customHeight="1" ht="26.75">
+    <row x14ac:dyDescent="0.25" r="44" customHeight="1" ht="19.5">
       <c r="A44" s="3" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="B44" s="4">
         <v>3</v>
@@ -3543,16 +3546,16 @@
         <v>43</v>
       </c>
       <c r="E44" s="7" t="s">
+        <v>204</v>
+      </c>
+      <c r="F44" s="7" t="s">
         <v>205</v>
       </c>
-      <c r="F44" s="7" t="s">
+      <c r="G44" s="7" t="s">
         <v>206</v>
       </c>
-      <c r="G44" s="7" t="s">
+      <c r="H44" s="7" t="s">
         <v>207</v>
-      </c>
-      <c r="H44" s="7" t="s">
-        <v>208</v>
       </c>
       <c r="I44" s="8" t="s">
         <v>18</v>
@@ -3567,9 +3570,9 @@
         <v>28</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="45" customHeight="1" ht="26.75">
+    <row x14ac:dyDescent="0.25" r="45" customHeight="1" ht="19.5">
       <c r="A45" s="3" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="B45" s="4">
         <v>3</v>
@@ -3579,16 +3582,16 @@
         <v>23</v>
       </c>
       <c r="E45" s="7" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="F45" s="7" t="s">
         <v>15</v>
       </c>
       <c r="G45" s="7" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="H45" s="7" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="I45" s="8" t="s">
         <v>18</v>
@@ -3597,15 +3600,15 @@
         <v>27</v>
       </c>
       <c r="K45" s="17" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="L45" s="10" t="s">
         <v>21</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="46" customHeight="1" ht="26.75">
+    <row x14ac:dyDescent="0.25" r="46" customHeight="1" ht="19.5">
       <c r="A46" s="3" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="B46" s="4">
         <v>3</v>
@@ -3617,16 +3620,16 @@
         <v>13</v>
       </c>
       <c r="E46" s="7" t="s">
+        <v>212</v>
+      </c>
+      <c r="F46" s="7" t="s">
         <v>213</v>
       </c>
-      <c r="F46" s="7" t="s">
+      <c r="G46" s="7" t="s">
         <v>214</v>
       </c>
-      <c r="G46" s="7" t="s">
+      <c r="H46" s="7" t="s">
         <v>215</v>
-      </c>
-      <c r="H46" s="7" t="s">
-        <v>216</v>
       </c>
       <c r="I46" s="8" t="s">
         <v>18</v>
@@ -3641,9 +3644,9 @@
         <v>21</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="47" customHeight="1" ht="26.75">
+    <row x14ac:dyDescent="0.25" r="47" customHeight="1" ht="19.5">
       <c r="A47" s="3" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="B47" s="4">
         <v>3</v>
@@ -3655,16 +3658,16 @@
         <v>13</v>
       </c>
       <c r="E47" s="7" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="F47" s="7" t="s">
         <v>15</v>
       </c>
       <c r="G47" s="7" t="s">
+        <v>218</v>
+      </c>
+      <c r="H47" s="7" t="s">
         <v>219</v>
-      </c>
-      <c r="H47" s="7" t="s">
-        <v>220</v>
       </c>
       <c r="I47" s="8" t="s">
         <v>18</v>
@@ -3673,15 +3676,15 @@
         <v>19</v>
       </c>
       <c r="K47" s="17" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="L47" s="10" t="s">
         <v>21</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="48" customHeight="1" ht="26.75">
+    <row x14ac:dyDescent="0.25" r="48" customHeight="1" ht="19.5">
       <c r="A48" s="3" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="B48" s="4">
         <v>3</v>
@@ -3693,16 +3696,16 @@
         <v>13</v>
       </c>
       <c r="E48" s="7" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="F48" s="7" t="s">
         <v>15</v>
       </c>
       <c r="G48" s="7" t="s">
+        <v>222</v>
+      </c>
+      <c r="H48" s="7" t="s">
         <v>223</v>
-      </c>
-      <c r="H48" s="7" t="s">
-        <v>224</v>
       </c>
       <c r="I48" s="8" t="s">
         <v>18</v>
@@ -3717,9 +3720,9 @@
         <v>21</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="49" customHeight="1" ht="26.75">
+    <row x14ac:dyDescent="0.25" r="49" customHeight="1" ht="19.5">
       <c r="A49" s="3" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="B49" s="4">
         <v>3</v>
@@ -3729,33 +3732,33 @@
         <v>35</v>
       </c>
       <c r="E49" s="7" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="F49" s="7" t="s">
         <v>15</v>
       </c>
       <c r="G49" s="7" t="s">
+        <v>226</v>
+      </c>
+      <c r="H49" s="7" t="s">
         <v>227</v>
       </c>
-      <c r="H49" s="7" t="s">
-        <v>228</v>
-      </c>
       <c r="I49" s="8" t="s">
         <v>18</v>
       </c>
       <c r="J49" s="14" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="K49" s="17" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="L49" s="18" t="s">
         <v>47</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="50" customHeight="1" ht="26.75">
+    <row x14ac:dyDescent="0.25" r="50" customHeight="1" ht="19.5">
       <c r="A50" s="3" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="B50" s="4">
         <v>3</v>
@@ -3765,16 +3768,16 @@
         <v>23</v>
       </c>
       <c r="E50" s="7" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="F50" s="7" t="s">
         <v>15</v>
       </c>
       <c r="G50" s="7" t="s">
+        <v>230</v>
+      </c>
+      <c r="H50" s="7" t="s">
         <v>231</v>
-      </c>
-      <c r="H50" s="7" t="s">
-        <v>232</v>
       </c>
       <c r="I50" s="8" t="s">
         <v>18</v>
@@ -3786,12 +3789,12 @@
         <v>79</v>
       </c>
       <c r="L50" s="25" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="51" customHeight="1" ht="26.75">
+        <v>122</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="51" customHeight="1" ht="19.5">
       <c r="A51" s="3" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="B51" s="4">
         <v>3</v>
@@ -3803,14 +3806,14 @@
         <v>13</v>
       </c>
       <c r="E51" s="7" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="F51" s="26"/>
       <c r="G51" s="7" t="s">
         <v>25</v>
       </c>
       <c r="H51" s="7" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="I51" s="8" t="s">
         <v>18</v>
@@ -3827,7 +3830,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="52" customHeight="1" ht="26.75">
       <c r="A52" s="3" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="B52" s="4">
         <v>3</v>
@@ -3837,22 +3840,22 @@
         <v>35</v>
       </c>
       <c r="E52" s="7" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="F52" s="7" t="s">
         <v>15</v>
       </c>
       <c r="G52" s="7" t="s">
+        <v>237</v>
+      </c>
+      <c r="H52" s="7" t="s">
         <v>238</v>
       </c>
-      <c r="H52" s="7" t="s">
-        <v>239</v>
-      </c>
       <c r="I52" s="8" t="s">
         <v>18</v>
       </c>
       <c r="J52" s="14" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="K52" s="21" t="s">
         <v>79</v>
@@ -3863,7 +3866,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="53" customHeight="1" ht="26.75">
       <c r="A53" s="3" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="B53" s="4">
         <v>3</v>
@@ -3873,16 +3876,16 @@
         <v>23</v>
       </c>
       <c r="E53" s="7" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="F53" s="7" t="s">
         <v>37</v>
       </c>
       <c r="G53" s="7" t="s">
+        <v>241</v>
+      </c>
+      <c r="H53" s="7" t="s">
         <v>242</v>
-      </c>
-      <c r="H53" s="7" t="s">
-        <v>243</v>
       </c>
       <c r="I53" s="8" t="s">
         <v>18</v>
@@ -3899,7 +3902,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="54" customHeight="1" ht="26.75">
       <c r="A54" s="3" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="B54" s="4">
         <v>3</v>
@@ -3909,16 +3912,16 @@
         <v>23</v>
       </c>
       <c r="E54" s="7" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="F54" s="7" t="s">
         <v>37</v>
       </c>
       <c r="G54" s="7" t="s">
+        <v>245</v>
+      </c>
+      <c r="H54" s="7" t="s">
         <v>246</v>
-      </c>
-      <c r="H54" s="7" t="s">
-        <v>247</v>
       </c>
       <c r="I54" s="8" t="s">
         <v>18</v>
@@ -3935,7 +3938,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="55" customHeight="1" ht="26.75">
       <c r="A55" s="3" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="B55" s="4">
         <v>3</v>
@@ -3947,14 +3950,14 @@
         <v>13</v>
       </c>
       <c r="E55" s="7" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="F55" s="26"/>
       <c r="G55" s="7" t="s">
         <v>77</v>
       </c>
       <c r="H55" s="7" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="I55" s="8" t="s">
         <v>18</v>
@@ -3971,7 +3974,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="56" customHeight="1" ht="26.75">
       <c r="A56" s="3" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="B56" s="4">
         <v>3</v>
@@ -3983,7 +3986,7 @@
         <v>35</v>
       </c>
       <c r="E56" s="7" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="F56" s="7" t="s">
         <v>15</v>
@@ -3992,13 +3995,13 @@
         <v>77</v>
       </c>
       <c r="H56" s="7" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="I56" s="8" t="s">
         <v>18</v>
       </c>
       <c r="J56" s="14" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="K56" s="21" t="s">
         <v>79</v>
@@ -4009,7 +4012,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="57" customHeight="1" ht="26.75">
       <c r="A57" s="3" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="B57" s="4">
         <v>3</v>
@@ -4021,16 +4024,16 @@
         <v>13</v>
       </c>
       <c r="E57" s="7" t="s">
+        <v>254</v>
+      </c>
+      <c r="F57" s="7" t="s">
         <v>255</v>
       </c>
-      <c r="F57" s="7" t="s">
+      <c r="G57" s="7" t="s">
         <v>256</v>
       </c>
-      <c r="G57" s="7" t="s">
+      <c r="H57" s="7" t="s">
         <v>257</v>
-      </c>
-      <c r="H57" s="7" t="s">
-        <v>258</v>
       </c>
       <c r="I57" s="8" t="s">
         <v>18</v>
@@ -4047,7 +4050,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="58" customHeight="1" ht="26.75">
       <c r="A58" s="3" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="B58" s="4">
         <v>3</v>
@@ -4057,7 +4060,7 @@
         <v>35</v>
       </c>
       <c r="E58" s="7" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="F58" s="7" t="s">
         <v>15</v>
@@ -4066,16 +4069,16 @@
         <v>86</v>
       </c>
       <c r="H58" s="7" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="I58" s="8" t="s">
         <v>18</v>
       </c>
       <c r="J58" s="14" t="s">
+        <v>98</v>
+      </c>
+      <c r="K58" s="12" t="s">
         <v>99</v>
-      </c>
-      <c r="K58" s="12" t="s">
-        <v>100</v>
       </c>
       <c r="L58" s="10" t="s">
         <v>21</v>
@@ -4083,7 +4086,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="59" customHeight="1" ht="26.75">
       <c r="A59" s="3" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="B59" s="4">
         <v>3</v>
@@ -4093,7 +4096,7 @@
         <v>23</v>
       </c>
       <c r="E59" s="7" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="F59" s="7" t="s">
         <v>15</v>
@@ -4102,7 +4105,7 @@
         <v>86</v>
       </c>
       <c r="H59" s="7" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="I59" s="8" t="s">
         <v>18</v>
@@ -4111,7 +4114,7 @@
         <v>27</v>
       </c>
       <c r="K59" s="12" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="L59" s="10" t="s">
         <v>21</v>
@@ -4119,7 +4122,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="60" customHeight="1" ht="26.75">
       <c r="A60" s="3" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="B60" s="4">
         <v>3</v>
@@ -4131,22 +4134,22 @@
         <v>13</v>
       </c>
       <c r="E60" s="7" t="s">
+        <v>265</v>
+      </c>
+      <c r="F60" s="7" t="s">
+        <v>255</v>
+      </c>
+      <c r="G60" s="7" t="s">
         <v>266</v>
       </c>
-      <c r="F60" s="7" t="s">
-        <v>256</v>
-      </c>
-      <c r="G60" s="7" t="s">
+      <c r="H60" s="7" t="s">
         <v>267</v>
       </c>
-      <c r="H60" s="7" t="s">
-        <v>268</v>
-      </c>
       <c r="I60" s="8" t="s">
         <v>18</v>
       </c>
       <c r="J60" s="21" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="K60" s="20" t="s">
         <v>62</v>
@@ -4157,7 +4160,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="61" customHeight="1" ht="26.75">
       <c r="A61" s="3" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="B61" s="4">
         <v>3</v>
@@ -4167,22 +4170,22 @@
         <v>35</v>
       </c>
       <c r="E61" s="7" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="F61" s="7" t="s">
         <v>15</v>
       </c>
       <c r="G61" s="7" t="s">
+        <v>270</v>
+      </c>
+      <c r="H61" s="7" t="s">
         <v>271</v>
       </c>
-      <c r="H61" s="7" t="s">
-        <v>272</v>
-      </c>
       <c r="I61" s="8" t="s">
         <v>18</v>
       </c>
       <c r="J61" s="14" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="K61" s="14" t="s">
         <v>33</v>
@@ -4193,7 +4196,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="62" customHeight="1" ht="26.75">
       <c r="A62" s="3" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="B62" s="4">
         <v>3</v>
@@ -4203,14 +4206,14 @@
         <v>35</v>
       </c>
       <c r="E62" s="7" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="F62" s="26"/>
       <c r="G62" s="7" t="s">
+        <v>274</v>
+      </c>
+      <c r="H62" s="7" t="s">
         <v>275</v>
-      </c>
-      <c r="H62" s="7" t="s">
-        <v>276</v>
       </c>
       <c r="I62" s="8" t="s">
         <v>18</v>
@@ -4219,15 +4222,15 @@
         <v>88</v>
       </c>
       <c r="K62" s="24" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="L62" s="25" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="63" customHeight="1" ht="26.75">
       <c r="A63" s="3" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="B63" s="4">
         <v>3</v>
@@ -4237,16 +4240,16 @@
         <v>23</v>
       </c>
       <c r="E63" s="7" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="F63" s="7" t="s">
         <v>15</v>
       </c>
       <c r="G63" s="7" t="s">
+        <v>278</v>
+      </c>
+      <c r="H63" s="7" t="s">
         <v>279</v>
-      </c>
-      <c r="H63" s="7" t="s">
-        <v>280</v>
       </c>
       <c r="I63" s="8" t="s">
         <v>18</v>
@@ -4258,12 +4261,12 @@
         <v>79</v>
       </c>
       <c r="L63" s="25" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="64" customHeight="1" ht="26.75">
       <c r="A64" s="3" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="B64" s="4">
         <v>3</v>
@@ -4273,16 +4276,16 @@
         <v>23</v>
       </c>
       <c r="E64" s="7" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="F64" s="7" t="s">
         <v>15</v>
       </c>
       <c r="G64" s="7" t="s">
+        <v>282</v>
+      </c>
+      <c r="H64" s="7" t="s">
         <v>283</v>
-      </c>
-      <c r="H64" s="7" t="s">
-        <v>284</v>
       </c>
       <c r="I64" s="8" t="s">
         <v>18</v>
@@ -4291,7 +4294,7 @@
         <v>27</v>
       </c>
       <c r="K64" s="12" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="L64" s="10" t="s">
         <v>21</v>
@@ -4299,7 +4302,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="65" customHeight="1" ht="26.75">
       <c r="A65" s="3" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="B65" s="4">
         <v>3</v>
@@ -4311,14 +4314,14 @@
         <v>13</v>
       </c>
       <c r="E65" s="7" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="F65" s="26"/>
       <c r="G65" s="7" t="s">
+        <v>286</v>
+      </c>
+      <c r="H65" s="7" t="s">
         <v>287</v>
-      </c>
-      <c r="H65" s="7" t="s">
-        <v>288</v>
       </c>
       <c r="I65" s="8" t="s">
         <v>18</v>
@@ -4327,15 +4330,15 @@
         <v>19</v>
       </c>
       <c r="K65" s="6" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="L65" s="25" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="66" customHeight="1" ht="26.75">
       <c r="A66" s="3" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="B66" s="4">
         <v>3</v>
@@ -4347,31 +4350,31 @@
         <v>13</v>
       </c>
       <c r="E66" s="7" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="F66" s="26"/>
       <c r="G66" s="7" t="s">
+        <v>290</v>
+      </c>
+      <c r="H66" s="7" t="s">
         <v>291</v>
       </c>
-      <c r="H66" s="7" t="s">
-        <v>292</v>
-      </c>
       <c r="I66" s="8" t="s">
         <v>18</v>
       </c>
       <c r="J66" s="8" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="K66" s="16" t="s">
         <v>41</v>
       </c>
       <c r="L66" s="25" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="67" customHeight="1" ht="26.75">
       <c r="A67" s="3" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="B67" s="4">
         <v>3</v>
@@ -4381,16 +4384,16 @@
         <v>23</v>
       </c>
       <c r="E67" s="7" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="F67" s="7" t="s">
         <v>15</v>
       </c>
       <c r="G67" s="7" t="s">
+        <v>294</v>
+      </c>
+      <c r="H67" s="7" t="s">
         <v>295</v>
-      </c>
-      <c r="H67" s="7" t="s">
-        <v>296</v>
       </c>
       <c r="I67" s="8" t="s">
         <v>18</v>
@@ -4399,7 +4402,7 @@
         <v>27</v>
       </c>
       <c r="K67" s="24" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="L67" s="18" t="s">
         <v>47</v>
@@ -4407,7 +4410,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="68" customHeight="1" ht="26.75">
       <c r="A68" s="3" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="B68" s="4">
         <v>3</v>
@@ -4419,16 +4422,16 @@
         <v>23</v>
       </c>
       <c r="E68" s="7" t="s">
+        <v>297</v>
+      </c>
+      <c r="F68" s="7" t="s">
         <v>298</v>
       </c>
-      <c r="F68" s="7" t="s">
+      <c r="G68" s="7" t="s">
         <v>299</v>
       </c>
-      <c r="G68" s="7" t="s">
+      <c r="H68" s="7" t="s">
         <v>300</v>
-      </c>
-      <c r="H68" s="7" t="s">
-        <v>301</v>
       </c>
       <c r="I68" s="8" t="s">
         <v>18</v>
@@ -4437,15 +4440,15 @@
         <v>27</v>
       </c>
       <c r="K68" s="17" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="L68" s="25" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="69" customHeight="1" ht="26.75">
       <c r="A69" s="3" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="B69" s="22"/>
       <c r="C69" s="22"/>
@@ -4453,16 +4456,16 @@
         <v>35</v>
       </c>
       <c r="E69" s="7" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="F69" s="7" t="s">
         <v>15</v>
       </c>
       <c r="G69" s="7" t="s">
+        <v>303</v>
+      </c>
+      <c r="H69" s="7" t="s">
         <v>304</v>
-      </c>
-      <c r="H69" s="7" t="s">
-        <v>305</v>
       </c>
       <c r="I69" s="8" t="s">
         <v>18</v>
@@ -4479,7 +4482,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="70" customHeight="1" ht="26.75">
       <c r="A70" s="3" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="B70" s="22"/>
       <c r="C70" s="22"/>
@@ -4487,22 +4490,22 @@
         <v>35</v>
       </c>
       <c r="E70" s="7" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="F70" s="7" t="s">
         <v>54</v>
       </c>
       <c r="G70" s="7" t="s">
+        <v>307</v>
+      </c>
+      <c r="H70" s="7" t="s">
         <v>308</v>
       </c>
-      <c r="H70" s="7" t="s">
+      <c r="I70" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="J70" s="15" t="s">
         <v>309</v>
-      </c>
-      <c r="I70" s="8" t="s">
-        <v>18</v>
-      </c>
-      <c r="J70" s="15" t="s">
-        <v>310</v>
       </c>
       <c r="K70" s="16" t="s">
         <v>41</v>
@@ -4513,7 +4516,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="71" customHeight="1" ht="26.75">
       <c r="A71" s="3" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="B71" s="22"/>
       <c r="C71" s="22"/>
@@ -4521,25 +4524,25 @@
         <v>35</v>
       </c>
       <c r="E71" s="7" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="F71" s="7" t="s">
         <v>15</v>
       </c>
       <c r="G71" s="7" t="s">
+        <v>312</v>
+      </c>
+      <c r="H71" s="7" t="s">
         <v>313</v>
       </c>
-      <c r="H71" s="7" t="s">
-        <v>314</v>
-      </c>
       <c r="I71" s="8" t="s">
         <v>18</v>
       </c>
       <c r="J71" s="15" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="K71" s="19" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="L71" s="18" t="s">
         <v>47</v>
@@ -4547,7 +4550,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="72" customHeight="1" ht="26.75">
       <c r="A72" s="3" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="B72" s="22"/>
       <c r="C72" s="22"/>
@@ -4555,22 +4558,22 @@
         <v>35</v>
       </c>
       <c r="E72" s="7" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="F72" s="7" t="s">
         <v>15</v>
       </c>
       <c r="G72" s="7" t="s">
+        <v>316</v>
+      </c>
+      <c r="H72" s="7" t="s">
         <v>317</v>
       </c>
-      <c r="H72" s="7" t="s">
+      <c r="I72" s="16" t="s">
         <v>318</v>
       </c>
-      <c r="I72" s="16" t="s">
-        <v>319</v>
-      </c>
       <c r="J72" s="15" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="K72" s="16" t="s">
         <v>41</v>
@@ -4581,7 +4584,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="73" customHeight="1" ht="26.75">
       <c r="A73" s="3" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="B73" s="22"/>
       <c r="C73" s="22"/>
@@ -4589,22 +4592,22 @@
         <v>35</v>
       </c>
       <c r="E73" s="7" t="s">
+        <v>320</v>
+      </c>
+      <c r="F73" s="7" t="s">
+        <v>213</v>
+      </c>
+      <c r="G73" s="7" t="s">
         <v>321</v>
       </c>
-      <c r="F73" s="7" t="s">
-        <v>214</v>
-      </c>
-      <c r="G73" s="7" t="s">
+      <c r="H73" s="7" t="s">
         <v>322</v>
       </c>
-      <c r="H73" s="7" t="s">
-        <v>323</v>
-      </c>
       <c r="I73" s="8" t="s">
         <v>18</v>
       </c>
       <c r="J73" s="15" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="K73" s="20" t="s">
         <v>62</v>
@@ -4615,7 +4618,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="74" customHeight="1" ht="26.75">
       <c r="A74" s="3" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="B74" s="22"/>
       <c r="C74" s="22"/>
@@ -4623,16 +4626,16 @@
         <v>35</v>
       </c>
       <c r="E74" s="7" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="F74" s="7" t="s">
         <v>15</v>
       </c>
       <c r="G74" s="7" t="s">
+        <v>325</v>
+      </c>
+      <c r="H74" s="7" t="s">
         <v>326</v>
-      </c>
-      <c r="H74" s="7" t="s">
-        <v>327</v>
       </c>
       <c r="I74" s="8" t="s">
         <v>18</v>
@@ -4649,7 +4652,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="75" customHeight="1" ht="26.75">
       <c r="A75" s="3" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="B75" s="22"/>
       <c r="C75" s="22"/>
@@ -4657,16 +4660,16 @@
         <v>35</v>
       </c>
       <c r="E75" s="7" t="s">
+        <v>328</v>
+      </c>
+      <c r="F75" s="7" t="s">
         <v>329</v>
       </c>
-      <c r="F75" s="7" t="s">
+      <c r="G75" s="7" t="s">
         <v>330</v>
       </c>
-      <c r="G75" s="7" t="s">
+      <c r="H75" s="7" t="s">
         <v>331</v>
-      </c>
-      <c r="H75" s="7" t="s">
-        <v>332</v>
       </c>
       <c r="I75" s="8" t="s">
         <v>18</v>
@@ -4675,7 +4678,7 @@
         <v>88</v>
       </c>
       <c r="K75" s="12" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="L75" s="18" t="s">
         <v>47</v>
@@ -4683,7 +4686,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="76" customHeight="1" ht="26.75">
       <c r="A76" s="3" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="B76" s="22"/>
       <c r="C76" s="22"/>
@@ -4691,16 +4694,16 @@
         <v>35</v>
       </c>
       <c r="E76" s="7" t="s">
+        <v>333</v>
+      </c>
+      <c r="F76" s="7" t="s">
+        <v>329</v>
+      </c>
+      <c r="G76" s="7" t="s">
+        <v>330</v>
+      </c>
+      <c r="H76" s="7" t="s">
         <v>334</v>
-      </c>
-      <c r="F76" s="7" t="s">
-        <v>330</v>
-      </c>
-      <c r="G76" s="7" t="s">
-        <v>331</v>
-      </c>
-      <c r="H76" s="7" t="s">
-        <v>335</v>
       </c>
       <c r="I76" s="8" t="s">
         <v>18</v>
@@ -4709,7 +4712,7 @@
         <v>88</v>
       </c>
       <c r="K76" s="12" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="L76" s="18" t="s">
         <v>47</v>
@@ -4717,7 +4720,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="77" customHeight="1" ht="26.75">
       <c r="A77" s="3" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="B77" s="22"/>
       <c r="C77" s="22"/>
@@ -4725,22 +4728,22 @@
         <v>35</v>
       </c>
       <c r="E77" s="7" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="F77" s="7" t="s">
         <v>15</v>
       </c>
       <c r="G77" s="7" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="H77" s="7" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="I77" s="8" t="s">
         <v>18</v>
       </c>
       <c r="J77" s="14" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="K77" s="16" t="s">
         <v>41</v>
@@ -4751,7 +4754,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="78" customHeight="1" ht="26.75">
       <c r="A78" s="3" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="B78" s="22"/>
       <c r="C78" s="22"/>
@@ -4759,25 +4762,25 @@
         <v>35</v>
       </c>
       <c r="E78" s="7" t="s">
+        <v>339</v>
+      </c>
+      <c r="F78" s="7" t="s">
         <v>340</v>
-      </c>
-      <c r="F78" s="7" t="s">
-        <v>341</v>
       </c>
       <c r="G78" s="7" t="s">
         <v>86</v>
       </c>
       <c r="H78" s="7" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="I78" s="16" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="J78" s="15" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="K78" s="12" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="L78" s="18" t="s">
         <v>47</v>
@@ -4785,7 +4788,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="79" customHeight="1" ht="26.75">
       <c r="A79" s="3" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="B79" s="22"/>
       <c r="C79" s="22"/>
@@ -4793,22 +4796,22 @@
         <v>35</v>
       </c>
       <c r="E79" s="7" t="s">
+        <v>343</v>
+      </c>
+      <c r="F79" s="7" t="s">
         <v>344</v>
       </c>
-      <c r="F79" s="7" t="s">
+      <c r="G79" s="7" t="s">
         <v>345</v>
       </c>
-      <c r="G79" s="7" t="s">
+      <c r="H79" s="7" t="s">
         <v>346</v>
       </c>
-      <c r="H79" s="7" t="s">
-        <v>347</v>
-      </c>
       <c r="I79" s="8" t="s">
         <v>18</v>
       </c>
       <c r="J79" s="15" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="K79" s="14" t="s">
         <v>33</v>
@@ -4819,7 +4822,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="80" customHeight="1" ht="26.75">
       <c r="A80" s="3" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="B80" s="22"/>
       <c r="C80" s="22"/>
@@ -4827,22 +4830,22 @@
         <v>35</v>
       </c>
       <c r="E80" s="7" t="s">
+        <v>348</v>
+      </c>
+      <c r="F80" s="7" t="s">
+        <v>213</v>
+      </c>
+      <c r="G80" s="7" t="s">
         <v>349</v>
       </c>
-      <c r="F80" s="7" t="s">
-        <v>214</v>
-      </c>
-      <c r="G80" s="7" t="s">
+      <c r="H80" s="7" t="s">
         <v>350</v>
       </c>
-      <c r="H80" s="7" t="s">
-        <v>351</v>
-      </c>
       <c r="I80" s="8" t="s">
         <v>18</v>
       </c>
       <c r="J80" s="15" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="K80" s="20" t="s">
         <v>62</v>
@@ -4853,7 +4856,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="81" customHeight="1" ht="26.75">
       <c r="A81" s="3" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="B81" s="22"/>
       <c r="C81" s="22"/>
@@ -4861,20 +4864,20 @@
         <v>35</v>
       </c>
       <c r="E81" s="7" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="F81" s="26"/>
       <c r="G81" s="7" t="s">
+        <v>353</v>
+      </c>
+      <c r="H81" s="7" t="s">
         <v>354</v>
       </c>
-      <c r="H81" s="7" t="s">
+      <c r="I81" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="J81" s="20" t="s">
         <v>355</v>
-      </c>
-      <c r="I81" s="8" t="s">
-        <v>18</v>
-      </c>
-      <c r="J81" s="20" t="s">
-        <v>356</v>
       </c>
       <c r="K81" s="20" t="s">
         <v>62</v>
@@ -4885,7 +4888,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="82" customHeight="1" ht="26.75">
       <c r="A82" s="3" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="B82" s="5">
         <v>3.1</v>
@@ -4895,16 +4898,16 @@
         <v>35</v>
       </c>
       <c r="E82" s="7" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="F82" s="7" t="s">
         <v>15</v>
       </c>
       <c r="G82" s="7" t="s">
+        <v>358</v>
+      </c>
+      <c r="H82" s="7" t="s">
         <v>359</v>
-      </c>
-      <c r="H82" s="7" t="s">
-        <v>360</v>
       </c>
       <c r="I82" s="8" t="s">
         <v>18</v>
@@ -4913,7 +4916,7 @@
         <v>88</v>
       </c>
       <c r="K82" s="11" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="L82" s="18" t="s">
         <v>47</v>
@@ -4921,7 +4924,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="83" customHeight="1" ht="26.75">
       <c r="A83" s="3" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="B83" s="5">
         <v>3.1</v>
@@ -4931,16 +4934,16 @@
         <v>35</v>
       </c>
       <c r="E83" s="7" t="s">
+        <v>362</v>
+      </c>
+      <c r="F83" s="7" t="s">
+        <v>255</v>
+      </c>
+      <c r="G83" s="7" t="s">
         <v>363</v>
       </c>
-      <c r="F83" s="7" t="s">
-        <v>256</v>
-      </c>
-      <c r="G83" s="7" t="s">
+      <c r="H83" s="7" t="s">
         <v>364</v>
-      </c>
-      <c r="H83" s="7" t="s">
-        <v>365</v>
       </c>
       <c r="I83" s="8" t="s">
         <v>18</v>
@@ -4957,7 +4960,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="84" customHeight="1" ht="26.75">
       <c r="A84" s="3" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="B84" s="4">
         <v>3</v>
@@ -4969,25 +4972,25 @@
         <v>35</v>
       </c>
       <c r="E84" s="7" t="s">
+        <v>366</v>
+      </c>
+      <c r="F84" s="7" t="s">
         <v>367</v>
       </c>
-      <c r="F84" s="7" t="s">
+      <c r="G84" s="7" t="s">
         <v>368</v>
       </c>
-      <c r="G84" s="7" t="s">
+      <c r="H84" s="7" t="s">
         <v>369</v>
       </c>
-      <c r="H84" s="7" t="s">
+      <c r="I84" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="J84" s="27" t="s">
         <v>370</v>
       </c>
-      <c r="I84" s="8" t="s">
-        <v>18</v>
-      </c>
-      <c r="J84" s="27" t="s">
-        <v>371</v>
-      </c>
       <c r="K84" s="23" t="s">
-        <v>89</v>
+        <v>79</v>
       </c>
       <c r="L84" s="18" t="s">
         <v>47</v>
@@ -4995,7 +4998,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="85" customHeight="1" ht="26.75">
       <c r="A85" s="3" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="B85" s="4">
         <v>3</v>
@@ -5007,25 +5010,25 @@
         <v>35</v>
       </c>
       <c r="E85" s="7" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="F85" s="7" t="s">
         <v>15</v>
       </c>
       <c r="G85" s="7" t="s">
+        <v>373</v>
+      </c>
+      <c r="H85" s="7" t="s">
         <v>374</v>
       </c>
-      <c r="H85" s="7" t="s">
-        <v>375</v>
-      </c>
       <c r="I85" s="8" t="s">
         <v>18</v>
       </c>
       <c r="J85" s="27" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="K85" s="19" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="L85" s="18" t="s">
         <v>47</v>
@@ -5033,7 +5036,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="86" customHeight="1" ht="26.75">
       <c r="A86" s="3" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="B86" s="4">
         <v>3</v>
@@ -5042,28 +5045,28 @@
         <v>30</v>
       </c>
       <c r="D86" s="16" t="s">
+        <v>376</v>
+      </c>
+      <c r="E86" s="7" t="s">
         <v>377</v>
       </c>
-      <c r="E86" s="7" t="s">
+      <c r="F86" s="7" t="s">
         <v>378</v>
       </c>
-      <c r="F86" s="7" t="s">
+      <c r="G86" s="7" t="s">
+        <v>286</v>
+      </c>
+      <c r="H86" s="7" t="s">
         <v>379</v>
       </c>
-      <c r="G86" s="7" t="s">
-        <v>287</v>
-      </c>
-      <c r="H86" s="7" t="s">
+      <c r="I86" s="17" t="s">
         <v>380</v>
       </c>
-      <c r="I86" s="17" t="s">
-        <v>381</v>
-      </c>
       <c r="J86" s="8" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="K86" s="6" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="L86" s="13" t="s">
         <v>28</v>
@@ -5071,7 +5074,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="87" customHeight="1" ht="26.75">
       <c r="A87" s="3" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="B87" s="4">
         <v>3</v>
@@ -5080,28 +5083,28 @@
         <v>30</v>
       </c>
       <c r="D87" s="16" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="E87" s="7" t="s">
+        <v>382</v>
+      </c>
+      <c r="F87" s="7" t="s">
+        <v>255</v>
+      </c>
+      <c r="G87" s="7" t="s">
+        <v>381</v>
+      </c>
+      <c r="H87" s="7" t="s">
         <v>383</v>
       </c>
-      <c r="F87" s="7" t="s">
-        <v>256</v>
-      </c>
-      <c r="G87" s="7" t="s">
-        <v>382</v>
-      </c>
-      <c r="H87" s="7" t="s">
-        <v>384</v>
-      </c>
       <c r="I87" s="17" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="J87" s="8" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="K87" s="11" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="L87" s="13" t="s">
         <v>28</v>
@@ -5109,7 +5112,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="88" customHeight="1" ht="26.75">
       <c r="A88" s="3" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="B88" s="4">
         <v>3</v>
@@ -5118,25 +5121,25 @@
         <v>30.1</v>
       </c>
       <c r="D88" s="16" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="E88" s="7" t="s">
+        <v>385</v>
+      </c>
+      <c r="F88" s="7" t="s">
+        <v>255</v>
+      </c>
+      <c r="G88" s="7" t="s">
         <v>386</v>
       </c>
-      <c r="F88" s="7" t="s">
-        <v>256</v>
-      </c>
-      <c r="G88" s="7" t="s">
+      <c r="H88" s="7" t="s">
         <v>387</v>
       </c>
-      <c r="H88" s="7" t="s">
-        <v>388</v>
-      </c>
       <c r="I88" s="17" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="J88" s="8" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="K88" s="20" t="s">
         <v>62</v>
@@ -5147,7 +5150,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="89" customHeight="1" ht="26.75">
       <c r="A89" s="3" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="B89" s="4">
         <v>3</v>
@@ -5156,28 +5159,28 @@
         <v>30</v>
       </c>
       <c r="D89" s="16" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="E89" s="7" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="F89" s="7" t="s">
         <v>54</v>
       </c>
       <c r="G89" s="7" t="s">
+        <v>390</v>
+      </c>
+      <c r="H89" s="7" t="s">
         <v>391</v>
       </c>
-      <c r="H89" s="7" t="s">
-        <v>392</v>
-      </c>
       <c r="I89" s="17" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="J89" s="8" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="K89" s="19" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="L89" s="13" t="s">
         <v>28</v>
@@ -5185,7 +5188,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="90" customHeight="1" ht="26.75">
       <c r="A90" s="3" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="B90" s="4">
         <v>3</v>
@@ -5194,25 +5197,25 @@
         <v>30</v>
       </c>
       <c r="D90" s="16" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="E90" s="7" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="F90" s="7" t="s">
         <v>54</v>
       </c>
       <c r="G90" s="7" t="s">
+        <v>394</v>
+      </c>
+      <c r="H90" s="7" t="s">
         <v>395</v>
       </c>
-      <c r="H90" s="7" t="s">
-        <v>396</v>
-      </c>
       <c r="I90" s="17" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="J90" s="8" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="K90" s="8" t="s">
         <v>20</v>
@@ -5223,7 +5226,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="91" customHeight="1" ht="26.75">
       <c r="A91" s="3" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
       <c r="B91" s="4">
         <v>3</v>
@@ -5232,25 +5235,25 @@
         <v>30</v>
       </c>
       <c r="D91" s="16" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="E91" s="7" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="F91" s="7" t="s">
         <v>54</v>
       </c>
       <c r="G91" s="7" t="s">
+        <v>398</v>
+      </c>
+      <c r="H91" s="7" t="s">
         <v>399</v>
       </c>
-      <c r="H91" s="7" t="s">
-        <v>400</v>
-      </c>
       <c r="I91" s="17" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="J91" s="8" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="K91" s="8" t="s">
         <v>20</v>
@@ -5261,7 +5264,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="92" customHeight="1" ht="26.75">
       <c r="A92" s="3" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="B92" s="4">
         <v>3</v>
@@ -5270,28 +5273,28 @@
         <v>30</v>
       </c>
       <c r="D92" s="16" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="E92" s="7" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="F92" s="7" t="s">
         <v>54</v>
       </c>
       <c r="G92" s="7" t="s">
+        <v>402</v>
+      </c>
+      <c r="H92" s="7" t="s">
         <v>403</v>
       </c>
-      <c r="H92" s="7" t="s">
-        <v>404</v>
-      </c>
       <c r="I92" s="17" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="J92" s="8" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="K92" s="19" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="L92" s="13" t="s">
         <v>28</v>
@@ -5299,7 +5302,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="93" customHeight="1" ht="26.75">
       <c r="A93" s="3" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
       <c r="B93" s="4">
         <v>3</v>
@@ -5308,28 +5311,28 @@
         <v>30</v>
       </c>
       <c r="D93" s="16" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="E93" s="7" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="F93" s="7" t="s">
         <v>54</v>
       </c>
       <c r="G93" s="7" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="H93" s="7" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="I93" s="17" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="J93" s="8" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="K93" s="17" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="L93" s="13" t="s">
         <v>28</v>
@@ -5337,7 +5340,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="94" customHeight="1" ht="26.75">
       <c r="A94" s="3" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="B94" s="4">
         <v>3</v>
@@ -5346,25 +5349,25 @@
         <v>30</v>
       </c>
       <c r="D94" s="16" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="E94" s="7" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="F94" s="7" t="s">
         <v>54</v>
       </c>
       <c r="G94" s="7" t="s">
+        <v>409</v>
+      </c>
+      <c r="H94" s="7" t="s">
         <v>410</v>
       </c>
-      <c r="H94" s="7" t="s">
-        <v>411</v>
-      </c>
       <c r="I94" s="17" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="J94" s="8" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="K94" s="14" t="s">
         <v>33</v>
@@ -5375,7 +5378,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="95" customHeight="1" ht="26.75">
       <c r="A95" s="3" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
       <c r="B95" s="4">
         <v>3</v>
@@ -5384,25 +5387,25 @@
         <v>30</v>
       </c>
       <c r="D95" s="16" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="E95" s="7" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="F95" s="7" t="s">
         <v>54</v>
       </c>
       <c r="G95" s="7" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
       <c r="H95" s="7" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="I95" s="17" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="J95" s="8" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="K95" s="8" t="s">
         <v>20</v>
@@ -5413,7 +5416,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="96" customHeight="1" ht="26.75">
       <c r="A96" s="3" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="B96" s="4">
         <v>3</v>
@@ -5422,28 +5425,28 @@
         <v>30</v>
       </c>
       <c r="D96" s="16" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="E96" s="7" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="F96" s="7" t="s">
         <v>54</v>
       </c>
       <c r="G96" s="7" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="H96" s="7" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
       <c r="I96" s="17" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="J96" s="8" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="K96" s="17" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="L96" s="13" t="s">
         <v>28</v>
@@ -5451,7 +5454,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="97" customHeight="1" ht="26.75">
       <c r="A97" s="3" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="B97" s="4">
         <v>3</v>
@@ -5463,25 +5466,25 @@
         <v>43</v>
       </c>
       <c r="E97" s="7" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
       <c r="F97" s="7" t="s">
         <v>54</v>
       </c>
       <c r="G97" s="7" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="H97" s="7" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="I97" s="17" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="J97" s="8" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="K97" s="17" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="L97" s="18" t="s">
         <v>47</v>
@@ -5489,7 +5492,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="98" customHeight="1" ht="26.75">
       <c r="A98" s="3" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="B98" s="4">
         <v>3</v>
@@ -5501,25 +5504,25 @@
         <v>43</v>
       </c>
       <c r="E98" s="7" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
       <c r="F98" s="7" t="s">
         <v>54</v>
       </c>
       <c r="G98" s="7" t="s">
+        <v>422</v>
+      </c>
+      <c r="H98" s="7" t="s">
         <v>423</v>
       </c>
-      <c r="H98" s="7" t="s">
-        <v>424</v>
-      </c>
       <c r="I98" s="17" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="J98" s="8" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="K98" s="12" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="L98" s="18" t="s">
         <v>47</v>
@@ -5527,7 +5530,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="99" customHeight="1" ht="26.75">
       <c r="A99" s="3" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="B99" s="4">
         <v>3</v>
@@ -5539,22 +5542,22 @@
         <v>43</v>
       </c>
       <c r="E99" s="7" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="F99" s="7" t="s">
         <v>54</v>
       </c>
       <c r="G99" s="7" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="H99" s="7" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
       <c r="I99" s="17" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="J99" s="8" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="K99" s="14" t="s">
         <v>33</v>
@@ -5565,7 +5568,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="100" customHeight="1" ht="26.75">
       <c r="A100" s="3" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
       <c r="B100" s="4">
         <v>3</v>
@@ -5577,7 +5580,7 @@
         <v>43</v>
       </c>
       <c r="E100" s="7" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="F100" s="7" t="s">
         <v>54</v>
@@ -5586,16 +5589,16 @@
         <v>77</v>
       </c>
       <c r="H100" s="7" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
       <c r="I100" s="17" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="J100" s="8" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="K100" s="23" t="s">
-        <v>89</v>
+        <v>79</v>
       </c>
       <c r="L100" s="18" t="s">
         <v>47</v>

</xml_diff>

<commit_message>
update known issues script and md file
</commit_message>
<xml_diff>
--- a/tools/data/latest.xlsx
+++ b/tools/data/latest.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10911"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{393F7791-64A9-674E-89B6-EB107CC2AF91}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4548FC3E-621C-6947-9470-2D39A7F95AF7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="14900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1044" uniqueCount="432">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1044" uniqueCount="431">
   <si>
     <t>Name</t>
   </si>
@@ -285,9 +285,6 @@
   </si>
   <si>
     <t>Ongoing/DR independent</t>
-  </si>
-  <si>
-    <t>Demographics</t>
   </si>
   <si>
     <t>[DD+DATA ERROR] Nail type field added for 2.0 all "Unknown"</t>
@@ -1344,7 +1341,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="22">
+  <fills count="21">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1433,11 +1430,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFDF2F4A"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="FFFFCB00"/>
       </patternFill>
     </fill>
@@ -1464,7 +1456,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1527,9 +1519,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="20" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="21" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -2453,8 +2442,8 @@
       <c r="J15" s="13" t="s">
         <v>89</v>
       </c>
-      <c r="K15" s="19" t="s">
-        <v>90</v>
+      <c r="K15" s="18" t="s">
+        <v>79</v>
       </c>
       <c r="L15" s="15" t="s">
         <v>47</v>
@@ -2462,7 +2451,7 @@
     </row>
     <row r="16" spans="1:12" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="2" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B16" s="3">
         <v>3</v>
@@ -2474,16 +2463,16 @@
         <v>23</v>
       </c>
       <c r="E16" s="3" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="F16" s="3" t="s">
         <v>15</v>
       </c>
       <c r="G16" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="H16" s="3" t="s">
         <v>93</v>
-      </c>
-      <c r="H16" s="3" t="s">
-        <v>94</v>
       </c>
       <c r="I16" s="5" t="s">
         <v>18</v>
@@ -2491,8 +2480,8 @@
       <c r="J16" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="K16" s="20" t="s">
-        <v>95</v>
+      <c r="K16" s="19" t="s">
+        <v>94</v>
       </c>
       <c r="L16" s="15" t="s">
         <v>47</v>
@@ -2500,7 +2489,7 @@
     </row>
     <row r="17" spans="1:12" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="2" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B17" s="3">
         <v>3</v>
@@ -2512,25 +2501,25 @@
         <v>35</v>
       </c>
       <c r="E17" s="3" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="F17" s="3" t="s">
         <v>15</v>
       </c>
       <c r="G17" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="H17" s="3" t="s">
         <v>98</v>
       </c>
-      <c r="H17" s="3" t="s">
+      <c r="I17" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="J17" s="11" t="s">
         <v>99</v>
       </c>
-      <c r="I17" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="J17" s="11" t="s">
+      <c r="K17" s="9" t="s">
         <v>100</v>
-      </c>
-      <c r="K17" s="9" t="s">
-        <v>101</v>
       </c>
       <c r="L17" s="10" t="s">
         <v>28</v>
@@ -2538,7 +2527,7 @@
     </row>
     <row r="18" spans="1:12" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="2" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B18" s="3">
         <v>3</v>
@@ -2550,16 +2539,16 @@
         <v>43</v>
       </c>
       <c r="E18" s="3" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="F18" s="3" t="s">
         <v>54</v>
       </c>
       <c r="G18" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="H18" s="3" t="s">
         <v>104</v>
-      </c>
-      <c r="H18" s="3" t="s">
-        <v>105</v>
       </c>
       <c r="I18" s="5" t="s">
         <v>18</v>
@@ -2567,8 +2556,8 @@
       <c r="J18" s="16" t="s">
         <v>57</v>
       </c>
-      <c r="K18" s="20" t="s">
-        <v>95</v>
+      <c r="K18" s="19" t="s">
+        <v>94</v>
       </c>
       <c r="L18" s="10" t="s">
         <v>28</v>
@@ -2576,7 +2565,7 @@
     </row>
     <row r="19" spans="1:12" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="2" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B19" s="3">
         <v>3</v>
@@ -2588,7 +2577,7 @@
         <v>13</v>
       </c>
       <c r="E19" s="3" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="F19" s="3" t="s">
         <v>15</v>
@@ -2597,7 +2586,7 @@
         <v>31</v>
       </c>
       <c r="H19" s="3" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="I19" s="5" t="s">
         <v>18</v>
@@ -2614,7 +2603,7 @@
     </row>
     <row r="20" spans="1:12" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="2" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B20" s="3">
         <v>3</v>
@@ -2626,7 +2615,7 @@
         <v>13</v>
       </c>
       <c r="E20" s="3" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="F20" s="3" t="s">
         <v>15</v>
@@ -2635,7 +2624,7 @@
         <v>25</v>
       </c>
       <c r="H20" s="3" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="I20" s="5" t="s">
         <v>18</v>
@@ -2652,7 +2641,7 @@
     </row>
     <row r="21" spans="1:12" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="2" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B21" s="3">
         <v>3</v>
@@ -2664,7 +2653,7 @@
         <v>13</v>
       </c>
       <c r="E21" s="3" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="F21" s="3" t="s">
         <v>15</v>
@@ -2673,7 +2662,7 @@
         <v>25</v>
       </c>
       <c r="H21" s="3" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="I21" s="5" t="s">
         <v>18</v>
@@ -2690,7 +2679,7 @@
     </row>
     <row r="22" spans="1:12" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B22" s="3">
         <v>3</v>
@@ -2702,16 +2691,16 @@
         <v>13</v>
       </c>
       <c r="E22" s="3" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="F22" s="3" t="s">
         <v>15</v>
       </c>
       <c r="G22" s="3" t="s">
+        <v>116</v>
+      </c>
+      <c r="H22" s="3" t="s">
         <v>117</v>
-      </c>
-      <c r="H22" s="3" t="s">
-        <v>118</v>
       </c>
       <c r="I22" s="5" t="s">
         <v>18</v>
@@ -2720,7 +2709,7 @@
         <v>19</v>
       </c>
       <c r="K22" s="14" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="L22" s="10" t="s">
         <v>28</v>
@@ -2728,7 +2717,7 @@
     </row>
     <row r="23" spans="1:12" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="2" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="B23" s="3">
         <v>3</v>
@@ -2740,16 +2729,16 @@
         <v>23</v>
       </c>
       <c r="E23" s="3" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F23" s="3" t="s">
         <v>15</v>
       </c>
       <c r="G23" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="H23" s="3" t="s">
         <v>122</v>
-      </c>
-      <c r="H23" s="3" t="s">
-        <v>123</v>
       </c>
       <c r="I23" s="5" t="s">
         <v>18</v>
@@ -2760,13 +2749,13 @@
       <c r="K23" s="11" t="s">
         <v>33</v>
       </c>
-      <c r="L23" s="21" t="s">
-        <v>124</v>
+      <c r="L23" s="20" t="s">
+        <v>123</v>
       </c>
     </row>
     <row r="24" spans="1:12" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="2" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B24" s="3">
         <v>3</v>
@@ -2778,16 +2767,16 @@
         <v>13</v>
       </c>
       <c r="E24" s="3" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="F24" s="3" t="s">
         <v>15</v>
       </c>
       <c r="G24" s="3" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="H24" s="3" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="I24" s="5" t="s">
         <v>18</v>
@@ -2796,7 +2785,7 @@
         <v>19</v>
       </c>
       <c r="K24" s="14" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="L24" s="15" t="s">
         <v>47</v>
@@ -2804,7 +2793,7 @@
     </row>
     <row r="25" spans="1:12" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="2" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="B25" s="3">
         <v>3</v>
@@ -2816,16 +2805,16 @@
         <v>13</v>
       </c>
       <c r="E25" s="3" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="F25" s="3" t="s">
         <v>54</v>
       </c>
       <c r="G25" s="3" t="s">
+        <v>129</v>
+      </c>
+      <c r="H25" s="3" t="s">
         <v>130</v>
-      </c>
-      <c r="H25" s="3" t="s">
-        <v>131</v>
       </c>
       <c r="I25" s="5" t="s">
         <v>18</v>
@@ -2834,7 +2823,7 @@
         <v>19</v>
       </c>
       <c r="K25" s="4" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="L25" s="10" t="s">
         <v>28</v>
@@ -2842,7 +2831,7 @@
     </row>
     <row r="26" spans="1:12" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="2" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="B26" s="3">
         <v>3</v>
@@ -2854,16 +2843,16 @@
         <v>13</v>
       </c>
       <c r="E26" s="3" t="s">
+        <v>133</v>
+      </c>
+      <c r="F26" s="3" t="s">
         <v>134</v>
       </c>
-      <c r="F26" s="3" t="s">
+      <c r="G26" s="3" t="s">
         <v>135</v>
       </c>
-      <c r="G26" s="3" t="s">
+      <c r="H26" s="3" t="s">
         <v>136</v>
-      </c>
-      <c r="H26" s="3" t="s">
-        <v>137</v>
       </c>
       <c r="I26" s="5" t="s">
         <v>18</v>
@@ -2880,7 +2869,7 @@
     </row>
     <row r="27" spans="1:12" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="2" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="B27" s="3">
         <v>3</v>
@@ -2892,25 +2881,25 @@
         <v>43</v>
       </c>
       <c r="E27" s="3" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="F27" s="3" t="s">
         <v>54</v>
       </c>
       <c r="G27" s="3" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="H27" s="3" t="s">
+        <v>139</v>
+      </c>
+      <c r="I27" s="22" t="s">
+        <v>430</v>
+      </c>
+      <c r="J27" s="5" t="s">
         <v>140</v>
       </c>
-      <c r="I27" s="23" t="s">
-        <v>431</v>
-      </c>
-      <c r="J27" s="5" t="s">
-        <v>141</v>
-      </c>
       <c r="K27" s="14" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="L27" s="15" t="s">
         <v>47</v>
@@ -2918,7 +2907,7 @@
     </row>
     <row r="28" spans="1:12" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="2" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B28" s="3">
         <v>3</v>
@@ -2930,16 +2919,16 @@
         <v>35</v>
       </c>
       <c r="E28" s="3" t="s">
+        <v>142</v>
+      </c>
+      <c r="F28" s="3" t="s">
         <v>143</v>
       </c>
-      <c r="F28" s="3" t="s">
+      <c r="G28" s="3" t="s">
         <v>144</v>
       </c>
-      <c r="G28" s="3" t="s">
+      <c r="H28" s="3" t="s">
         <v>145</v>
-      </c>
-      <c r="H28" s="3" t="s">
-        <v>146</v>
       </c>
       <c r="I28" s="5" t="s">
         <v>18</v>
@@ -2948,7 +2937,7 @@
         <v>40</v>
       </c>
       <c r="K28" s="14" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="L28" s="10" t="s">
         <v>28</v>
@@ -2956,7 +2945,7 @@
     </row>
     <row r="29" spans="1:12" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="2" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="B29" s="3">
         <v>3</v>
@@ -2968,16 +2957,16 @@
         <v>43</v>
       </c>
       <c r="E29" s="3" t="s">
+        <v>147</v>
+      </c>
+      <c r="F29" s="3" t="s">
         <v>148</v>
       </c>
-      <c r="F29" s="3" t="s">
+      <c r="G29" s="3" t="s">
         <v>149</v>
       </c>
-      <c r="G29" s="3" t="s">
+      <c r="H29" s="3" t="s">
         <v>150</v>
-      </c>
-      <c r="H29" s="3" t="s">
-        <v>151</v>
       </c>
       <c r="I29" s="5" t="s">
         <v>18</v>
@@ -2986,7 +2975,7 @@
         <v>19</v>
       </c>
       <c r="K29" s="14" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="L29" s="10" t="s">
         <v>28</v>
@@ -2994,7 +2983,7 @@
     </row>
     <row r="30" spans="1:12" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="2" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="B30" s="3">
         <v>3</v>
@@ -3006,16 +2995,16 @@
         <v>13</v>
       </c>
       <c r="E30" s="3" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="F30" s="3" t="s">
         <v>15</v>
       </c>
       <c r="G30" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="H30" s="3" t="s">
         <v>154</v>
-      </c>
-      <c r="H30" s="3" t="s">
-        <v>155</v>
       </c>
       <c r="I30" s="5" t="s">
         <v>18</v>
@@ -3032,7 +3021,7 @@
     </row>
     <row r="31" spans="1:12" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="2" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="B31" s="3">
         <v>3</v>
@@ -3044,25 +3033,25 @@
         <v>43</v>
       </c>
       <c r="E31" s="3" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="F31" s="3" t="s">
         <v>54</v>
       </c>
       <c r="G31" s="3" t="s">
+        <v>157</v>
+      </c>
+      <c r="H31" s="3" t="s">
         <v>158</v>
       </c>
-      <c r="H31" s="3" t="s">
+      <c r="I31" s="22" t="s">
+        <v>430</v>
+      </c>
+      <c r="J31" s="5" t="s">
+        <v>140</v>
+      </c>
+      <c r="K31" s="16" t="s">
         <v>159</v>
-      </c>
-      <c r="I31" s="23" t="s">
-        <v>431</v>
-      </c>
-      <c r="J31" s="5" t="s">
-        <v>141</v>
-      </c>
-      <c r="K31" s="16" t="s">
-        <v>160</v>
       </c>
       <c r="L31" s="15" t="s">
         <v>47</v>
@@ -3070,7 +3059,7 @@
     </row>
     <row r="32" spans="1:12" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="2" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B32" s="3">
         <v>3</v>
@@ -3082,16 +3071,16 @@
         <v>23</v>
       </c>
       <c r="E32" s="3" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="F32" s="3" t="s">
         <v>15</v>
       </c>
       <c r="G32" s="3" t="s">
+        <v>162</v>
+      </c>
+      <c r="H32" s="3" t="s">
         <v>163</v>
-      </c>
-      <c r="H32" s="3" t="s">
-        <v>164</v>
       </c>
       <c r="I32" s="5" t="s">
         <v>18</v>
@@ -3100,7 +3089,7 @@
         <v>27</v>
       </c>
       <c r="K32" s="16" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="L32" s="15" t="s">
         <v>47</v>
@@ -3108,7 +3097,7 @@
     </row>
     <row r="33" spans="1:12" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="2" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="B33" s="3">
         <v>3</v>
@@ -3120,22 +3109,22 @@
         <v>43</v>
       </c>
       <c r="E33" s="3" t="s">
+        <v>165</v>
+      </c>
+      <c r="F33" s="3" t="s">
         <v>166</v>
       </c>
-      <c r="F33" s="3" t="s">
+      <c r="G33" s="3" t="s">
         <v>167</v>
       </c>
-      <c r="G33" s="3" t="s">
+      <c r="H33" s="3" t="s">
         <v>168</v>
       </c>
-      <c r="H33" s="3" t="s">
+      <c r="I33" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="J33" s="18" t="s">
         <v>169</v>
-      </c>
-      <c r="I33" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="J33" s="18" t="s">
-        <v>170</v>
       </c>
       <c r="K33" s="13" t="s">
         <v>41</v>
@@ -3146,7 +3135,7 @@
     </row>
     <row r="34" spans="1:12" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" s="2" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="B34" s="3">
         <v>3</v>
@@ -3158,16 +3147,16 @@
         <v>23</v>
       </c>
       <c r="E34" s="3" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="F34" s="3" t="s">
         <v>37</v>
       </c>
       <c r="G34" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="H34" s="3" t="s">
         <v>173</v>
-      </c>
-      <c r="H34" s="3" t="s">
-        <v>174</v>
       </c>
       <c r="I34" s="5" t="s">
         <v>18</v>
@@ -3184,7 +3173,7 @@
     </row>
     <row r="35" spans="1:12" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="2" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B35" s="3">
         <v>3</v>
@@ -3196,22 +3185,22 @@
         <v>43</v>
       </c>
       <c r="E35" s="3" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="F35" s="3" t="s">
         <v>54</v>
       </c>
       <c r="G35" s="3" t="s">
+        <v>176</v>
+      </c>
+      <c r="H35" s="3" t="s">
         <v>177</v>
       </c>
-      <c r="H35" s="3" t="s">
-        <v>178</v>
-      </c>
       <c r="I35" s="5" t="s">
         <v>18</v>
       </c>
       <c r="J35" s="18" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="K35" s="17" t="s">
         <v>62</v>
@@ -3222,7 +3211,7 @@
     </row>
     <row r="36" spans="1:12" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="2" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="B36" s="3">
         <v>3</v>
@@ -3234,16 +3223,16 @@
         <v>13</v>
       </c>
       <c r="E36" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="F36" s="3" t="s">
         <v>180</v>
-      </c>
-      <c r="F36" s="3" t="s">
-        <v>181</v>
       </c>
       <c r="G36" s="3" t="s">
         <v>45</v>
       </c>
       <c r="H36" s="3" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="I36" s="5" t="s">
         <v>18</v>
@@ -3260,7 +3249,7 @@
     </row>
     <row r="37" spans="1:12" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A37" s="2" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="B37" s="3">
         <v>3</v>
@@ -3272,16 +3261,16 @@
         <v>13</v>
       </c>
       <c r="E37" s="3" t="s">
+        <v>183</v>
+      </c>
+      <c r="F37" s="3" t="s">
+        <v>180</v>
+      </c>
+      <c r="G37" s="3" t="s">
         <v>184</v>
       </c>
-      <c r="F37" s="3" t="s">
+      <c r="H37" s="3" t="s">
         <v>181</v>
-      </c>
-      <c r="G37" s="3" t="s">
-        <v>185</v>
-      </c>
-      <c r="H37" s="3" t="s">
-        <v>182</v>
       </c>
       <c r="I37" s="5" t="s">
         <v>18</v>
@@ -3298,7 +3287,7 @@
     </row>
     <row r="38" spans="1:12" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A38" s="2" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="B38" s="3">
         <v>3</v>
@@ -3310,16 +3299,16 @@
         <v>13</v>
       </c>
       <c r="E38" s="3" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="F38" s="3" t="s">
         <v>15</v>
       </c>
       <c r="G38" s="3" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="H38" s="3" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="I38" s="5" t="s">
         <v>18</v>
@@ -3328,7 +3317,7 @@
         <v>19</v>
       </c>
       <c r="K38" s="16" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="L38" s="7" t="s">
         <v>21</v>
@@ -3336,7 +3325,7 @@
     </row>
     <row r="39" spans="1:12" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A39" s="2" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="B39" s="3">
         <v>3</v>
@@ -3348,16 +3337,16 @@
         <v>13</v>
       </c>
       <c r="E39" s="3" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="F39" s="3" t="s">
         <v>15</v>
       </c>
       <c r="G39" s="3" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="H39" s="3" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="I39" s="5" t="s">
         <v>18</v>
@@ -3366,7 +3355,7 @@
         <v>19</v>
       </c>
       <c r="K39" s="16" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="L39" s="10" t="s">
         <v>28</v>
@@ -3374,7 +3363,7 @@
     </row>
     <row r="40" spans="1:12" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A40" s="2" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="B40" s="3">
         <v>3</v>
@@ -3386,16 +3375,16 @@
         <v>13</v>
       </c>
       <c r="E40" s="3" t="s">
+        <v>192</v>
+      </c>
+      <c r="F40" s="3" t="s">
+        <v>180</v>
+      </c>
+      <c r="G40" s="3" t="s">
         <v>193</v>
       </c>
-      <c r="F40" s="3" t="s">
+      <c r="H40" s="3" t="s">
         <v>181</v>
-      </c>
-      <c r="G40" s="3" t="s">
-        <v>194</v>
-      </c>
-      <c r="H40" s="3" t="s">
-        <v>182</v>
       </c>
       <c r="I40" s="5" t="s">
         <v>18</v>
@@ -3404,7 +3393,7 @@
         <v>19</v>
       </c>
       <c r="K40" s="14" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="L40" s="10" t="s">
         <v>28</v>
@@ -3412,7 +3401,7 @@
     </row>
     <row r="41" spans="1:12" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A41" s="2" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B41" s="3">
         <v>3</v>
@@ -3424,16 +3413,16 @@
         <v>13</v>
       </c>
       <c r="E41" s="3" t="s">
+        <v>195</v>
+      </c>
+      <c r="F41" s="3" t="s">
+        <v>180</v>
+      </c>
+      <c r="G41" s="3" t="s">
         <v>196</v>
       </c>
-      <c r="F41" s="3" t="s">
+      <c r="H41" s="3" t="s">
         <v>181</v>
-      </c>
-      <c r="G41" s="3" t="s">
-        <v>197</v>
-      </c>
-      <c r="H41" s="3" t="s">
-        <v>182</v>
       </c>
       <c r="I41" s="5" t="s">
         <v>18</v>
@@ -3450,7 +3439,7 @@
     </row>
     <row r="42" spans="1:12" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A42" s="2" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B42" s="3">
         <v>3</v>
@@ -3462,16 +3451,16 @@
         <v>13</v>
       </c>
       <c r="E42" s="3" t="s">
+        <v>198</v>
+      </c>
+      <c r="F42" s="3" t="s">
+        <v>180</v>
+      </c>
+      <c r="G42" s="3" t="s">
         <v>199</v>
       </c>
-      <c r="F42" s="3" t="s">
+      <c r="H42" s="3" t="s">
         <v>181</v>
-      </c>
-      <c r="G42" s="3" t="s">
-        <v>200</v>
-      </c>
-      <c r="H42" s="3" t="s">
-        <v>182</v>
       </c>
       <c r="I42" s="5" t="s">
         <v>18</v>
@@ -3488,7 +3477,7 @@
     </row>
     <row r="43" spans="1:12" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A43" s="2" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="B43" s="3">
         <v>3</v>
@@ -3500,16 +3489,16 @@
         <v>13</v>
       </c>
       <c r="E43" s="3" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="F43" s="3" t="s">
         <v>15</v>
       </c>
       <c r="G43" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="H43" s="3" t="s">
         <v>203</v>
-      </c>
-      <c r="H43" s="3" t="s">
-        <v>204</v>
       </c>
       <c r="I43" s="5" t="s">
         <v>18</v>
@@ -3526,7 +3515,7 @@
     </row>
     <row r="44" spans="1:12" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A44" s="2" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="B44" s="3">
         <v>3</v>
@@ -3538,16 +3527,16 @@
         <v>43</v>
       </c>
       <c r="E44" s="3" t="s">
+        <v>205</v>
+      </c>
+      <c r="F44" s="3" t="s">
         <v>206</v>
       </c>
-      <c r="F44" s="3" t="s">
+      <c r="G44" s="3" t="s">
         <v>207</v>
       </c>
-      <c r="G44" s="3" t="s">
+      <c r="H44" s="3" t="s">
         <v>208</v>
-      </c>
-      <c r="H44" s="3" t="s">
-        <v>209</v>
       </c>
       <c r="I44" s="5" t="s">
         <v>18</v>
@@ -3564,7 +3553,7 @@
     </row>
     <row r="45" spans="1:12" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A45" s="2" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="B45" s="3">
         <v>3</v>
@@ -3576,16 +3565,16 @@
         <v>23</v>
       </c>
       <c r="E45" s="3" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="F45" s="3" t="s">
         <v>15</v>
       </c>
       <c r="G45" s="3" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="H45" s="3" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="I45" s="5" t="s">
         <v>18</v>
@@ -3594,7 +3583,7 @@
         <v>27</v>
       </c>
       <c r="K45" s="14" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="L45" s="7" t="s">
         <v>21</v>
@@ -3602,7 +3591,7 @@
     </row>
     <row r="46" spans="1:12" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A46" s="2" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="B46" s="3">
         <v>3</v>
@@ -3614,16 +3603,16 @@
         <v>13</v>
       </c>
       <c r="E46" s="3" t="s">
+        <v>213</v>
+      </c>
+      <c r="F46" s="3" t="s">
         <v>214</v>
       </c>
-      <c r="F46" s="3" t="s">
+      <c r="G46" s="3" t="s">
         <v>215</v>
       </c>
-      <c r="G46" s="3" t="s">
+      <c r="H46" s="3" t="s">
         <v>216</v>
-      </c>
-      <c r="H46" s="3" t="s">
-        <v>217</v>
       </c>
       <c r="I46" s="5" t="s">
         <v>18</v>
@@ -3640,7 +3629,7 @@
     </row>
     <row r="47" spans="1:12" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A47" s="2" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="B47" s="3">
         <v>3</v>
@@ -3652,16 +3641,16 @@
         <v>13</v>
       </c>
       <c r="E47" s="3" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="F47" s="3" t="s">
         <v>15</v>
       </c>
       <c r="G47" s="3" t="s">
+        <v>219</v>
+      </c>
+      <c r="H47" s="3" t="s">
         <v>220</v>
-      </c>
-      <c r="H47" s="3" t="s">
-        <v>221</v>
       </c>
       <c r="I47" s="5" t="s">
         <v>18</v>
@@ -3670,7 +3659,7 @@
         <v>19</v>
       </c>
       <c r="K47" s="14" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="L47" s="7" t="s">
         <v>21</v>
@@ -3678,7 +3667,7 @@
     </row>
     <row r="48" spans="1:12" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A48" s="2" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="B48" s="3">
         <v>3</v>
@@ -3690,16 +3679,16 @@
         <v>13</v>
       </c>
       <c r="E48" s="3" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="F48" s="3" t="s">
         <v>15</v>
       </c>
       <c r="G48" s="3" t="s">
+        <v>223</v>
+      </c>
+      <c r="H48" s="3" t="s">
         <v>224</v>
-      </c>
-      <c r="H48" s="3" t="s">
-        <v>225</v>
       </c>
       <c r="I48" s="5" t="s">
         <v>18</v>
@@ -3716,7 +3705,7 @@
     </row>
     <row r="49" spans="1:12" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A49" s="2" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="B49" s="3">
         <v>3</v>
@@ -3728,25 +3717,25 @@
         <v>35</v>
       </c>
       <c r="E49" s="3" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="F49" s="3" t="s">
         <v>15</v>
       </c>
       <c r="G49" s="3" t="s">
+        <v>227</v>
+      </c>
+      <c r="H49" s="3" t="s">
         <v>228</v>
       </c>
-      <c r="H49" s="3" t="s">
-        <v>229</v>
-      </c>
       <c r="I49" s="5" t="s">
         <v>18</v>
       </c>
       <c r="J49" s="11" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="K49" s="14" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="L49" s="15" t="s">
         <v>47</v>
@@ -3754,7 +3743,7 @@
     </row>
     <row r="50" spans="1:12" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A50" s="2" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="B50" s="3">
         <v>3</v>
@@ -3766,16 +3755,16 @@
         <v>23</v>
       </c>
       <c r="E50" s="3" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="F50" s="3" t="s">
         <v>15</v>
       </c>
       <c r="G50" s="3" t="s">
+        <v>231</v>
+      </c>
+      <c r="H50" s="3" t="s">
         <v>232</v>
-      </c>
-      <c r="H50" s="3" t="s">
-        <v>233</v>
       </c>
       <c r="I50" s="5" t="s">
         <v>18</v>
@@ -3786,13 +3775,13 @@
       <c r="K50" s="18" t="s">
         <v>79</v>
       </c>
-      <c r="L50" s="21" t="s">
-        <v>124</v>
+      <c r="L50" s="20" t="s">
+        <v>123</v>
       </c>
     </row>
     <row r="51" spans="1:12" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A51" s="2" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="B51" s="3">
         <v>3</v>
@@ -3804,7 +3793,7 @@
         <v>13</v>
       </c>
       <c r="E51" s="3" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="F51" t="s">
         <v>85</v>
@@ -3813,7 +3802,7 @@
         <v>25</v>
       </c>
       <c r="H51" s="3" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="I51" s="5" t="s">
         <v>18</v>
@@ -3830,7 +3819,7 @@
     </row>
     <row r="52" spans="1:12" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A52" s="2" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="B52" s="3">
         <v>3</v>
@@ -3842,22 +3831,22 @@
         <v>35</v>
       </c>
       <c r="E52" s="3" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="F52" s="3" t="s">
         <v>15</v>
       </c>
       <c r="G52" s="3" t="s">
+        <v>238</v>
+      </c>
+      <c r="H52" s="3" t="s">
         <v>239</v>
       </c>
-      <c r="H52" s="3" t="s">
-        <v>240</v>
-      </c>
       <c r="I52" s="5" t="s">
         <v>18</v>
       </c>
       <c r="J52" s="11" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="K52" s="18" t="s">
         <v>79</v>
@@ -3868,7 +3857,7 @@
     </row>
     <row r="53" spans="1:12" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A53" s="2" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="B53" s="3">
         <v>3</v>
@@ -3880,16 +3869,16 @@
         <v>23</v>
       </c>
       <c r="E53" s="3" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="F53" s="3" t="s">
         <v>37</v>
       </c>
       <c r="G53" s="3" t="s">
+        <v>242</v>
+      </c>
+      <c r="H53" s="3" t="s">
         <v>243</v>
-      </c>
-      <c r="H53" s="3" t="s">
-        <v>244</v>
       </c>
       <c r="I53" s="5" t="s">
         <v>18</v>
@@ -3906,7 +3895,7 @@
     </row>
     <row r="54" spans="1:12" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A54" s="2" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="B54" s="3">
         <v>3</v>
@@ -3918,16 +3907,16 @@
         <v>23</v>
       </c>
       <c r="E54" s="3" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="F54" s="3" t="s">
         <v>37</v>
       </c>
       <c r="G54" s="3" t="s">
+        <v>246</v>
+      </c>
+      <c r="H54" s="3" t="s">
         <v>247</v>
-      </c>
-      <c r="H54" s="3" t="s">
-        <v>248</v>
       </c>
       <c r="I54" s="5" t="s">
         <v>18</v>
@@ -3944,7 +3933,7 @@
     </row>
     <row r="55" spans="1:12" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A55" s="2" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="B55" s="3">
         <v>3</v>
@@ -3956,7 +3945,7 @@
         <v>13</v>
       </c>
       <c r="E55" s="3" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="F55" t="s">
         <v>85</v>
@@ -3965,7 +3954,7 @@
         <v>77</v>
       </c>
       <c r="H55" s="3" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="I55" s="5" t="s">
         <v>18</v>
@@ -3982,7 +3971,7 @@
     </row>
     <row r="56" spans="1:12" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A56" s="2" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="B56" s="3">
         <v>3</v>
@@ -3994,7 +3983,7 @@
         <v>35</v>
       </c>
       <c r="E56" s="3" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="F56" s="3" t="s">
         <v>15</v>
@@ -4003,13 +3992,13 @@
         <v>77</v>
       </c>
       <c r="H56" s="3" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="I56" s="5" t="s">
         <v>18</v>
       </c>
       <c r="J56" s="11" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="K56" s="18" t="s">
         <v>79</v>
@@ -4020,7 +4009,7 @@
     </row>
     <row r="57" spans="1:12" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A57" s="2" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="B57" s="3">
         <v>3</v>
@@ -4032,16 +4021,16 @@
         <v>13</v>
       </c>
       <c r="E57" s="3" t="s">
+        <v>255</v>
+      </c>
+      <c r="F57" s="3" t="s">
         <v>256</v>
       </c>
-      <c r="F57" s="3" t="s">
+      <c r="G57" s="3" t="s">
         <v>257</v>
       </c>
-      <c r="G57" s="3" t="s">
+      <c r="H57" s="3" t="s">
         <v>258</v>
-      </c>
-      <c r="H57" s="3" t="s">
-        <v>259</v>
       </c>
       <c r="I57" s="5" t="s">
         <v>18</v>
@@ -4058,7 +4047,7 @@
     </row>
     <row r="58" spans="1:12" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A58" s="2" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="B58" s="3">
         <v>3</v>
@@ -4070,7 +4059,7 @@
         <v>35</v>
       </c>
       <c r="E58" s="3" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="F58" s="3" t="s">
         <v>15</v>
@@ -4079,16 +4068,16 @@
         <v>87</v>
       </c>
       <c r="H58" s="3" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="I58" s="5" t="s">
         <v>18</v>
       </c>
       <c r="J58" s="11" t="s">
+        <v>99</v>
+      </c>
+      <c r="K58" s="9" t="s">
         <v>100</v>
-      </c>
-      <c r="K58" s="9" t="s">
-        <v>101</v>
       </c>
       <c r="L58" s="7" t="s">
         <v>21</v>
@@ -4096,7 +4085,7 @@
     </row>
     <row r="59" spans="1:12" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A59" s="2" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="B59" s="3">
         <v>3</v>
@@ -4108,7 +4097,7 @@
         <v>23</v>
       </c>
       <c r="E59" s="3" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="F59" s="3" t="s">
         <v>15</v>
@@ -4117,7 +4106,7 @@
         <v>87</v>
       </c>
       <c r="H59" s="3" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="I59" s="5" t="s">
         <v>18</v>
@@ -4126,7 +4115,7 @@
         <v>27</v>
       </c>
       <c r="K59" s="9" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="L59" s="7" t="s">
         <v>21</v>
@@ -4134,7 +4123,7 @@
     </row>
     <row r="60" spans="1:12" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A60" s="2" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="B60" s="3">
         <v>3</v>
@@ -4146,22 +4135,22 @@
         <v>13</v>
       </c>
       <c r="E60" s="3" t="s">
+        <v>266</v>
+      </c>
+      <c r="F60" s="3" t="s">
+        <v>256</v>
+      </c>
+      <c r="G60" s="3" t="s">
         <v>267</v>
       </c>
-      <c r="F60" s="3" t="s">
-        <v>257</v>
-      </c>
-      <c r="G60" s="3" t="s">
+      <c r="H60" s="3" t="s">
         <v>268</v>
       </c>
-      <c r="H60" s="3" t="s">
-        <v>269</v>
-      </c>
       <c r="I60" s="5" t="s">
         <v>18</v>
       </c>
       <c r="J60" s="18" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="K60" s="17" t="s">
         <v>62</v>
@@ -4172,7 +4161,7 @@
     </row>
     <row r="61" spans="1:12" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A61" s="2" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="B61" s="3">
         <v>3</v>
@@ -4184,22 +4173,22 @@
         <v>35</v>
       </c>
       <c r="E61" s="3" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="F61" s="3" t="s">
         <v>15</v>
       </c>
       <c r="G61" s="3" t="s">
+        <v>271</v>
+      </c>
+      <c r="H61" s="3" t="s">
         <v>272</v>
       </c>
-      <c r="H61" s="3" t="s">
-        <v>273</v>
-      </c>
       <c r="I61" s="5" t="s">
         <v>18</v>
       </c>
       <c r="J61" s="11" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="K61" s="11" t="s">
         <v>33</v>
@@ -4210,7 +4199,7 @@
     </row>
     <row r="62" spans="1:12" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A62" s="2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="B62" s="3">
         <v>3</v>
@@ -4222,16 +4211,16 @@
         <v>35</v>
       </c>
       <c r="E62" s="3" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="F62" t="s">
         <v>85</v>
       </c>
       <c r="G62" s="3" t="s">
+        <v>275</v>
+      </c>
+      <c r="H62" s="3" t="s">
         <v>276</v>
-      </c>
-      <c r="H62" s="3" t="s">
-        <v>277</v>
       </c>
       <c r="I62" s="5" t="s">
         <v>18</v>
@@ -4239,16 +4228,16 @@
       <c r="J62" s="13" t="s">
         <v>89</v>
       </c>
-      <c r="K62" s="20" t="s">
-        <v>95</v>
-      </c>
-      <c r="L62" s="21" t="s">
-        <v>124</v>
+      <c r="K62" s="19" t="s">
+        <v>94</v>
+      </c>
+      <c r="L62" s="20" t="s">
+        <v>123</v>
       </c>
     </row>
     <row r="63" spans="1:12" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A63" s="2" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="B63" s="3">
         <v>3</v>
@@ -4260,16 +4249,16 @@
         <v>23</v>
       </c>
       <c r="E63" s="3" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="F63" s="3" t="s">
         <v>15</v>
       </c>
       <c r="G63" s="3" t="s">
+        <v>279</v>
+      </c>
+      <c r="H63" s="3" t="s">
         <v>280</v>
-      </c>
-      <c r="H63" s="3" t="s">
-        <v>281</v>
       </c>
       <c r="I63" s="5" t="s">
         <v>18</v>
@@ -4280,13 +4269,13 @@
       <c r="K63" s="18" t="s">
         <v>79</v>
       </c>
-      <c r="L63" s="21" t="s">
-        <v>124</v>
+      <c r="L63" s="20" t="s">
+        <v>123</v>
       </c>
     </row>
     <row r="64" spans="1:12" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A64" s="2" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="B64" s="3">
         <v>3</v>
@@ -4298,16 +4287,16 @@
         <v>23</v>
       </c>
       <c r="E64" s="3" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="F64" s="3" t="s">
         <v>15</v>
       </c>
       <c r="G64" s="3" t="s">
+        <v>283</v>
+      </c>
+      <c r="H64" s="3" t="s">
         <v>284</v>
-      </c>
-      <c r="H64" s="3" t="s">
-        <v>285</v>
       </c>
       <c r="I64" s="5" t="s">
         <v>18</v>
@@ -4316,7 +4305,7 @@
         <v>27</v>
       </c>
       <c r="K64" s="9" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="L64" s="7" t="s">
         <v>21</v>
@@ -4324,7 +4313,7 @@
     </row>
     <row r="65" spans="1:12" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A65" s="2" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="B65" s="3">
         <v>3</v>
@@ -4336,16 +4325,16 @@
         <v>13</v>
       </c>
       <c r="E65" s="3" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="F65" t="s">
         <v>85</v>
       </c>
       <c r="G65" s="3" t="s">
+        <v>287</v>
+      </c>
+      <c r="H65" s="3" t="s">
         <v>288</v>
-      </c>
-      <c r="H65" s="3" t="s">
-        <v>289</v>
       </c>
       <c r="I65" s="5" t="s">
         <v>18</v>
@@ -4354,15 +4343,15 @@
         <v>19</v>
       </c>
       <c r="K65" s="4" t="s">
-        <v>132</v>
-      </c>
-      <c r="L65" s="21" t="s">
-        <v>124</v>
+        <v>131</v>
+      </c>
+      <c r="L65" s="20" t="s">
+        <v>123</v>
       </c>
     </row>
     <row r="66" spans="1:12" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A66" s="2" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="B66" s="3">
         <v>3</v>
@@ -4374,33 +4363,33 @@
         <v>13</v>
       </c>
       <c r="E66" s="3" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="F66" t="s">
         <v>85</v>
       </c>
       <c r="G66" s="3" t="s">
+        <v>291</v>
+      </c>
+      <c r="H66" s="3" t="s">
         <v>292</v>
       </c>
-      <c r="H66" s="3" t="s">
-        <v>293</v>
-      </c>
-      <c r="I66" s="23" t="s">
-        <v>431</v>
+      <c r="I66" s="22" t="s">
+        <v>430</v>
       </c>
       <c r="J66" s="5" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="K66" s="13" t="s">
         <v>41</v>
       </c>
-      <c r="L66" s="21" t="s">
-        <v>124</v>
+      <c r="L66" s="20" t="s">
+        <v>123</v>
       </c>
     </row>
     <row r="67" spans="1:12" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A67" s="2" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="B67" s="3">
         <v>3</v>
@@ -4412,16 +4401,16 @@
         <v>23</v>
       </c>
       <c r="E67" s="3" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="F67" s="3" t="s">
         <v>15</v>
       </c>
       <c r="G67" s="3" t="s">
+        <v>295</v>
+      </c>
+      <c r="H67" s="3" t="s">
         <v>296</v>
-      </c>
-      <c r="H67" s="3" t="s">
-        <v>297</v>
       </c>
       <c r="I67" s="5" t="s">
         <v>18</v>
@@ -4429,8 +4418,8 @@
       <c r="J67" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="K67" s="20" t="s">
-        <v>95</v>
+      <c r="K67" s="19" t="s">
+        <v>94</v>
       </c>
       <c r="L67" s="15" t="s">
         <v>47</v>
@@ -4438,7 +4427,7 @@
     </row>
     <row r="68" spans="1:12" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A68" s="2" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="B68" s="3">
         <v>3</v>
@@ -4450,16 +4439,16 @@
         <v>23</v>
       </c>
       <c r="E68" s="3" t="s">
+        <v>298</v>
+      </c>
+      <c r="F68" s="3" t="s">
         <v>299</v>
       </c>
-      <c r="F68" s="3" t="s">
+      <c r="G68" s="3" t="s">
         <v>300</v>
       </c>
-      <c r="G68" s="3" t="s">
+      <c r="H68" s="3" t="s">
         <v>301</v>
-      </c>
-      <c r="H68" s="3" t="s">
-        <v>302</v>
       </c>
       <c r="I68" s="5" t="s">
         <v>18</v>
@@ -4468,15 +4457,15 @@
         <v>27</v>
       </c>
       <c r="K68" s="14" t="s">
-        <v>119</v>
-      </c>
-      <c r="L68" s="21" t="s">
-        <v>124</v>
+        <v>118</v>
+      </c>
+      <c r="L68" s="20" t="s">
+        <v>123</v>
       </c>
     </row>
     <row r="69" spans="1:12" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A69" s="2" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="B69" t="s">
         <v>85</v>
@@ -4488,16 +4477,16 @@
         <v>35</v>
       </c>
       <c r="E69" s="3" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="F69" s="3" t="s">
         <v>15</v>
       </c>
       <c r="G69" s="3" t="s">
+        <v>304</v>
+      </c>
+      <c r="H69" s="3" t="s">
         <v>305</v>
-      </c>
-      <c r="H69" s="3" t="s">
-        <v>306</v>
       </c>
       <c r="I69" s="5" t="s">
         <v>18</v>
@@ -4514,7 +4503,7 @@
     </row>
     <row r="70" spans="1:12" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A70" s="2" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="B70" t="s">
         <v>85</v>
@@ -4526,22 +4515,22 @@
         <v>35</v>
       </c>
       <c r="E70" s="3" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="F70" s="3" t="s">
         <v>54</v>
       </c>
       <c r="G70" s="3" t="s">
+        <v>308</v>
+      </c>
+      <c r="H70" s="3" t="s">
         <v>309</v>
       </c>
-      <c r="H70" s="3" t="s">
+      <c r="I70" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="J70" s="12" t="s">
         <v>310</v>
-      </c>
-      <c r="I70" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="J70" s="12" t="s">
-        <v>311</v>
       </c>
       <c r="K70" s="13" t="s">
         <v>41</v>
@@ -4552,7 +4541,7 @@
     </row>
     <row r="71" spans="1:12" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A71" s="2" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="B71" t="s">
         <v>85</v>
@@ -4564,25 +4553,25 @@
         <v>35</v>
       </c>
       <c r="E71" s="3" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="F71" s="3" t="s">
         <v>15</v>
       </c>
       <c r="G71" s="3" t="s">
+        <v>313</v>
+      </c>
+      <c r="H71" s="3" t="s">
         <v>314</v>
       </c>
-      <c r="H71" s="3" t="s">
-        <v>315</v>
-      </c>
       <c r="I71" s="5" t="s">
         <v>18</v>
       </c>
       <c r="J71" s="12" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="K71" s="16" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="L71" s="15" t="s">
         <v>47</v>
@@ -4590,7 +4579,7 @@
     </row>
     <row r="72" spans="1:12" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A72" s="2" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="B72" t="s">
         <v>85</v>
@@ -4602,22 +4591,22 @@
         <v>35</v>
       </c>
       <c r="E72" s="3" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="F72" s="3" t="s">
         <v>15</v>
       </c>
       <c r="G72" s="3" t="s">
+        <v>317</v>
+      </c>
+      <c r="H72" s="3" t="s">
         <v>318</v>
       </c>
-      <c r="H72" s="3" t="s">
+      <c r="I72" s="13" t="s">
         <v>319</v>
       </c>
-      <c r="I72" s="13" t="s">
-        <v>320</v>
-      </c>
       <c r="J72" s="12" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="K72" s="13" t="s">
         <v>41</v>
@@ -4628,7 +4617,7 @@
     </row>
     <row r="73" spans="1:12" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A73" s="2" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="B73" t="s">
         <v>85</v>
@@ -4640,22 +4629,22 @@
         <v>35</v>
       </c>
       <c r="E73" s="3" t="s">
+        <v>321</v>
+      </c>
+      <c r="F73" s="3" t="s">
+        <v>214</v>
+      </c>
+      <c r="G73" s="3" t="s">
         <v>322</v>
       </c>
-      <c r="F73" s="3" t="s">
-        <v>215</v>
-      </c>
-      <c r="G73" s="3" t="s">
+      <c r="H73" s="3" t="s">
         <v>323</v>
       </c>
-      <c r="H73" s="3" t="s">
-        <v>324</v>
-      </c>
       <c r="I73" s="5" t="s">
         <v>18</v>
       </c>
       <c r="J73" s="12" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="K73" s="17" t="s">
         <v>62</v>
@@ -4666,7 +4655,7 @@
     </row>
     <row r="74" spans="1:12" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A74" s="2" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="B74" t="s">
         <v>85</v>
@@ -4678,16 +4667,16 @@
         <v>35</v>
       </c>
       <c r="E74" s="3" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="F74" s="3" t="s">
         <v>15</v>
       </c>
       <c r="G74" s="3" t="s">
+        <v>326</v>
+      </c>
+      <c r="H74" s="3" t="s">
         <v>327</v>
-      </c>
-      <c r="H74" s="3" t="s">
-        <v>328</v>
       </c>
       <c r="I74" s="5" t="s">
         <v>18</v>
@@ -4704,7 +4693,7 @@
     </row>
     <row r="75" spans="1:12" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A75" s="2" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="B75" t="s">
         <v>85</v>
@@ -4716,16 +4705,16 @@
         <v>35</v>
       </c>
       <c r="E75" s="3" t="s">
+        <v>329</v>
+      </c>
+      <c r="F75" s="3" t="s">
         <v>330</v>
       </c>
-      <c r="F75" s="3" t="s">
+      <c r="G75" s="3" t="s">
         <v>331</v>
       </c>
-      <c r="G75" s="3" t="s">
+      <c r="H75" s="3" t="s">
         <v>332</v>
-      </c>
-      <c r="H75" s="3" t="s">
-        <v>333</v>
       </c>
       <c r="I75" s="5" t="s">
         <v>18</v>
@@ -4734,7 +4723,7 @@
         <v>89</v>
       </c>
       <c r="K75" s="9" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="L75" s="15" t="s">
         <v>47</v>
@@ -4742,7 +4731,7 @@
     </row>
     <row r="76" spans="1:12" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A76" s="2" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="B76" t="s">
         <v>85</v>
@@ -4754,16 +4743,16 @@
         <v>35</v>
       </c>
       <c r="E76" s="3" t="s">
+        <v>334</v>
+      </c>
+      <c r="F76" s="3" t="s">
+        <v>330</v>
+      </c>
+      <c r="G76" s="3" t="s">
+        <v>331</v>
+      </c>
+      <c r="H76" s="3" t="s">
         <v>335</v>
-      </c>
-      <c r="F76" s="3" t="s">
-        <v>331</v>
-      </c>
-      <c r="G76" s="3" t="s">
-        <v>332</v>
-      </c>
-      <c r="H76" s="3" t="s">
-        <v>336</v>
       </c>
       <c r="I76" s="5" t="s">
         <v>18</v>
@@ -4772,7 +4761,7 @@
         <v>89</v>
       </c>
       <c r="K76" s="9" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="L76" s="15" t="s">
         <v>47</v>
@@ -4780,7 +4769,7 @@
     </row>
     <row r="77" spans="1:12" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A77" s="2" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="B77" t="s">
         <v>85</v>
@@ -4792,22 +4781,22 @@
         <v>35</v>
       </c>
       <c r="E77" s="3" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="F77" s="3" t="s">
         <v>15</v>
       </c>
       <c r="G77" s="3" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="H77" s="3" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="I77" s="5" t="s">
         <v>18</v>
       </c>
       <c r="J77" s="11" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="K77" s="13" t="s">
         <v>41</v>
@@ -4818,7 +4807,7 @@
     </row>
     <row r="78" spans="1:12" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A78" s="2" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="B78" t="s">
         <v>85</v>
@@ -4830,25 +4819,25 @@
         <v>35</v>
       </c>
       <c r="E78" s="3" t="s">
+        <v>340</v>
+      </c>
+      <c r="F78" s="3" t="s">
         <v>341</v>
-      </c>
-      <c r="F78" s="3" t="s">
-        <v>342</v>
       </c>
       <c r="G78" s="3" t="s">
         <v>87</v>
       </c>
       <c r="H78" s="3" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="I78" s="13" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="J78" s="12" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="K78" s="9" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="L78" s="15" t="s">
         <v>47</v>
@@ -4856,7 +4845,7 @@
     </row>
     <row r="79" spans="1:12" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A79" s="2" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="B79" t="s">
         <v>85</v>
@@ -4868,22 +4857,22 @@
         <v>35</v>
       </c>
       <c r="E79" s="3" t="s">
+        <v>344</v>
+      </c>
+      <c r="F79" s="3" t="s">
         <v>345</v>
       </c>
-      <c r="F79" s="3" t="s">
+      <c r="G79" s="3" t="s">
         <v>346</v>
       </c>
-      <c r="G79" s="3" t="s">
+      <c r="H79" s="3" t="s">
         <v>347</v>
       </c>
-      <c r="H79" s="3" t="s">
-        <v>348</v>
-      </c>
       <c r="I79" s="5" t="s">
         <v>18</v>
       </c>
       <c r="J79" s="12" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="K79" s="11" t="s">
         <v>33</v>
@@ -4894,7 +4883,7 @@
     </row>
     <row r="80" spans="1:12" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A80" s="2" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="B80" t="s">
         <v>85</v>
@@ -4906,22 +4895,22 @@
         <v>35</v>
       </c>
       <c r="E80" s="3" t="s">
+        <v>349</v>
+      </c>
+      <c r="F80" s="3" t="s">
+        <v>214</v>
+      </c>
+      <c r="G80" s="3" t="s">
         <v>350</v>
       </c>
-      <c r="F80" s="3" t="s">
-        <v>215</v>
-      </c>
-      <c r="G80" s="3" t="s">
+      <c r="H80" s="3" t="s">
         <v>351</v>
       </c>
-      <c r="H80" s="3" t="s">
-        <v>352</v>
-      </c>
       <c r="I80" s="5" t="s">
         <v>18</v>
       </c>
       <c r="J80" s="12" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="K80" s="17" t="s">
         <v>62</v>
@@ -4932,7 +4921,7 @@
     </row>
     <row r="81" spans="1:12" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A81" s="2" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="B81" t="s">
         <v>85</v>
@@ -4944,22 +4933,22 @@
         <v>35</v>
       </c>
       <c r="E81" s="3" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="F81" t="s">
         <v>85</v>
       </c>
       <c r="G81" s="3" t="s">
+        <v>354</v>
+      </c>
+      <c r="H81" s="3" t="s">
         <v>355</v>
       </c>
-      <c r="H81" s="3" t="s">
+      <c r="I81" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="J81" s="17" t="s">
         <v>356</v>
-      </c>
-      <c r="I81" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="J81" s="17" t="s">
-        <v>357</v>
       </c>
       <c r="K81" s="17" t="s">
         <v>62</v>
@@ -4970,7 +4959,7 @@
     </row>
     <row r="82" spans="1:12" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A82" s="2" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="B82" s="3">
         <v>3.1</v>
@@ -4982,16 +4971,16 @@
         <v>35</v>
       </c>
       <c r="E82" s="3" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="F82" s="3" t="s">
         <v>15</v>
       </c>
       <c r="G82" s="3" t="s">
+        <v>359</v>
+      </c>
+      <c r="H82" s="3" t="s">
         <v>360</v>
-      </c>
-      <c r="H82" s="3" t="s">
-        <v>361</v>
       </c>
       <c r="I82" s="5" t="s">
         <v>18</v>
@@ -5000,7 +4989,7 @@
         <v>89</v>
       </c>
       <c r="K82" s="8" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="L82" s="15" t="s">
         <v>47</v>
@@ -5008,7 +4997,7 @@
     </row>
     <row r="83" spans="1:12" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A83" s="2" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="B83" s="3">
         <v>3.1</v>
@@ -5020,16 +5009,16 @@
         <v>35</v>
       </c>
       <c r="E83" s="3" t="s">
+        <v>363</v>
+      </c>
+      <c r="F83" s="3" t="s">
+        <v>256</v>
+      </c>
+      <c r="G83" s="3" t="s">
         <v>364</v>
       </c>
-      <c r="F83" s="3" t="s">
-        <v>257</v>
-      </c>
-      <c r="G83" s="3" t="s">
+      <c r="H83" s="3" t="s">
         <v>365</v>
-      </c>
-      <c r="H83" s="3" t="s">
-        <v>366</v>
       </c>
       <c r="I83" s="5" t="s">
         <v>18</v>
@@ -5046,7 +5035,7 @@
     </row>
     <row r="84" spans="1:12" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A84" s="2" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="B84" s="3">
         <v>3</v>
@@ -5058,25 +5047,25 @@
         <v>35</v>
       </c>
       <c r="E84" s="3" t="s">
+        <v>367</v>
+      </c>
+      <c r="F84" s="3" t="s">
         <v>368</v>
       </c>
-      <c r="F84" s="3" t="s">
+      <c r="G84" s="3" t="s">
         <v>369</v>
       </c>
-      <c r="G84" s="3" t="s">
+      <c r="H84" s="3" t="s">
         <v>370</v>
       </c>
-      <c r="H84" s="3" t="s">
+      <c r="I84" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="J84" s="21" t="s">
         <v>371</v>
       </c>
-      <c r="I84" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="J84" s="22" t="s">
-        <v>372</v>
-      </c>
-      <c r="K84" s="19" t="s">
-        <v>90</v>
+      <c r="K84" s="18" t="s">
+        <v>79</v>
       </c>
       <c r="L84" s="15" t="s">
         <v>47</v>
@@ -5084,7 +5073,7 @@
     </row>
     <row r="85" spans="1:12" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A85" s="2" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="B85" s="3">
         <v>3</v>
@@ -5096,25 +5085,25 @@
         <v>35</v>
       </c>
       <c r="E85" s="3" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="F85" s="3" t="s">
         <v>15</v>
       </c>
       <c r="G85" s="3" t="s">
+        <v>374</v>
+      </c>
+      <c r="H85" s="3" t="s">
         <v>375</v>
       </c>
-      <c r="H85" s="3" t="s">
-        <v>376</v>
-      </c>
       <c r="I85" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="J85" s="22" t="s">
-        <v>372</v>
+      <c r="J85" s="21" t="s">
+        <v>371</v>
       </c>
       <c r="K85" s="16" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="L85" s="15" t="s">
         <v>47</v>
@@ -5122,7 +5111,7 @@
     </row>
     <row r="86" spans="1:12" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A86" s="2" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="B86" s="3">
         <v>3</v>
@@ -5131,28 +5120,28 @@
         <v>30</v>
       </c>
       <c r="D86" s="13" t="s">
+        <v>377</v>
+      </c>
+      <c r="E86" s="3" t="s">
         <v>378</v>
       </c>
-      <c r="E86" s="3" t="s">
+      <c r="F86" s="3" t="s">
         <v>379</v>
       </c>
-      <c r="F86" s="3" t="s">
+      <c r="G86" s="3" t="s">
+        <v>287</v>
+      </c>
+      <c r="H86" s="3" t="s">
         <v>380</v>
       </c>
-      <c r="G86" s="3" t="s">
-        <v>288</v>
-      </c>
-      <c r="H86" s="3" t="s">
-        <v>381</v>
-      </c>
-      <c r="I86" s="23" t="s">
-        <v>431</v>
+      <c r="I86" s="22" t="s">
+        <v>430</v>
       </c>
       <c r="J86" s="5" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="K86" s="4" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="L86" s="10" t="s">
         <v>28</v>
@@ -5160,7 +5149,7 @@
     </row>
     <row r="87" spans="1:12" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A87" s="2" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="B87" s="3">
         <v>3</v>
@@ -5169,28 +5158,28 @@
         <v>30</v>
       </c>
       <c r="D87" s="13" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="E87" s="3" t="s">
+        <v>382</v>
+      </c>
+      <c r="F87" s="3" t="s">
+        <v>256</v>
+      </c>
+      <c r="G87" s="3" t="s">
+        <v>381</v>
+      </c>
+      <c r="H87" s="3" t="s">
         <v>383</v>
       </c>
-      <c r="F87" s="3" t="s">
-        <v>257</v>
-      </c>
-      <c r="G87" s="3" t="s">
-        <v>382</v>
-      </c>
-      <c r="H87" s="3" t="s">
-        <v>384</v>
-      </c>
       <c r="I87" s="14" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
       <c r="J87" s="5" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="K87" s="8" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="L87" s="10" t="s">
         <v>28</v>
@@ -5198,7 +5187,7 @@
     </row>
     <row r="88" spans="1:12" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A88" s="2" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="B88" s="3">
         <v>3</v>
@@ -5207,25 +5196,25 @@
         <v>30.1</v>
       </c>
       <c r="D88" s="13" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="E88" s="3" t="s">
+        <v>385</v>
+      </c>
+      <c r="F88" s="3" t="s">
+        <v>256</v>
+      </c>
+      <c r="G88" s="3" t="s">
         <v>386</v>
       </c>
-      <c r="F88" s="3" t="s">
-        <v>257</v>
-      </c>
-      <c r="G88" s="3" t="s">
+      <c r="H88" s="3" t="s">
         <v>387</v>
       </c>
-      <c r="H88" s="3" t="s">
-        <v>388</v>
-      </c>
       <c r="I88" s="14" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
       <c r="J88" s="5" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="K88" s="17" t="s">
         <v>62</v>
@@ -5236,7 +5225,7 @@
     </row>
     <row r="89" spans="1:12" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A89" s="2" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="B89" s="3">
         <v>3</v>
@@ -5245,28 +5234,28 @@
         <v>30</v>
       </c>
       <c r="D89" s="13" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="E89" s="3" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="F89" s="3" t="s">
         <v>54</v>
       </c>
       <c r="G89" s="3" t="s">
+        <v>390</v>
+      </c>
+      <c r="H89" s="3" t="s">
         <v>391</v>
       </c>
-      <c r="H89" s="3" t="s">
-        <v>392</v>
-      </c>
       <c r="I89" s="14" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
       <c r="J89" s="5" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="K89" s="16" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="L89" s="10" t="s">
         <v>28</v>
@@ -5274,7 +5263,7 @@
     </row>
     <row r="90" spans="1:12" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A90" s="2" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="B90" s="3">
         <v>3</v>
@@ -5283,25 +5272,25 @@
         <v>30</v>
       </c>
       <c r="D90" s="13" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="E90" s="3" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="F90" s="3" t="s">
         <v>54</v>
       </c>
       <c r="G90" s="3" t="s">
+        <v>394</v>
+      </c>
+      <c r="H90" s="3" t="s">
         <v>395</v>
       </c>
-      <c r="H90" s="3" t="s">
-        <v>396</v>
-      </c>
       <c r="I90" s="14" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
       <c r="J90" s="5" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="K90" s="5" t="s">
         <v>20</v>
@@ -5312,7 +5301,7 @@
     </row>
     <row r="91" spans="1:12" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A91" s="2" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
       <c r="B91" s="3">
         <v>3</v>
@@ -5321,25 +5310,25 @@
         <v>30</v>
       </c>
       <c r="D91" s="13" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="E91" s="3" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="F91" s="3" t="s">
         <v>54</v>
       </c>
       <c r="G91" s="3" t="s">
+        <v>398</v>
+      </c>
+      <c r="H91" s="3" t="s">
         <v>399</v>
       </c>
-      <c r="H91" s="3" t="s">
-        <v>400</v>
-      </c>
       <c r="I91" s="14" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
       <c r="J91" s="5" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="K91" s="5" t="s">
         <v>20</v>
@@ -5350,7 +5339,7 @@
     </row>
     <row r="92" spans="1:12" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A92" s="2" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="B92" s="3">
         <v>3</v>
@@ -5359,28 +5348,28 @@
         <v>30</v>
       </c>
       <c r="D92" s="13" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="E92" s="3" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="F92" s="3" t="s">
         <v>54</v>
       </c>
       <c r="G92" s="3" t="s">
+        <v>402</v>
+      </c>
+      <c r="H92" s="3" t="s">
         <v>403</v>
       </c>
-      <c r="H92" s="3" t="s">
-        <v>404</v>
-      </c>
       <c r="I92" s="14" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
       <c r="J92" s="5" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="K92" s="16" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="L92" s="10" t="s">
         <v>28</v>
@@ -5388,7 +5377,7 @@
     </row>
     <row r="93" spans="1:12" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A93" s="2" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
       <c r="B93" s="3">
         <v>3</v>
@@ -5397,28 +5386,28 @@
         <v>30</v>
       </c>
       <c r="D93" s="13" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="E93" s="3" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="F93" s="3" t="s">
         <v>54</v>
       </c>
       <c r="G93" s="3" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="H93" s="3" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="I93" s="14" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
       <c r="J93" s="5" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="K93" s="14" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="L93" s="10" t="s">
         <v>28</v>
@@ -5426,7 +5415,7 @@
     </row>
     <row r="94" spans="1:12" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A94" s="2" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="B94" s="3">
         <v>3</v>
@@ -5435,25 +5424,25 @@
         <v>30</v>
       </c>
       <c r="D94" s="13" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="E94" s="3" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="F94" s="3" t="s">
         <v>54</v>
       </c>
       <c r="G94" s="3" t="s">
+        <v>409</v>
+      </c>
+      <c r="H94" s="3" t="s">
         <v>410</v>
       </c>
-      <c r="H94" s="3" t="s">
-        <v>411</v>
-      </c>
       <c r="I94" s="14" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
       <c r="J94" s="5" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="K94" s="11" t="s">
         <v>33</v>
@@ -5464,7 +5453,7 @@
     </row>
     <row r="95" spans="1:12" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A95" s="2" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
       <c r="B95" s="3">
         <v>3</v>
@@ -5473,25 +5462,25 @@
         <v>30</v>
       </c>
       <c r="D95" s="13" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="E95" s="3" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="F95" s="3" t="s">
         <v>54</v>
       </c>
       <c r="G95" s="3" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
       <c r="H95" s="3" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="I95" s="14" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
       <c r="J95" s="5" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="K95" s="5" t="s">
         <v>20</v>
@@ -5502,7 +5491,7 @@
     </row>
     <row r="96" spans="1:12" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A96" s="2" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="B96" s="3">
         <v>3</v>
@@ -5511,28 +5500,28 @@
         <v>30</v>
       </c>
       <c r="D96" s="13" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="E96" s="3" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="F96" s="3" t="s">
         <v>54</v>
       </c>
       <c r="G96" s="3" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="H96" s="3" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
       <c r="I96" s="14" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
       <c r="J96" s="5" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="K96" s="14" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="L96" s="10" t="s">
         <v>28</v>
@@ -5540,7 +5529,7 @@
     </row>
     <row r="97" spans="1:12" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A97" s="2" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="B97" s="3">
         <v>3</v>
@@ -5552,25 +5541,25 @@
         <v>43</v>
       </c>
       <c r="E97" s="3" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
       <c r="F97" s="3" t="s">
         <v>54</v>
       </c>
       <c r="G97" s="3" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="H97" s="3" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="I97" s="14" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
       <c r="J97" s="5" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="K97" s="14" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="L97" s="15" t="s">
         <v>47</v>
@@ -5578,7 +5567,7 @@
     </row>
     <row r="98" spans="1:12" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A98" s="2" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="B98" s="3">
         <v>3</v>
@@ -5590,25 +5579,25 @@
         <v>43</v>
       </c>
       <c r="E98" s="3" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
       <c r="F98" s="3" t="s">
         <v>54</v>
       </c>
       <c r="G98" s="3" t="s">
+        <v>422</v>
+      </c>
+      <c r="H98" s="3" t="s">
         <v>423</v>
       </c>
-      <c r="H98" s="3" t="s">
-        <v>424</v>
-      </c>
       <c r="I98" s="14" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
       <c r="J98" s="5" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="K98" s="9" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="L98" s="15" t="s">
         <v>47</v>
@@ -5616,7 +5605,7 @@
     </row>
     <row r="99" spans="1:12" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A99" s="2" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="B99" s="3">
         <v>3</v>
@@ -5628,22 +5617,22 @@
         <v>43</v>
       </c>
       <c r="E99" s="3" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="F99" s="3" t="s">
         <v>54</v>
       </c>
       <c r="G99" s="3" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="H99" s="3" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
       <c r="I99" s="14" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
       <c r="J99" s="5" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="K99" s="11" t="s">
         <v>33</v>
@@ -5654,7 +5643,7 @@
     </row>
     <row r="100" spans="1:12" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A100" s="2" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
       <c r="B100" s="3">
         <v>3</v>
@@ -5666,7 +5655,7 @@
         <v>43</v>
       </c>
       <c r="E100" s="3" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="F100" s="3" t="s">
         <v>54</v>
@@ -5675,16 +5664,16 @@
         <v>77</v>
       </c>
       <c r="H100" s="3" t="s">
+        <v>429</v>
+      </c>
+      <c r="I100" s="14" t="s">
         <v>430</v>
       </c>
-      <c r="I100" s="14" t="s">
-        <v>431</v>
-      </c>
       <c r="J100" s="5" t="s">
-        <v>141</v>
-      </c>
-      <c r="K100" s="19" t="s">
-        <v>90</v>
+        <v>140</v>
+      </c>
+      <c r="K100" s="18" t="s">
+        <v>79</v>
       </c>
       <c r="L100" s="15" t="s">
         <v>47</v>

</xml_diff>